<commit_message>
Auto backup: 2026-08-03 18:50:25
</commit_message>
<xml_diff>
--- a/QuanLyKhoXe.xlsx
+++ b/QuanLyKhoXe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BuonBanXe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFC16BE-92CA-41B2-9AFC-DAF845FCF8E4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882DB478-1B51-464E-95FC-C5AE1E59E0DF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="68">
   <si>
     <t>QUẢN LÝ KHO XE — NHẬP · CỌC · BÁN · LÃI</t>
   </si>
@@ -227,6 +227,9 @@
   <si>
     <t>• File có sẵn 200 dòng. Cần thêm thì copy 1 dòng trống kéo xuống là công thức tự theo.</t>
   </si>
+  <si>
+    <t>poscher</t>
+  </si>
 </sst>
 </file>
 
@@ -301,7 +304,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -326,6 +329,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -356,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -396,6 +405,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -721,11 +738,11 @@
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="7" max="7" width="18" style="24" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="14" style="24" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="24" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="24" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="17" style="24" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
     <col min="13" max="13" width="17" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
@@ -795,19 +812,19 @@
       <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="21" t="s">
         <v>12</v>
       </c>
       <c r="L3" s="1" t="s">
@@ -837,40 +854,36 @@
       <c r="B4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="4">
-        <v>10000000</v>
-      </c>
+      <c r="C4" s="4"/>
       <c r="D4" s="5">
         <f>DATE(2026,7,25)+TIME(9,0,0)</f>
         <v>46228.375</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="6" t="str">
         <f t="shared" ref="E4:E35" si="1">IF(C4="","",C4*1.35)</f>
-        <v>13500000</v>
+        <v/>
       </c>
       <c r="F4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="23">
         <v>1000000</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="23">
         <v>13000000</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="25">
         <f t="shared" ref="J4:J35" si="2">IF(OR(I4="",H4=""),"",MAX(0,I4-H4))</f>
         <v>12000000</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="26">
         <f>DATE(2026,7,26)+TIME(14,30,0)</f>
         <v>46229.604166666664</v>
       </c>
-      <c r="L4" s="4">
-        <v>13000000</v>
-      </c>
+      <c r="L4" s="4"/>
       <c r="M4" s="5">
         <f>DATE(2026,7,27)+TIME(16,0,0)</f>
         <v>46230.666666666664</v>
@@ -879,44 +892,50 @@
         <f t="shared" ref="N4:N35" ca="1" si="3">IF(D4="","",IF(M4&lt;&gt;"",IF(M4-D4&gt;=2,"Đủ","Chưa"),IF(NOW()-D4&gt;=2,"Đủ","Chưa")))</f>
         <v>Đủ</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="6" t="str">
         <f t="shared" ref="O4:O35" si="4">IF(L4="","",L4*0.05)</f>
-        <v>650000</v>
-      </c>
-      <c r="P4" s="6">
+        <v/>
+      </c>
+      <c r="P4" s="6" t="str">
         <f t="shared" ref="P4:P35" si="5">IF(OR(L4="",C4=""),"",L4*0.95-C4)</f>
-        <v>2350000</v>
+        <v/>
       </c>
       <c r="Q4" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="2">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B5" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
+      <c r="D5" s="5">
+        <v>46235.070833333331</v>
+      </c>
       <c r="E5" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="6" t="str">
+      <c r="F5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K5" s="5"/>
+      <c r="K5" s="26"/>
       <c r="L5" s="4"/>
       <c r="M5" s="5"/>
       <c r="N5" s="2" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v/>
+        <v>Đủ</v>
       </c>
       <c r="O5" s="6" t="str">
         <f t="shared" si="4"/>
@@ -941,14 +960,14 @@
         <v/>
       </c>
       <c r="F6" s="7"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="6" t="str">
+      <c r="G6" s="22"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K6" s="5"/>
+      <c r="K6" s="26"/>
       <c r="L6" s="4"/>
       <c r="M6" s="5"/>
       <c r="N6" s="2" t="str">
@@ -978,14 +997,14 @@
         <v/>
       </c>
       <c r="F7" s="7"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="6" t="str">
+      <c r="G7" s="22"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K7" s="5"/>
+      <c r="K7" s="26"/>
       <c r="L7" s="4"/>
       <c r="M7" s="5"/>
       <c r="N7" s="2" t="str">
@@ -1015,14 +1034,14 @@
         <v/>
       </c>
       <c r="F8" s="7"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="6" t="str">
+      <c r="G8" s="22"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K8" s="5"/>
+      <c r="K8" s="26"/>
       <c r="L8" s="4"/>
       <c r="M8" s="5"/>
       <c r="N8" s="2" t="str">
@@ -1052,14 +1071,14 @@
         <v/>
       </c>
       <c r="F9" s="7"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="6" t="str">
+      <c r="G9" s="22"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K9" s="5"/>
+      <c r="K9" s="26"/>
       <c r="L9" s="4"/>
       <c r="M9" s="5"/>
       <c r="N9" s="2" t="str">
@@ -1089,14 +1108,14 @@
         <v/>
       </c>
       <c r="F10" s="7"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="6" t="str">
+      <c r="G10" s="22"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K10" s="5"/>
+      <c r="K10" s="26"/>
       <c r="L10" s="4"/>
       <c r="M10" s="5"/>
       <c r="N10" s="2" t="str">
@@ -1126,14 +1145,14 @@
         <v/>
       </c>
       <c r="F11" s="7"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="6" t="str">
+      <c r="G11" s="22"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K11" s="5"/>
+      <c r="K11" s="26"/>
       <c r="L11" s="4"/>
       <c r="M11" s="5"/>
       <c r="N11" s="2" t="str">
@@ -1163,14 +1182,14 @@
         <v/>
       </c>
       <c r="F12" s="7"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="6" t="str">
+      <c r="G12" s="22"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K12" s="5"/>
+      <c r="K12" s="26"/>
       <c r="L12" s="4"/>
       <c r="M12" s="5"/>
       <c r="N12" s="2" t="str">
@@ -1200,14 +1219,14 @@
         <v/>
       </c>
       <c r="F13" s="7"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="6" t="str">
+      <c r="G13" s="22"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K13" s="5"/>
+      <c r="K13" s="26"/>
       <c r="L13" s="4"/>
       <c r="M13" s="5"/>
       <c r="N13" s="2" t="str">
@@ -1237,14 +1256,14 @@
         <v/>
       </c>
       <c r="F14" s="7"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="6" t="str">
+      <c r="G14" s="22"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K14" s="5"/>
+      <c r="K14" s="26"/>
       <c r="L14" s="4"/>
       <c r="M14" s="5"/>
       <c r="N14" s="2" t="str">
@@ -1274,14 +1293,14 @@
         <v/>
       </c>
       <c r="F15" s="7"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="6" t="str">
+      <c r="G15" s="22"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K15" s="5"/>
+      <c r="K15" s="26"/>
       <c r="L15" s="4"/>
       <c r="M15" s="5"/>
       <c r="N15" s="2" t="str">
@@ -1311,14 +1330,14 @@
         <v/>
       </c>
       <c r="F16" s="7"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="6" t="str">
+      <c r="G16" s="22"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K16" s="5"/>
+      <c r="K16" s="26"/>
       <c r="L16" s="4"/>
       <c r="M16" s="5"/>
       <c r="N16" s="2" t="str">
@@ -1348,14 +1367,14 @@
         <v/>
       </c>
       <c r="F17" s="7"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="6" t="str">
+      <c r="G17" s="22"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K17" s="5"/>
+      <c r="K17" s="26"/>
       <c r="L17" s="4"/>
       <c r="M17" s="5"/>
       <c r="N17" s="2" t="str">
@@ -1385,14 +1404,14 @@
         <v/>
       </c>
       <c r="F18" s="7"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="6" t="str">
+      <c r="G18" s="22"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K18" s="5"/>
+      <c r="K18" s="26"/>
       <c r="L18" s="4"/>
       <c r="M18" s="5"/>
       <c r="N18" s="2" t="str">
@@ -1422,14 +1441,14 @@
         <v/>
       </c>
       <c r="F19" s="7"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="6" t="str">
+      <c r="G19" s="22"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K19" s="5"/>
+      <c r="K19" s="26"/>
       <c r="L19" s="4"/>
       <c r="M19" s="5"/>
       <c r="N19" s="2" t="str">
@@ -1459,14 +1478,14 @@
         <v/>
       </c>
       <c r="F20" s="7"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="6" t="str">
+      <c r="G20" s="22"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K20" s="5"/>
+      <c r="K20" s="26"/>
       <c r="L20" s="4"/>
       <c r="M20" s="5"/>
       <c r="N20" s="2" t="str">
@@ -1496,14 +1515,14 @@
         <v/>
       </c>
       <c r="F21" s="7"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="6" t="str">
+      <c r="G21" s="22"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K21" s="5"/>
+      <c r="K21" s="26"/>
       <c r="L21" s="4"/>
       <c r="M21" s="5"/>
       <c r="N21" s="2" t="str">
@@ -1533,14 +1552,14 @@
         <v/>
       </c>
       <c r="F22" s="7"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="6" t="str">
+      <c r="G22" s="22"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K22" s="5"/>
+      <c r="K22" s="26"/>
       <c r="L22" s="4"/>
       <c r="M22" s="5"/>
       <c r="N22" s="2" t="str">
@@ -1570,14 +1589,14 @@
         <v/>
       </c>
       <c r="F23" s="7"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="6" t="str">
+      <c r="G23" s="22"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K23" s="5"/>
+      <c r="K23" s="26"/>
       <c r="L23" s="4"/>
       <c r="M23" s="5"/>
       <c r="N23" s="2" t="str">
@@ -1607,14 +1626,14 @@
         <v/>
       </c>
       <c r="F24" s="7"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="6" t="str">
+      <c r="G24" s="22"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K24" s="5"/>
+      <c r="K24" s="26"/>
       <c r="L24" s="4"/>
       <c r="M24" s="5"/>
       <c r="N24" s="2" t="str">
@@ -1644,14 +1663,14 @@
         <v/>
       </c>
       <c r="F25" s="7"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="6" t="str">
+      <c r="G25" s="22"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K25" s="5"/>
+      <c r="K25" s="26"/>
       <c r="L25" s="4"/>
       <c r="M25" s="5"/>
       <c r="N25" s="2" t="str">
@@ -1681,14 +1700,14 @@
         <v/>
       </c>
       <c r="F26" s="7"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="6" t="str">
+      <c r="G26" s="22"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K26" s="5"/>
+      <c r="K26" s="26"/>
       <c r="L26" s="4"/>
       <c r="M26" s="5"/>
       <c r="N26" s="2" t="str">
@@ -1718,14 +1737,14 @@
         <v/>
       </c>
       <c r="F27" s="7"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="6" t="str">
+      <c r="G27" s="22"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K27" s="5"/>
+      <c r="K27" s="26"/>
       <c r="L27" s="4"/>
       <c r="M27" s="5"/>
       <c r="N27" s="2" t="str">
@@ -1755,14 +1774,14 @@
         <v/>
       </c>
       <c r="F28" s="7"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="6" t="str">
+      <c r="G28" s="22"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K28" s="5"/>
+      <c r="K28" s="26"/>
       <c r="L28" s="4"/>
       <c r="M28" s="5"/>
       <c r="N28" s="2" t="str">
@@ -1792,14 +1811,14 @@
         <v/>
       </c>
       <c r="F29" s="7"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="6" t="str">
+      <c r="G29" s="22"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K29" s="5"/>
+      <c r="K29" s="26"/>
       <c r="L29" s="4"/>
       <c r="M29" s="5"/>
       <c r="N29" s="2" t="str">
@@ -1829,14 +1848,14 @@
         <v/>
       </c>
       <c r="F30" s="7"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="6" t="str">
+      <c r="G30" s="22"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K30" s="5"/>
+      <c r="K30" s="26"/>
       <c r="L30" s="4"/>
       <c r="M30" s="5"/>
       <c r="N30" s="2" t="str">
@@ -1866,14 +1885,14 @@
         <v/>
       </c>
       <c r="F31" s="7"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="6" t="str">
+      <c r="G31" s="22"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K31" s="5"/>
+      <c r="K31" s="26"/>
       <c r="L31" s="4"/>
       <c r="M31" s="5"/>
       <c r="N31" s="2" t="str">
@@ -1903,14 +1922,14 @@
         <v/>
       </c>
       <c r="F32" s="7"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="6" t="str">
+      <c r="G32" s="22"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K32" s="5"/>
+      <c r="K32" s="26"/>
       <c r="L32" s="4"/>
       <c r="M32" s="5"/>
       <c r="N32" s="2" t="str">
@@ -1940,14 +1959,14 @@
         <v/>
       </c>
       <c r="F33" s="7"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="6" t="str">
+      <c r="G33" s="22"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K33" s="5"/>
+      <c r="K33" s="26"/>
       <c r="L33" s="4"/>
       <c r="M33" s="5"/>
       <c r="N33" s="2" t="str">
@@ -1977,14 +1996,14 @@
         <v/>
       </c>
       <c r="F34" s="7"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="6" t="str">
+      <c r="G34" s="22"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K34" s="5"/>
+      <c r="K34" s="26"/>
       <c r="L34" s="4"/>
       <c r="M34" s="5"/>
       <c r="N34" s="2" t="str">
@@ -2014,14 +2033,14 @@
         <v/>
       </c>
       <c r="F35" s="7"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="6" t="str">
+      <c r="G35" s="22"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="25" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K35" s="5"/>
+      <c r="K35" s="26"/>
       <c r="L35" s="4"/>
       <c r="M35" s="5"/>
       <c r="N35" s="2" t="str">
@@ -2051,14 +2070,14 @@
         <v/>
       </c>
       <c r="F36" s="7"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="6" t="str">
+      <c r="G36" s="22"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="25" t="str">
         <f t="shared" ref="J36:J67" si="8">IF(OR(I36="",H36=""),"",MAX(0,I36-H36))</f>
         <v/>
       </c>
-      <c r="K36" s="5"/>
+      <c r="K36" s="26"/>
       <c r="L36" s="4"/>
       <c r="M36" s="5"/>
       <c r="N36" s="2" t="str">
@@ -2088,14 +2107,14 @@
         <v/>
       </c>
       <c r="F37" s="7"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="6" t="str">
+      <c r="G37" s="22"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K37" s="5"/>
+      <c r="K37" s="26"/>
       <c r="L37" s="4"/>
       <c r="M37" s="5"/>
       <c r="N37" s="2" t="str">
@@ -2125,14 +2144,14 @@
         <v/>
       </c>
       <c r="F38" s="7"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="4"/>
-      <c r="I38" s="4"/>
-      <c r="J38" s="6" t="str">
+      <c r="G38" s="22"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K38" s="5"/>
+      <c r="K38" s="26"/>
       <c r="L38" s="4"/>
       <c r="M38" s="5"/>
       <c r="N38" s="2" t="str">
@@ -2162,14 +2181,14 @@
         <v/>
       </c>
       <c r="F39" s="7"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="6" t="str">
+      <c r="G39" s="22"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K39" s="5"/>
+      <c r="K39" s="26"/>
       <c r="L39" s="4"/>
       <c r="M39" s="5"/>
       <c r="N39" s="2" t="str">
@@ -2199,14 +2218,14 @@
         <v/>
       </c>
       <c r="F40" s="7"/>
-      <c r="G40" s="3"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="4"/>
-      <c r="J40" s="6" t="str">
+      <c r="G40" s="22"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K40" s="5"/>
+      <c r="K40" s="26"/>
       <c r="L40" s="4"/>
       <c r="M40" s="5"/>
       <c r="N40" s="2" t="str">
@@ -2236,14 +2255,14 @@
         <v/>
       </c>
       <c r="F41" s="7"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="6" t="str">
+      <c r="G41" s="22"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K41" s="5"/>
+      <c r="K41" s="26"/>
       <c r="L41" s="4"/>
       <c r="M41" s="5"/>
       <c r="N41" s="2" t="str">
@@ -2273,14 +2292,14 @@
         <v/>
       </c>
       <c r="F42" s="7"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4"/>
-      <c r="J42" s="6" t="str">
+      <c r="G42" s="22"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K42" s="5"/>
+      <c r="K42" s="26"/>
       <c r="L42" s="4"/>
       <c r="M42" s="5"/>
       <c r="N42" s="2" t="str">
@@ -2310,14 +2329,14 @@
         <v/>
       </c>
       <c r="F43" s="7"/>
-      <c r="G43" s="3"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="6" t="str">
+      <c r="G43" s="22"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="23"/>
+      <c r="J43" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K43" s="5"/>
+      <c r="K43" s="26"/>
       <c r="L43" s="4"/>
       <c r="M43" s="5"/>
       <c r="N43" s="2" t="str">
@@ -2347,14 +2366,14 @@
         <v/>
       </c>
       <c r="F44" s="7"/>
-      <c r="G44" s="3"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="6" t="str">
+      <c r="G44" s="22"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K44" s="5"/>
+      <c r="K44" s="26"/>
       <c r="L44" s="4"/>
       <c r="M44" s="5"/>
       <c r="N44" s="2" t="str">
@@ -2384,14 +2403,14 @@
         <v/>
       </c>
       <c r="F45" s="7"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="6" t="str">
+      <c r="G45" s="22"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
+      <c r="J45" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K45" s="5"/>
+      <c r="K45" s="26"/>
       <c r="L45" s="4"/>
       <c r="M45" s="5"/>
       <c r="N45" s="2" t="str">
@@ -2421,14 +2440,14 @@
         <v/>
       </c>
       <c r="F46" s="7"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
-      <c r="J46" s="6" t="str">
+      <c r="G46" s="22"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K46" s="5"/>
+      <c r="K46" s="26"/>
       <c r="L46" s="4"/>
       <c r="M46" s="5"/>
       <c r="N46" s="2" t="str">
@@ -2458,14 +2477,14 @@
         <v/>
       </c>
       <c r="F47" s="7"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="6" t="str">
+      <c r="G47" s="22"/>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K47" s="5"/>
+      <c r="K47" s="26"/>
       <c r="L47" s="4"/>
       <c r="M47" s="5"/>
       <c r="N47" s="2" t="str">
@@ -2495,14 +2514,14 @@
         <v/>
       </c>
       <c r="F48" s="7"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="6" t="str">
+      <c r="G48" s="22"/>
+      <c r="H48" s="23"/>
+      <c r="I48" s="23"/>
+      <c r="J48" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K48" s="5"/>
+      <c r="K48" s="26"/>
       <c r="L48" s="4"/>
       <c r="M48" s="5"/>
       <c r="N48" s="2" t="str">
@@ -2532,14 +2551,14 @@
         <v/>
       </c>
       <c r="F49" s="7"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
-      <c r="J49" s="6" t="str">
+      <c r="G49" s="22"/>
+      <c r="H49" s="23"/>
+      <c r="I49" s="23"/>
+      <c r="J49" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K49" s="5"/>
+      <c r="K49" s="26"/>
       <c r="L49" s="4"/>
       <c r="M49" s="5"/>
       <c r="N49" s="2" t="str">
@@ -2569,14 +2588,14 @@
         <v/>
       </c>
       <c r="F50" s="7"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="6" t="str">
+      <c r="G50" s="22"/>
+      <c r="H50" s="23"/>
+      <c r="I50" s="23"/>
+      <c r="J50" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K50" s="5"/>
+      <c r="K50" s="26"/>
       <c r="L50" s="4"/>
       <c r="M50" s="5"/>
       <c r="N50" s="2" t="str">
@@ -2606,14 +2625,14 @@
         <v/>
       </c>
       <c r="F51" s="7"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="6" t="str">
+      <c r="G51" s="22"/>
+      <c r="H51" s="23"/>
+      <c r="I51" s="23"/>
+      <c r="J51" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K51" s="5"/>
+      <c r="K51" s="26"/>
       <c r="L51" s="4"/>
       <c r="M51" s="5"/>
       <c r="N51" s="2" t="str">
@@ -2643,14 +2662,14 @@
         <v/>
       </c>
       <c r="F52" s="7"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-      <c r="J52" s="6" t="str">
+      <c r="G52" s="22"/>
+      <c r="H52" s="23"/>
+      <c r="I52" s="23"/>
+      <c r="J52" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K52" s="5"/>
+      <c r="K52" s="26"/>
       <c r="L52" s="4"/>
       <c r="M52" s="5"/>
       <c r="N52" s="2" t="str">
@@ -2680,14 +2699,14 @@
         <v/>
       </c>
       <c r="F53" s="7"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="4"/>
-      <c r="I53" s="4"/>
-      <c r="J53" s="6" t="str">
+      <c r="G53" s="22"/>
+      <c r="H53" s="23"/>
+      <c r="I53" s="23"/>
+      <c r="J53" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K53" s="5"/>
+      <c r="K53" s="26"/>
       <c r="L53" s="4"/>
       <c r="M53" s="5"/>
       <c r="N53" s="2" t="str">
@@ -2717,14 +2736,14 @@
         <v/>
       </c>
       <c r="F54" s="7"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="4"/>
-      <c r="I54" s="4"/>
-      <c r="J54" s="6" t="str">
+      <c r="G54" s="22"/>
+      <c r="H54" s="23"/>
+      <c r="I54" s="23"/>
+      <c r="J54" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K54" s="5"/>
+      <c r="K54" s="26"/>
       <c r="L54" s="4"/>
       <c r="M54" s="5"/>
       <c r="N54" s="2" t="str">
@@ -2754,14 +2773,14 @@
         <v/>
       </c>
       <c r="F55" s="7"/>
-      <c r="G55" s="3"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="6" t="str">
+      <c r="G55" s="22"/>
+      <c r="H55" s="23"/>
+      <c r="I55" s="23"/>
+      <c r="J55" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K55" s="5"/>
+      <c r="K55" s="26"/>
       <c r="L55" s="4"/>
       <c r="M55" s="5"/>
       <c r="N55" s="2" t="str">
@@ -2791,14 +2810,14 @@
         <v/>
       </c>
       <c r="F56" s="7"/>
-      <c r="G56" s="3"/>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4"/>
-      <c r="J56" s="6" t="str">
+      <c r="G56" s="22"/>
+      <c r="H56" s="23"/>
+      <c r="I56" s="23"/>
+      <c r="J56" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K56" s="5"/>
+      <c r="K56" s="26"/>
       <c r="L56" s="4"/>
       <c r="M56" s="5"/>
       <c r="N56" s="2" t="str">
@@ -2828,14 +2847,14 @@
         <v/>
       </c>
       <c r="F57" s="7"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="4"/>
-      <c r="I57" s="4"/>
-      <c r="J57" s="6" t="str">
+      <c r="G57" s="22"/>
+      <c r="H57" s="23"/>
+      <c r="I57" s="23"/>
+      <c r="J57" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K57" s="5"/>
+      <c r="K57" s="26"/>
       <c r="L57" s="4"/>
       <c r="M57" s="5"/>
       <c r="N57" s="2" t="str">
@@ -2865,14 +2884,14 @@
         <v/>
       </c>
       <c r="F58" s="7"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
-      <c r="J58" s="6" t="str">
+      <c r="G58" s="22"/>
+      <c r="H58" s="23"/>
+      <c r="I58" s="23"/>
+      <c r="J58" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K58" s="5"/>
+      <c r="K58" s="26"/>
       <c r="L58" s="4"/>
       <c r="M58" s="5"/>
       <c r="N58" s="2" t="str">
@@ -2902,14 +2921,14 @@
         <v/>
       </c>
       <c r="F59" s="7"/>
-      <c r="G59" s="3"/>
-      <c r="H59" s="4"/>
-      <c r="I59" s="4"/>
-      <c r="J59" s="6" t="str">
+      <c r="G59" s="22"/>
+      <c r="H59" s="23"/>
+      <c r="I59" s="23"/>
+      <c r="J59" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K59" s="5"/>
+      <c r="K59" s="26"/>
       <c r="L59" s="4"/>
       <c r="M59" s="5"/>
       <c r="N59" s="2" t="str">
@@ -2939,14 +2958,14 @@
         <v/>
       </c>
       <c r="F60" s="7"/>
-      <c r="G60" s="3"/>
-      <c r="H60" s="4"/>
-      <c r="I60" s="4"/>
-      <c r="J60" s="6" t="str">
+      <c r="G60" s="22"/>
+      <c r="H60" s="23"/>
+      <c r="I60" s="23"/>
+      <c r="J60" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K60" s="5"/>
+      <c r="K60" s="26"/>
       <c r="L60" s="4"/>
       <c r="M60" s="5"/>
       <c r="N60" s="2" t="str">
@@ -2976,14 +2995,14 @@
         <v/>
       </c>
       <c r="F61" s="7"/>
-      <c r="G61" s="3"/>
-      <c r="H61" s="4"/>
-      <c r="I61" s="4"/>
-      <c r="J61" s="6" t="str">
+      <c r="G61" s="22"/>
+      <c r="H61" s="23"/>
+      <c r="I61" s="23"/>
+      <c r="J61" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K61" s="5"/>
+      <c r="K61" s="26"/>
       <c r="L61" s="4"/>
       <c r="M61" s="5"/>
       <c r="N61" s="2" t="str">
@@ -3013,14 +3032,14 @@
         <v/>
       </c>
       <c r="F62" s="7"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="4"/>
-      <c r="I62" s="4"/>
-      <c r="J62" s="6" t="str">
+      <c r="G62" s="22"/>
+      <c r="H62" s="23"/>
+      <c r="I62" s="23"/>
+      <c r="J62" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K62" s="5"/>
+      <c r="K62" s="26"/>
       <c r="L62" s="4"/>
       <c r="M62" s="5"/>
       <c r="N62" s="2" t="str">
@@ -3050,14 +3069,14 @@
         <v/>
       </c>
       <c r="F63" s="7"/>
-      <c r="G63" s="3"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
-      <c r="J63" s="6" t="str">
+      <c r="G63" s="22"/>
+      <c r="H63" s="23"/>
+      <c r="I63" s="23"/>
+      <c r="J63" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K63" s="5"/>
+      <c r="K63" s="26"/>
       <c r="L63" s="4"/>
       <c r="M63" s="5"/>
       <c r="N63" s="2" t="str">
@@ -3087,14 +3106,14 @@
         <v/>
       </c>
       <c r="F64" s="7"/>
-      <c r="G64" s="3"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
-      <c r="J64" s="6" t="str">
+      <c r="G64" s="22"/>
+      <c r="H64" s="23"/>
+      <c r="I64" s="23"/>
+      <c r="J64" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K64" s="5"/>
+      <c r="K64" s="26"/>
       <c r="L64" s="4"/>
       <c r="M64" s="5"/>
       <c r="N64" s="2" t="str">
@@ -3124,14 +3143,14 @@
         <v/>
       </c>
       <c r="F65" s="7"/>
-      <c r="G65" s="3"/>
-      <c r="H65" s="4"/>
-      <c r="I65" s="4"/>
-      <c r="J65" s="6" t="str">
+      <c r="G65" s="22"/>
+      <c r="H65" s="23"/>
+      <c r="I65" s="23"/>
+      <c r="J65" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K65" s="5"/>
+      <c r="K65" s="26"/>
       <c r="L65" s="4"/>
       <c r="M65" s="5"/>
       <c r="N65" s="2" t="str">
@@ -3161,14 +3180,14 @@
         <v/>
       </c>
       <c r="F66" s="7"/>
-      <c r="G66" s="3"/>
-      <c r="H66" s="4"/>
-      <c r="I66" s="4"/>
-      <c r="J66" s="6" t="str">
+      <c r="G66" s="22"/>
+      <c r="H66" s="23"/>
+      <c r="I66" s="23"/>
+      <c r="J66" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K66" s="5"/>
+      <c r="K66" s="26"/>
       <c r="L66" s="4"/>
       <c r="M66" s="5"/>
       <c r="N66" s="2" t="str">
@@ -3198,14 +3217,14 @@
         <v/>
       </c>
       <c r="F67" s="7"/>
-      <c r="G67" s="3"/>
-      <c r="H67" s="4"/>
-      <c r="I67" s="4"/>
-      <c r="J67" s="6" t="str">
+      <c r="G67" s="22"/>
+      <c r="H67" s="23"/>
+      <c r="I67" s="23"/>
+      <c r="J67" s="25" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K67" s="5"/>
+      <c r="K67" s="26"/>
       <c r="L67" s="4"/>
       <c r="M67" s="5"/>
       <c r="N67" s="2" t="str">
@@ -3235,14 +3254,14 @@
         <v/>
       </c>
       <c r="F68" s="7"/>
-      <c r="G68" s="3"/>
-      <c r="H68" s="4"/>
-      <c r="I68" s="4"/>
-      <c r="J68" s="6" t="str">
+      <c r="G68" s="22"/>
+      <c r="H68" s="23"/>
+      <c r="I68" s="23"/>
+      <c r="J68" s="25" t="str">
         <f t="shared" ref="J68:J99" si="14">IF(OR(I68="",H68=""),"",MAX(0,I68-H68))</f>
         <v/>
       </c>
-      <c r="K68" s="5"/>
+      <c r="K68" s="26"/>
       <c r="L68" s="4"/>
       <c r="M68" s="5"/>
       <c r="N68" s="2" t="str">
@@ -3272,14 +3291,14 @@
         <v/>
       </c>
       <c r="F69" s="7"/>
-      <c r="G69" s="3"/>
-      <c r="H69" s="4"/>
-      <c r="I69" s="4"/>
-      <c r="J69" s="6" t="str">
+      <c r="G69" s="22"/>
+      <c r="H69" s="23"/>
+      <c r="I69" s="23"/>
+      <c r="J69" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K69" s="5"/>
+      <c r="K69" s="26"/>
       <c r="L69" s="4"/>
       <c r="M69" s="5"/>
       <c r="N69" s="2" t="str">
@@ -3309,14 +3328,14 @@
         <v/>
       </c>
       <c r="F70" s="7"/>
-      <c r="G70" s="3"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="6" t="str">
+      <c r="G70" s="22"/>
+      <c r="H70" s="23"/>
+      <c r="I70" s="23"/>
+      <c r="J70" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K70" s="5"/>
+      <c r="K70" s="26"/>
       <c r="L70" s="4"/>
       <c r="M70" s="5"/>
       <c r="N70" s="2" t="str">
@@ -3346,14 +3365,14 @@
         <v/>
       </c>
       <c r="F71" s="7"/>
-      <c r="G71" s="3"/>
-      <c r="H71" s="4"/>
-      <c r="I71" s="4"/>
-      <c r="J71" s="6" t="str">
+      <c r="G71" s="22"/>
+      <c r="H71" s="23"/>
+      <c r="I71" s="23"/>
+      <c r="J71" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K71" s="5"/>
+      <c r="K71" s="26"/>
       <c r="L71" s="4"/>
       <c r="M71" s="5"/>
       <c r="N71" s="2" t="str">
@@ -3383,14 +3402,14 @@
         <v/>
       </c>
       <c r="F72" s="7"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="4"/>
-      <c r="I72" s="4"/>
-      <c r="J72" s="6" t="str">
+      <c r="G72" s="22"/>
+      <c r="H72" s="23"/>
+      <c r="I72" s="23"/>
+      <c r="J72" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K72" s="5"/>
+      <c r="K72" s="26"/>
       <c r="L72" s="4"/>
       <c r="M72" s="5"/>
       <c r="N72" s="2" t="str">
@@ -3420,14 +3439,14 @@
         <v/>
       </c>
       <c r="F73" s="7"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="4"/>
-      <c r="I73" s="4"/>
-      <c r="J73" s="6" t="str">
+      <c r="G73" s="22"/>
+      <c r="H73" s="23"/>
+      <c r="I73" s="23"/>
+      <c r="J73" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K73" s="5"/>
+      <c r="K73" s="26"/>
       <c r="L73" s="4"/>
       <c r="M73" s="5"/>
       <c r="N73" s="2" t="str">
@@ -3457,14 +3476,14 @@
         <v/>
       </c>
       <c r="F74" s="7"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="4"/>
-      <c r="I74" s="4"/>
-      <c r="J74" s="6" t="str">
+      <c r="G74" s="22"/>
+      <c r="H74" s="23"/>
+      <c r="I74" s="23"/>
+      <c r="J74" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K74" s="5"/>
+      <c r="K74" s="26"/>
       <c r="L74" s="4"/>
       <c r="M74" s="5"/>
       <c r="N74" s="2" t="str">
@@ -3494,14 +3513,14 @@
         <v/>
       </c>
       <c r="F75" s="7"/>
-      <c r="G75" s="3"/>
-      <c r="H75" s="4"/>
-      <c r="I75" s="4"/>
-      <c r="J75" s="6" t="str">
+      <c r="G75" s="22"/>
+      <c r="H75" s="23"/>
+      <c r="I75" s="23"/>
+      <c r="J75" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K75" s="5"/>
+      <c r="K75" s="26"/>
       <c r="L75" s="4"/>
       <c r="M75" s="5"/>
       <c r="N75" s="2" t="str">
@@ -3531,14 +3550,14 @@
         <v/>
       </c>
       <c r="F76" s="7"/>
-      <c r="G76" s="3"/>
-      <c r="H76" s="4"/>
-      <c r="I76" s="4"/>
-      <c r="J76" s="6" t="str">
+      <c r="G76" s="22"/>
+      <c r="H76" s="23"/>
+      <c r="I76" s="23"/>
+      <c r="J76" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K76" s="5"/>
+      <c r="K76" s="26"/>
       <c r="L76" s="4"/>
       <c r="M76" s="5"/>
       <c r="N76" s="2" t="str">
@@ -3568,14 +3587,14 @@
         <v/>
       </c>
       <c r="F77" s="7"/>
-      <c r="G77" s="3"/>
-      <c r="H77" s="4"/>
-      <c r="I77" s="4"/>
-      <c r="J77" s="6" t="str">
+      <c r="G77" s="22"/>
+      <c r="H77" s="23"/>
+      <c r="I77" s="23"/>
+      <c r="J77" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K77" s="5"/>
+      <c r="K77" s="26"/>
       <c r="L77" s="4"/>
       <c r="M77" s="5"/>
       <c r="N77" s="2" t="str">
@@ -3605,14 +3624,14 @@
         <v/>
       </c>
       <c r="F78" s="7"/>
-      <c r="G78" s="3"/>
-      <c r="H78" s="4"/>
-      <c r="I78" s="4"/>
-      <c r="J78" s="6" t="str">
+      <c r="G78" s="22"/>
+      <c r="H78" s="23"/>
+      <c r="I78" s="23"/>
+      <c r="J78" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K78" s="5"/>
+      <c r="K78" s="26"/>
       <c r="L78" s="4"/>
       <c r="M78" s="5"/>
       <c r="N78" s="2" t="str">
@@ -3642,14 +3661,14 @@
         <v/>
       </c>
       <c r="F79" s="7"/>
-      <c r="G79" s="3"/>
-      <c r="H79" s="4"/>
-      <c r="I79" s="4"/>
-      <c r="J79" s="6" t="str">
+      <c r="G79" s="22"/>
+      <c r="H79" s="23"/>
+      <c r="I79" s="23"/>
+      <c r="J79" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K79" s="5"/>
+      <c r="K79" s="26"/>
       <c r="L79" s="4"/>
       <c r="M79" s="5"/>
       <c r="N79" s="2" t="str">
@@ -3679,14 +3698,14 @@
         <v/>
       </c>
       <c r="F80" s="7"/>
-      <c r="G80" s="3"/>
-      <c r="H80" s="4"/>
-      <c r="I80" s="4"/>
-      <c r="J80" s="6" t="str">
+      <c r="G80" s="22"/>
+      <c r="H80" s="23"/>
+      <c r="I80" s="23"/>
+      <c r="J80" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K80" s="5"/>
+      <c r="K80" s="26"/>
       <c r="L80" s="4"/>
       <c r="M80" s="5"/>
       <c r="N80" s="2" t="str">
@@ -3716,14 +3735,14 @@
         <v/>
       </c>
       <c r="F81" s="7"/>
-      <c r="G81" s="3"/>
-      <c r="H81" s="4"/>
-      <c r="I81" s="4"/>
-      <c r="J81" s="6" t="str">
+      <c r="G81" s="22"/>
+      <c r="H81" s="23"/>
+      <c r="I81" s="23"/>
+      <c r="J81" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K81" s="5"/>
+      <c r="K81" s="26"/>
       <c r="L81" s="4"/>
       <c r="M81" s="5"/>
       <c r="N81" s="2" t="str">
@@ -3753,14 +3772,14 @@
         <v/>
       </c>
       <c r="F82" s="7"/>
-      <c r="G82" s="3"/>
-      <c r="H82" s="4"/>
-      <c r="I82" s="4"/>
-      <c r="J82" s="6" t="str">
+      <c r="G82" s="22"/>
+      <c r="H82" s="23"/>
+      <c r="I82" s="23"/>
+      <c r="J82" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K82" s="5"/>
+      <c r="K82" s="26"/>
       <c r="L82" s="4"/>
       <c r="M82" s="5"/>
       <c r="N82" s="2" t="str">
@@ -3790,14 +3809,14 @@
         <v/>
       </c>
       <c r="F83" s="7"/>
-      <c r="G83" s="3"/>
-      <c r="H83" s="4"/>
-      <c r="I83" s="4"/>
-      <c r="J83" s="6" t="str">
+      <c r="G83" s="22"/>
+      <c r="H83" s="23"/>
+      <c r="I83" s="23"/>
+      <c r="J83" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K83" s="5"/>
+      <c r="K83" s="26"/>
       <c r="L83" s="4"/>
       <c r="M83" s="5"/>
       <c r="N83" s="2" t="str">
@@ -3827,14 +3846,14 @@
         <v/>
       </c>
       <c r="F84" s="7"/>
-      <c r="G84" s="3"/>
-      <c r="H84" s="4"/>
-      <c r="I84" s="4"/>
-      <c r="J84" s="6" t="str">
+      <c r="G84" s="22"/>
+      <c r="H84" s="23"/>
+      <c r="I84" s="23"/>
+      <c r="J84" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K84" s="5"/>
+      <c r="K84" s="26"/>
       <c r="L84" s="4"/>
       <c r="M84" s="5"/>
       <c r="N84" s="2" t="str">
@@ -3864,14 +3883,14 @@
         <v/>
       </c>
       <c r="F85" s="7"/>
-      <c r="G85" s="3"/>
-      <c r="H85" s="4"/>
-      <c r="I85" s="4"/>
-      <c r="J85" s="6" t="str">
+      <c r="G85" s="22"/>
+      <c r="H85" s="23"/>
+      <c r="I85" s="23"/>
+      <c r="J85" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K85" s="5"/>
+      <c r="K85" s="26"/>
       <c r="L85" s="4"/>
       <c r="M85" s="5"/>
       <c r="N85" s="2" t="str">
@@ -3901,14 +3920,14 @@
         <v/>
       </c>
       <c r="F86" s="7"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="4"/>
-      <c r="I86" s="4"/>
-      <c r="J86" s="6" t="str">
+      <c r="G86" s="22"/>
+      <c r="H86" s="23"/>
+      <c r="I86" s="23"/>
+      <c r="J86" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K86" s="5"/>
+      <c r="K86" s="26"/>
       <c r="L86" s="4"/>
       <c r="M86" s="5"/>
       <c r="N86" s="2" t="str">
@@ -3938,14 +3957,14 @@
         <v/>
       </c>
       <c r="F87" s="7"/>
-      <c r="G87" s="3"/>
-      <c r="H87" s="4"/>
-      <c r="I87" s="4"/>
-      <c r="J87" s="6" t="str">
+      <c r="G87" s="22"/>
+      <c r="H87" s="23"/>
+      <c r="I87" s="23"/>
+      <c r="J87" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K87" s="5"/>
+      <c r="K87" s="26"/>
       <c r="L87" s="4"/>
       <c r="M87" s="5"/>
       <c r="N87" s="2" t="str">
@@ -3975,14 +3994,14 @@
         <v/>
       </c>
       <c r="F88" s="7"/>
-      <c r="G88" s="3"/>
-      <c r="H88" s="4"/>
-      <c r="I88" s="4"/>
-      <c r="J88" s="6" t="str">
+      <c r="G88" s="22"/>
+      <c r="H88" s="23"/>
+      <c r="I88" s="23"/>
+      <c r="J88" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K88" s="5"/>
+      <c r="K88" s="26"/>
       <c r="L88" s="4"/>
       <c r="M88" s="5"/>
       <c r="N88" s="2" t="str">
@@ -4012,14 +4031,14 @@
         <v/>
       </c>
       <c r="F89" s="7"/>
-      <c r="G89" s="3"/>
-      <c r="H89" s="4"/>
-      <c r="I89" s="4"/>
-      <c r="J89" s="6" t="str">
+      <c r="G89" s="22"/>
+      <c r="H89" s="23"/>
+      <c r="I89" s="23"/>
+      <c r="J89" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K89" s="5"/>
+      <c r="K89" s="26"/>
       <c r="L89" s="4"/>
       <c r="M89" s="5"/>
       <c r="N89" s="2" t="str">
@@ -4049,14 +4068,14 @@
         <v/>
       </c>
       <c r="F90" s="7"/>
-      <c r="G90" s="3"/>
-      <c r="H90" s="4"/>
-      <c r="I90" s="4"/>
-      <c r="J90" s="6" t="str">
+      <c r="G90" s="22"/>
+      <c r="H90" s="23"/>
+      <c r="I90" s="23"/>
+      <c r="J90" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K90" s="5"/>
+      <c r="K90" s="26"/>
       <c r="L90" s="4"/>
       <c r="M90" s="5"/>
       <c r="N90" s="2" t="str">
@@ -4086,14 +4105,14 @@
         <v/>
       </c>
       <c r="F91" s="7"/>
-      <c r="G91" s="3"/>
-      <c r="H91" s="4"/>
-      <c r="I91" s="4"/>
-      <c r="J91" s="6" t="str">
+      <c r="G91" s="22"/>
+      <c r="H91" s="23"/>
+      <c r="I91" s="23"/>
+      <c r="J91" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K91" s="5"/>
+      <c r="K91" s="26"/>
       <c r="L91" s="4"/>
       <c r="M91" s="5"/>
       <c r="N91" s="2" t="str">
@@ -4123,14 +4142,14 @@
         <v/>
       </c>
       <c r="F92" s="7"/>
-      <c r="G92" s="3"/>
-      <c r="H92" s="4"/>
-      <c r="I92" s="4"/>
-      <c r="J92" s="6" t="str">
+      <c r="G92" s="22"/>
+      <c r="H92" s="23"/>
+      <c r="I92" s="23"/>
+      <c r="J92" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K92" s="5"/>
+      <c r="K92" s="26"/>
       <c r="L92" s="4"/>
       <c r="M92" s="5"/>
       <c r="N92" s="2" t="str">
@@ -4160,14 +4179,14 @@
         <v/>
       </c>
       <c r="F93" s="7"/>
-      <c r="G93" s="3"/>
-      <c r="H93" s="4"/>
-      <c r="I93" s="4"/>
-      <c r="J93" s="6" t="str">
+      <c r="G93" s="22"/>
+      <c r="H93" s="23"/>
+      <c r="I93" s="23"/>
+      <c r="J93" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K93" s="5"/>
+      <c r="K93" s="26"/>
       <c r="L93" s="4"/>
       <c r="M93" s="5"/>
       <c r="N93" s="2" t="str">
@@ -4197,14 +4216,14 @@
         <v/>
       </c>
       <c r="F94" s="7"/>
-      <c r="G94" s="3"/>
-      <c r="H94" s="4"/>
-      <c r="I94" s="4"/>
-      <c r="J94" s="6" t="str">
+      <c r="G94" s="22"/>
+      <c r="H94" s="23"/>
+      <c r="I94" s="23"/>
+      <c r="J94" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K94" s="5"/>
+      <c r="K94" s="26"/>
       <c r="L94" s="4"/>
       <c r="M94" s="5"/>
       <c r="N94" s="2" t="str">
@@ -4234,14 +4253,14 @@
         <v/>
       </c>
       <c r="F95" s="7"/>
-      <c r="G95" s="3"/>
-      <c r="H95" s="4"/>
-      <c r="I95" s="4"/>
-      <c r="J95" s="6" t="str">
+      <c r="G95" s="22"/>
+      <c r="H95" s="23"/>
+      <c r="I95" s="23"/>
+      <c r="J95" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K95" s="5"/>
+      <c r="K95" s="26"/>
       <c r="L95" s="4"/>
       <c r="M95" s="5"/>
       <c r="N95" s="2" t="str">
@@ -4271,14 +4290,14 @@
         <v/>
       </c>
       <c r="F96" s="7"/>
-      <c r="G96" s="3"/>
-      <c r="H96" s="4"/>
-      <c r="I96" s="4"/>
-      <c r="J96" s="6" t="str">
+      <c r="G96" s="22"/>
+      <c r="H96" s="23"/>
+      <c r="I96" s="23"/>
+      <c r="J96" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K96" s="5"/>
+      <c r="K96" s="26"/>
       <c r="L96" s="4"/>
       <c r="M96" s="5"/>
       <c r="N96" s="2" t="str">
@@ -4308,14 +4327,14 @@
         <v/>
       </c>
       <c r="F97" s="7"/>
-      <c r="G97" s="3"/>
-      <c r="H97" s="4"/>
-      <c r="I97" s="4"/>
-      <c r="J97" s="6" t="str">
+      <c r="G97" s="22"/>
+      <c r="H97" s="23"/>
+      <c r="I97" s="23"/>
+      <c r="J97" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K97" s="5"/>
+      <c r="K97" s="26"/>
       <c r="L97" s="4"/>
       <c r="M97" s="5"/>
       <c r="N97" s="2" t="str">
@@ -4345,14 +4364,14 @@
         <v/>
       </c>
       <c r="F98" s="7"/>
-      <c r="G98" s="3"/>
-      <c r="H98" s="4"/>
-      <c r="I98" s="4"/>
-      <c r="J98" s="6" t="str">
+      <c r="G98" s="22"/>
+      <c r="H98" s="23"/>
+      <c r="I98" s="23"/>
+      <c r="J98" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K98" s="5"/>
+      <c r="K98" s="26"/>
       <c r="L98" s="4"/>
       <c r="M98" s="5"/>
       <c r="N98" s="2" t="str">
@@ -4382,14 +4401,14 @@
         <v/>
       </c>
       <c r="F99" s="7"/>
-      <c r="G99" s="3"/>
-      <c r="H99" s="4"/>
-      <c r="I99" s="4"/>
-      <c r="J99" s="6" t="str">
+      <c r="G99" s="22"/>
+      <c r="H99" s="23"/>
+      <c r="I99" s="23"/>
+      <c r="J99" s="25" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K99" s="5"/>
+      <c r="K99" s="26"/>
       <c r="L99" s="4"/>
       <c r="M99" s="5"/>
       <c r="N99" s="2" t="str">
@@ -4419,14 +4438,14 @@
         <v/>
       </c>
       <c r="F100" s="7"/>
-      <c r="G100" s="3"/>
-      <c r="H100" s="4"/>
-      <c r="I100" s="4"/>
-      <c r="J100" s="6" t="str">
+      <c r="G100" s="22"/>
+      <c r="H100" s="23"/>
+      <c r="I100" s="23"/>
+      <c r="J100" s="25" t="str">
         <f t="shared" ref="J100:J131" si="20">IF(OR(I100="",H100=""),"",MAX(0,I100-H100))</f>
         <v/>
       </c>
-      <c r="K100" s="5"/>
+      <c r="K100" s="26"/>
       <c r="L100" s="4"/>
       <c r="M100" s="5"/>
       <c r="N100" s="2" t="str">
@@ -4456,14 +4475,14 @@
         <v/>
       </c>
       <c r="F101" s="7"/>
-      <c r="G101" s="3"/>
-      <c r="H101" s="4"/>
-      <c r="I101" s="4"/>
-      <c r="J101" s="6" t="str">
+      <c r="G101" s="22"/>
+      <c r="H101" s="23"/>
+      <c r="I101" s="23"/>
+      <c r="J101" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K101" s="5"/>
+      <c r="K101" s="26"/>
       <c r="L101" s="4"/>
       <c r="M101" s="5"/>
       <c r="N101" s="2" t="str">
@@ -4493,14 +4512,14 @@
         <v/>
       </c>
       <c r="F102" s="7"/>
-      <c r="G102" s="3"/>
-      <c r="H102" s="4"/>
-      <c r="I102" s="4"/>
-      <c r="J102" s="6" t="str">
+      <c r="G102" s="22"/>
+      <c r="H102" s="23"/>
+      <c r="I102" s="23"/>
+      <c r="J102" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K102" s="5"/>
+      <c r="K102" s="26"/>
       <c r="L102" s="4"/>
       <c r="M102" s="5"/>
       <c r="N102" s="2" t="str">
@@ -4530,14 +4549,14 @@
         <v/>
       </c>
       <c r="F103" s="7"/>
-      <c r="G103" s="3"/>
-      <c r="H103" s="4"/>
-      <c r="I103" s="4"/>
-      <c r="J103" s="6" t="str">
+      <c r="G103" s="22"/>
+      <c r="H103" s="23"/>
+      <c r="I103" s="23"/>
+      <c r="J103" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K103" s="5"/>
+      <c r="K103" s="26"/>
       <c r="L103" s="4"/>
       <c r="M103" s="5"/>
       <c r="N103" s="2" t="str">
@@ -4567,14 +4586,14 @@
         <v/>
       </c>
       <c r="F104" s="7"/>
-      <c r="G104" s="3"/>
-      <c r="H104" s="4"/>
-      <c r="I104" s="4"/>
-      <c r="J104" s="6" t="str">
+      <c r="G104" s="22"/>
+      <c r="H104" s="23"/>
+      <c r="I104" s="23"/>
+      <c r="J104" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K104" s="5"/>
+      <c r="K104" s="26"/>
       <c r="L104" s="4"/>
       <c r="M104" s="5"/>
       <c r="N104" s="2" t="str">
@@ -4604,14 +4623,14 @@
         <v/>
       </c>
       <c r="F105" s="7"/>
-      <c r="G105" s="3"/>
-      <c r="H105" s="4"/>
-      <c r="I105" s="4"/>
-      <c r="J105" s="6" t="str">
+      <c r="G105" s="22"/>
+      <c r="H105" s="23"/>
+      <c r="I105" s="23"/>
+      <c r="J105" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K105" s="5"/>
+      <c r="K105" s="26"/>
       <c r="L105" s="4"/>
       <c r="M105" s="5"/>
       <c r="N105" s="2" t="str">
@@ -4641,14 +4660,14 @@
         <v/>
       </c>
       <c r="F106" s="7"/>
-      <c r="G106" s="3"/>
-      <c r="H106" s="4"/>
-      <c r="I106" s="4"/>
-      <c r="J106" s="6" t="str">
+      <c r="G106" s="22"/>
+      <c r="H106" s="23"/>
+      <c r="I106" s="23"/>
+      <c r="J106" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K106" s="5"/>
+      <c r="K106" s="26"/>
       <c r="L106" s="4"/>
       <c r="M106" s="5"/>
       <c r="N106" s="2" t="str">
@@ -4678,14 +4697,14 @@
         <v/>
       </c>
       <c r="F107" s="7"/>
-      <c r="G107" s="3"/>
-      <c r="H107" s="4"/>
-      <c r="I107" s="4"/>
-      <c r="J107" s="6" t="str">
+      <c r="G107" s="22"/>
+      <c r="H107" s="23"/>
+      <c r="I107" s="23"/>
+      <c r="J107" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K107" s="5"/>
+      <c r="K107" s="26"/>
       <c r="L107" s="4"/>
       <c r="M107" s="5"/>
       <c r="N107" s="2" t="str">
@@ -4715,14 +4734,14 @@
         <v/>
       </c>
       <c r="F108" s="7"/>
-      <c r="G108" s="3"/>
-      <c r="H108" s="4"/>
-      <c r="I108" s="4"/>
-      <c r="J108" s="6" t="str">
+      <c r="G108" s="22"/>
+      <c r="H108" s="23"/>
+      <c r="I108" s="23"/>
+      <c r="J108" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K108" s="5"/>
+      <c r="K108" s="26"/>
       <c r="L108" s="4"/>
       <c r="M108" s="5"/>
       <c r="N108" s="2" t="str">
@@ -4752,14 +4771,14 @@
         <v/>
       </c>
       <c r="F109" s="7"/>
-      <c r="G109" s="3"/>
-      <c r="H109" s="4"/>
-      <c r="I109" s="4"/>
-      <c r="J109" s="6" t="str">
+      <c r="G109" s="22"/>
+      <c r="H109" s="23"/>
+      <c r="I109" s="23"/>
+      <c r="J109" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K109" s="5"/>
+      <c r="K109" s="26"/>
       <c r="L109" s="4"/>
       <c r="M109" s="5"/>
       <c r="N109" s="2" t="str">
@@ -4789,14 +4808,14 @@
         <v/>
       </c>
       <c r="F110" s="7"/>
-      <c r="G110" s="3"/>
-      <c r="H110" s="4"/>
-      <c r="I110" s="4"/>
-      <c r="J110" s="6" t="str">
+      <c r="G110" s="22"/>
+      <c r="H110" s="23"/>
+      <c r="I110" s="23"/>
+      <c r="J110" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K110" s="5"/>
+      <c r="K110" s="26"/>
       <c r="L110" s="4"/>
       <c r="M110" s="5"/>
       <c r="N110" s="2" t="str">
@@ -4826,14 +4845,14 @@
         <v/>
       </c>
       <c r="F111" s="7"/>
-      <c r="G111" s="3"/>
-      <c r="H111" s="4"/>
-      <c r="I111" s="4"/>
-      <c r="J111" s="6" t="str">
+      <c r="G111" s="22"/>
+      <c r="H111" s="23"/>
+      <c r="I111" s="23"/>
+      <c r="J111" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K111" s="5"/>
+      <c r="K111" s="26"/>
       <c r="L111" s="4"/>
       <c r="M111" s="5"/>
       <c r="N111" s="2" t="str">
@@ -4863,14 +4882,14 @@
         <v/>
       </c>
       <c r="F112" s="7"/>
-      <c r="G112" s="3"/>
-      <c r="H112" s="4"/>
-      <c r="I112" s="4"/>
-      <c r="J112" s="6" t="str">
+      <c r="G112" s="22"/>
+      <c r="H112" s="23"/>
+      <c r="I112" s="23"/>
+      <c r="J112" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K112" s="5"/>
+      <c r="K112" s="26"/>
       <c r="L112" s="4"/>
       <c r="M112" s="5"/>
       <c r="N112" s="2" t="str">
@@ -4900,14 +4919,14 @@
         <v/>
       </c>
       <c r="F113" s="7"/>
-      <c r="G113" s="3"/>
-      <c r="H113" s="4"/>
-      <c r="I113" s="4"/>
-      <c r="J113" s="6" t="str">
+      <c r="G113" s="22"/>
+      <c r="H113" s="23"/>
+      <c r="I113" s="23"/>
+      <c r="J113" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K113" s="5"/>
+      <c r="K113" s="26"/>
       <c r="L113" s="4"/>
       <c r="M113" s="5"/>
       <c r="N113" s="2" t="str">
@@ -4937,14 +4956,14 @@
         <v/>
       </c>
       <c r="F114" s="7"/>
-      <c r="G114" s="3"/>
-      <c r="H114" s="4"/>
-      <c r="I114" s="4"/>
-      <c r="J114" s="6" t="str">
+      <c r="G114" s="22"/>
+      <c r="H114" s="23"/>
+      <c r="I114" s="23"/>
+      <c r="J114" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K114" s="5"/>
+      <c r="K114" s="26"/>
       <c r="L114" s="4"/>
       <c r="M114" s="5"/>
       <c r="N114" s="2" t="str">
@@ -4974,14 +4993,14 @@
         <v/>
       </c>
       <c r="F115" s="7"/>
-      <c r="G115" s="3"/>
-      <c r="H115" s="4"/>
-      <c r="I115" s="4"/>
-      <c r="J115" s="6" t="str">
+      <c r="G115" s="22"/>
+      <c r="H115" s="23"/>
+      <c r="I115" s="23"/>
+      <c r="J115" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K115" s="5"/>
+      <c r="K115" s="26"/>
       <c r="L115" s="4"/>
       <c r="M115" s="5"/>
       <c r="N115" s="2" t="str">
@@ -5011,14 +5030,14 @@
         <v/>
       </c>
       <c r="F116" s="7"/>
-      <c r="G116" s="3"/>
-      <c r="H116" s="4"/>
-      <c r="I116" s="4"/>
-      <c r="J116" s="6" t="str">
+      <c r="G116" s="22"/>
+      <c r="H116" s="23"/>
+      <c r="I116" s="23"/>
+      <c r="J116" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K116" s="5"/>
+      <c r="K116" s="26"/>
       <c r="L116" s="4"/>
       <c r="M116" s="5"/>
       <c r="N116" s="2" t="str">
@@ -5048,14 +5067,14 @@
         <v/>
       </c>
       <c r="F117" s="7"/>
-      <c r="G117" s="3"/>
-      <c r="H117" s="4"/>
-      <c r="I117" s="4"/>
-      <c r="J117" s="6" t="str">
+      <c r="G117" s="22"/>
+      <c r="H117" s="23"/>
+      <c r="I117" s="23"/>
+      <c r="J117" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K117" s="5"/>
+      <c r="K117" s="26"/>
       <c r="L117" s="4"/>
       <c r="M117" s="5"/>
       <c r="N117" s="2" t="str">
@@ -5085,14 +5104,14 @@
         <v/>
       </c>
       <c r="F118" s="7"/>
-      <c r="G118" s="3"/>
-      <c r="H118" s="4"/>
-      <c r="I118" s="4"/>
-      <c r="J118" s="6" t="str">
+      <c r="G118" s="22"/>
+      <c r="H118" s="23"/>
+      <c r="I118" s="23"/>
+      <c r="J118" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K118" s="5"/>
+      <c r="K118" s="26"/>
       <c r="L118" s="4"/>
       <c r="M118" s="5"/>
       <c r="N118" s="2" t="str">
@@ -5122,14 +5141,14 @@
         <v/>
       </c>
       <c r="F119" s="7"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="4"/>
-      <c r="I119" s="4"/>
-      <c r="J119" s="6" t="str">
+      <c r="G119" s="22"/>
+      <c r="H119" s="23"/>
+      <c r="I119" s="23"/>
+      <c r="J119" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K119" s="5"/>
+      <c r="K119" s="26"/>
       <c r="L119" s="4"/>
       <c r="M119" s="5"/>
       <c r="N119" s="2" t="str">
@@ -5159,14 +5178,14 @@
         <v/>
       </c>
       <c r="F120" s="7"/>
-      <c r="G120" s="3"/>
-      <c r="H120" s="4"/>
-      <c r="I120" s="4"/>
-      <c r="J120" s="6" t="str">
+      <c r="G120" s="22"/>
+      <c r="H120" s="23"/>
+      <c r="I120" s="23"/>
+      <c r="J120" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K120" s="5"/>
+      <c r="K120" s="26"/>
       <c r="L120" s="4"/>
       <c r="M120" s="5"/>
       <c r="N120" s="2" t="str">
@@ -5196,14 +5215,14 @@
         <v/>
       </c>
       <c r="F121" s="7"/>
-      <c r="G121" s="3"/>
-      <c r="H121" s="4"/>
-      <c r="I121" s="4"/>
-      <c r="J121" s="6" t="str">
+      <c r="G121" s="22"/>
+      <c r="H121" s="23"/>
+      <c r="I121" s="23"/>
+      <c r="J121" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K121" s="5"/>
+      <c r="K121" s="26"/>
       <c r="L121" s="4"/>
       <c r="M121" s="5"/>
       <c r="N121" s="2" t="str">
@@ -5233,14 +5252,14 @@
         <v/>
       </c>
       <c r="F122" s="7"/>
-      <c r="G122" s="3"/>
-      <c r="H122" s="4"/>
-      <c r="I122" s="4"/>
-      <c r="J122" s="6" t="str">
+      <c r="G122" s="22"/>
+      <c r="H122" s="23"/>
+      <c r="I122" s="23"/>
+      <c r="J122" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K122" s="5"/>
+      <c r="K122" s="26"/>
       <c r="L122" s="4"/>
       <c r="M122" s="5"/>
       <c r="N122" s="2" t="str">
@@ -5270,14 +5289,14 @@
         <v/>
       </c>
       <c r="F123" s="7"/>
-      <c r="G123" s="3"/>
-      <c r="H123" s="4"/>
-      <c r="I123" s="4"/>
-      <c r="J123" s="6" t="str">
+      <c r="G123" s="22"/>
+      <c r="H123" s="23"/>
+      <c r="I123" s="23"/>
+      <c r="J123" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K123" s="5"/>
+      <c r="K123" s="26"/>
       <c r="L123" s="4"/>
       <c r="M123" s="5"/>
       <c r="N123" s="2" t="str">
@@ -5307,14 +5326,14 @@
         <v/>
       </c>
       <c r="F124" s="7"/>
-      <c r="G124" s="3"/>
-      <c r="H124" s="4"/>
-      <c r="I124" s="4"/>
-      <c r="J124" s="6" t="str">
+      <c r="G124" s="22"/>
+      <c r="H124" s="23"/>
+      <c r="I124" s="23"/>
+      <c r="J124" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K124" s="5"/>
+      <c r="K124" s="26"/>
       <c r="L124" s="4"/>
       <c r="M124" s="5"/>
       <c r="N124" s="2" t="str">
@@ -5344,14 +5363,14 @@
         <v/>
       </c>
       <c r="F125" s="7"/>
-      <c r="G125" s="3"/>
-      <c r="H125" s="4"/>
-      <c r="I125" s="4"/>
-      <c r="J125" s="6" t="str">
+      <c r="G125" s="22"/>
+      <c r="H125" s="23"/>
+      <c r="I125" s="23"/>
+      <c r="J125" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K125" s="5"/>
+      <c r="K125" s="26"/>
       <c r="L125" s="4"/>
       <c r="M125" s="5"/>
       <c r="N125" s="2" t="str">
@@ -5381,14 +5400,14 @@
         <v/>
       </c>
       <c r="F126" s="7"/>
-      <c r="G126" s="3"/>
-      <c r="H126" s="4"/>
-      <c r="I126" s="4"/>
-      <c r="J126" s="6" t="str">
+      <c r="G126" s="22"/>
+      <c r="H126" s="23"/>
+      <c r="I126" s="23"/>
+      <c r="J126" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K126" s="5"/>
+      <c r="K126" s="26"/>
       <c r="L126" s="4"/>
       <c r="M126" s="5"/>
       <c r="N126" s="2" t="str">
@@ -5418,14 +5437,14 @@
         <v/>
       </c>
       <c r="F127" s="7"/>
-      <c r="G127" s="3"/>
-      <c r="H127" s="4"/>
-      <c r="I127" s="4"/>
-      <c r="J127" s="6" t="str">
+      <c r="G127" s="22"/>
+      <c r="H127" s="23"/>
+      <c r="I127" s="23"/>
+      <c r="J127" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K127" s="5"/>
+      <c r="K127" s="26"/>
       <c r="L127" s="4"/>
       <c r="M127" s="5"/>
       <c r="N127" s="2" t="str">
@@ -5455,14 +5474,14 @@
         <v/>
       </c>
       <c r="F128" s="7"/>
-      <c r="G128" s="3"/>
-      <c r="H128" s="4"/>
-      <c r="I128" s="4"/>
-      <c r="J128" s="6" t="str">
+      <c r="G128" s="22"/>
+      <c r="H128" s="23"/>
+      <c r="I128" s="23"/>
+      <c r="J128" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K128" s="5"/>
+      <c r="K128" s="26"/>
       <c r="L128" s="4"/>
       <c r="M128" s="5"/>
       <c r="N128" s="2" t="str">
@@ -5492,14 +5511,14 @@
         <v/>
       </c>
       <c r="F129" s="7"/>
-      <c r="G129" s="3"/>
-      <c r="H129" s="4"/>
-      <c r="I129" s="4"/>
-      <c r="J129" s="6" t="str">
+      <c r="G129" s="22"/>
+      <c r="H129" s="23"/>
+      <c r="I129" s="23"/>
+      <c r="J129" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K129" s="5"/>
+      <c r="K129" s="26"/>
       <c r="L129" s="4"/>
       <c r="M129" s="5"/>
       <c r="N129" s="2" t="str">
@@ -5529,14 +5548,14 @@
         <v/>
       </c>
       <c r="F130" s="7"/>
-      <c r="G130" s="3"/>
-      <c r="H130" s="4"/>
-      <c r="I130" s="4"/>
-      <c r="J130" s="6" t="str">
+      <c r="G130" s="22"/>
+      <c r="H130" s="23"/>
+      <c r="I130" s="23"/>
+      <c r="J130" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K130" s="5"/>
+      <c r="K130" s="26"/>
       <c r="L130" s="4"/>
       <c r="M130" s="5"/>
       <c r="N130" s="2" t="str">
@@ -5566,14 +5585,14 @@
         <v/>
       </c>
       <c r="F131" s="7"/>
-      <c r="G131" s="3"/>
-      <c r="H131" s="4"/>
-      <c r="I131" s="4"/>
-      <c r="J131" s="6" t="str">
+      <c r="G131" s="22"/>
+      <c r="H131" s="23"/>
+      <c r="I131" s="23"/>
+      <c r="J131" s="25" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K131" s="5"/>
+      <c r="K131" s="26"/>
       <c r="L131" s="4"/>
       <c r="M131" s="5"/>
       <c r="N131" s="2" t="str">
@@ -5603,14 +5622,14 @@
         <v/>
       </c>
       <c r="F132" s="7"/>
-      <c r="G132" s="3"/>
-      <c r="H132" s="4"/>
-      <c r="I132" s="4"/>
-      <c r="J132" s="6" t="str">
+      <c r="G132" s="22"/>
+      <c r="H132" s="23"/>
+      <c r="I132" s="23"/>
+      <c r="J132" s="25" t="str">
         <f t="shared" ref="J132:J163" si="26">IF(OR(I132="",H132=""),"",MAX(0,I132-H132))</f>
         <v/>
       </c>
-      <c r="K132" s="5"/>
+      <c r="K132" s="26"/>
       <c r="L132" s="4"/>
       <c r="M132" s="5"/>
       <c r="N132" s="2" t="str">
@@ -5640,14 +5659,14 @@
         <v/>
       </c>
       <c r="F133" s="7"/>
-      <c r="G133" s="3"/>
-      <c r="H133" s="4"/>
-      <c r="I133" s="4"/>
-      <c r="J133" s="6" t="str">
+      <c r="G133" s="22"/>
+      <c r="H133" s="23"/>
+      <c r="I133" s="23"/>
+      <c r="J133" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K133" s="5"/>
+      <c r="K133" s="26"/>
       <c r="L133" s="4"/>
       <c r="M133" s="5"/>
       <c r="N133" s="2" t="str">
@@ -5677,14 +5696,14 @@
         <v/>
       </c>
       <c r="F134" s="7"/>
-      <c r="G134" s="3"/>
-      <c r="H134" s="4"/>
-      <c r="I134" s="4"/>
-      <c r="J134" s="6" t="str">
+      <c r="G134" s="22"/>
+      <c r="H134" s="23"/>
+      <c r="I134" s="23"/>
+      <c r="J134" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K134" s="5"/>
+      <c r="K134" s="26"/>
       <c r="L134" s="4"/>
       <c r="M134" s="5"/>
       <c r="N134" s="2" t="str">
@@ -5714,14 +5733,14 @@
         <v/>
       </c>
       <c r="F135" s="7"/>
-      <c r="G135" s="3"/>
-      <c r="H135" s="4"/>
-      <c r="I135" s="4"/>
-      <c r="J135" s="6" t="str">
+      <c r="G135" s="22"/>
+      <c r="H135" s="23"/>
+      <c r="I135" s="23"/>
+      <c r="J135" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K135" s="5"/>
+      <c r="K135" s="26"/>
       <c r="L135" s="4"/>
       <c r="M135" s="5"/>
       <c r="N135" s="2" t="str">
@@ -5751,14 +5770,14 @@
         <v/>
       </c>
       <c r="F136" s="7"/>
-      <c r="G136" s="3"/>
-      <c r="H136" s="4"/>
-      <c r="I136" s="4"/>
-      <c r="J136" s="6" t="str">
+      <c r="G136" s="22"/>
+      <c r="H136" s="23"/>
+      <c r="I136" s="23"/>
+      <c r="J136" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K136" s="5"/>
+      <c r="K136" s="26"/>
       <c r="L136" s="4"/>
       <c r="M136" s="5"/>
       <c r="N136" s="2" t="str">
@@ -5788,14 +5807,14 @@
         <v/>
       </c>
       <c r="F137" s="7"/>
-      <c r="G137" s="3"/>
-      <c r="H137" s="4"/>
-      <c r="I137" s="4"/>
-      <c r="J137" s="6" t="str">
+      <c r="G137" s="22"/>
+      <c r="H137" s="23"/>
+      <c r="I137" s="23"/>
+      <c r="J137" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K137" s="5"/>
+      <c r="K137" s="26"/>
       <c r="L137" s="4"/>
       <c r="M137" s="5"/>
       <c r="N137" s="2" t="str">
@@ -5825,14 +5844,14 @@
         <v/>
       </c>
       <c r="F138" s="7"/>
-      <c r="G138" s="3"/>
-      <c r="H138" s="4"/>
-      <c r="I138" s="4"/>
-      <c r="J138" s="6" t="str">
+      <c r="G138" s="22"/>
+      <c r="H138" s="23"/>
+      <c r="I138" s="23"/>
+      <c r="J138" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K138" s="5"/>
+      <c r="K138" s="26"/>
       <c r="L138" s="4"/>
       <c r="M138" s="5"/>
       <c r="N138" s="2" t="str">
@@ -5862,14 +5881,14 @@
         <v/>
       </c>
       <c r="F139" s="7"/>
-      <c r="G139" s="3"/>
-      <c r="H139" s="4"/>
-      <c r="I139" s="4"/>
-      <c r="J139" s="6" t="str">
+      <c r="G139" s="22"/>
+      <c r="H139" s="23"/>
+      <c r="I139" s="23"/>
+      <c r="J139" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K139" s="5"/>
+      <c r="K139" s="26"/>
       <c r="L139" s="4"/>
       <c r="M139" s="5"/>
       <c r="N139" s="2" t="str">
@@ -5899,14 +5918,14 @@
         <v/>
       </c>
       <c r="F140" s="7"/>
-      <c r="G140" s="3"/>
-      <c r="H140" s="4"/>
-      <c r="I140" s="4"/>
-      <c r="J140" s="6" t="str">
+      <c r="G140" s="22"/>
+      <c r="H140" s="23"/>
+      <c r="I140" s="23"/>
+      <c r="J140" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K140" s="5"/>
+      <c r="K140" s="26"/>
       <c r="L140" s="4"/>
       <c r="M140" s="5"/>
       <c r="N140" s="2" t="str">
@@ -5936,14 +5955,14 @@
         <v/>
       </c>
       <c r="F141" s="7"/>
-      <c r="G141" s="3"/>
-      <c r="H141" s="4"/>
-      <c r="I141" s="4"/>
-      <c r="J141" s="6" t="str">
+      <c r="G141" s="22"/>
+      <c r="H141" s="23"/>
+      <c r="I141" s="23"/>
+      <c r="J141" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K141" s="5"/>
+      <c r="K141" s="26"/>
       <c r="L141" s="4"/>
       <c r="M141" s="5"/>
       <c r="N141" s="2" t="str">
@@ -5973,14 +5992,14 @@
         <v/>
       </c>
       <c r="F142" s="7"/>
-      <c r="G142" s="3"/>
-      <c r="H142" s="4"/>
-      <c r="I142" s="4"/>
-      <c r="J142" s="6" t="str">
+      <c r="G142" s="22"/>
+      <c r="H142" s="23"/>
+      <c r="I142" s="23"/>
+      <c r="J142" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K142" s="5"/>
+      <c r="K142" s="26"/>
       <c r="L142" s="4"/>
       <c r="M142" s="5"/>
       <c r="N142" s="2" t="str">
@@ -6010,14 +6029,14 @@
         <v/>
       </c>
       <c r="F143" s="7"/>
-      <c r="G143" s="3"/>
-      <c r="H143" s="4"/>
-      <c r="I143" s="4"/>
-      <c r="J143" s="6" t="str">
+      <c r="G143" s="22"/>
+      <c r="H143" s="23"/>
+      <c r="I143" s="23"/>
+      <c r="J143" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K143" s="5"/>
+      <c r="K143" s="26"/>
       <c r="L143" s="4"/>
       <c r="M143" s="5"/>
       <c r="N143" s="2" t="str">
@@ -6047,14 +6066,14 @@
         <v/>
       </c>
       <c r="F144" s="7"/>
-      <c r="G144" s="3"/>
-      <c r="H144" s="4"/>
-      <c r="I144" s="4"/>
-      <c r="J144" s="6" t="str">
+      <c r="G144" s="22"/>
+      <c r="H144" s="23"/>
+      <c r="I144" s="23"/>
+      <c r="J144" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K144" s="5"/>
+      <c r="K144" s="26"/>
       <c r="L144" s="4"/>
       <c r="M144" s="5"/>
       <c r="N144" s="2" t="str">
@@ -6084,14 +6103,14 @@
         <v/>
       </c>
       <c r="F145" s="7"/>
-      <c r="G145" s="3"/>
-      <c r="H145" s="4"/>
-      <c r="I145" s="4"/>
-      <c r="J145" s="6" t="str">
+      <c r="G145" s="22"/>
+      <c r="H145" s="23"/>
+      <c r="I145" s="23"/>
+      <c r="J145" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K145" s="5"/>
+      <c r="K145" s="26"/>
       <c r="L145" s="4"/>
       <c r="M145" s="5"/>
       <c r="N145" s="2" t="str">
@@ -6121,14 +6140,14 @@
         <v/>
       </c>
       <c r="F146" s="7"/>
-      <c r="G146" s="3"/>
-      <c r="H146" s="4"/>
-      <c r="I146" s="4"/>
-      <c r="J146" s="6" t="str">
+      <c r="G146" s="22"/>
+      <c r="H146" s="23"/>
+      <c r="I146" s="23"/>
+      <c r="J146" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K146" s="5"/>
+      <c r="K146" s="26"/>
       <c r="L146" s="4"/>
       <c r="M146" s="5"/>
       <c r="N146" s="2" t="str">
@@ -6158,14 +6177,14 @@
         <v/>
       </c>
       <c r="F147" s="7"/>
-      <c r="G147" s="3"/>
-      <c r="H147" s="4"/>
-      <c r="I147" s="4"/>
-      <c r="J147" s="6" t="str">
+      <c r="G147" s="22"/>
+      <c r="H147" s="23"/>
+      <c r="I147" s="23"/>
+      <c r="J147" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K147" s="5"/>
+      <c r="K147" s="26"/>
       <c r="L147" s="4"/>
       <c r="M147" s="5"/>
       <c r="N147" s="2" t="str">
@@ -6195,14 +6214,14 @@
         <v/>
       </c>
       <c r="F148" s="7"/>
-      <c r="G148" s="3"/>
-      <c r="H148" s="4"/>
-      <c r="I148" s="4"/>
-      <c r="J148" s="6" t="str">
+      <c r="G148" s="22"/>
+      <c r="H148" s="23"/>
+      <c r="I148" s="23"/>
+      <c r="J148" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K148" s="5"/>
+      <c r="K148" s="26"/>
       <c r="L148" s="4"/>
       <c r="M148" s="5"/>
       <c r="N148" s="2" t="str">
@@ -6232,14 +6251,14 @@
         <v/>
       </c>
       <c r="F149" s="7"/>
-      <c r="G149" s="3"/>
-      <c r="H149" s="4"/>
-      <c r="I149" s="4"/>
-      <c r="J149" s="6" t="str">
+      <c r="G149" s="22"/>
+      <c r="H149" s="23"/>
+      <c r="I149" s="23"/>
+      <c r="J149" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K149" s="5"/>
+      <c r="K149" s="26"/>
       <c r="L149" s="4"/>
       <c r="M149" s="5"/>
       <c r="N149" s="2" t="str">
@@ -6269,14 +6288,14 @@
         <v/>
       </c>
       <c r="F150" s="7"/>
-      <c r="G150" s="3"/>
-      <c r="H150" s="4"/>
-      <c r="I150" s="4"/>
-      <c r="J150" s="6" t="str">
+      <c r="G150" s="22"/>
+      <c r="H150" s="23"/>
+      <c r="I150" s="23"/>
+      <c r="J150" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K150" s="5"/>
+      <c r="K150" s="26"/>
       <c r="L150" s="4"/>
       <c r="M150" s="5"/>
       <c r="N150" s="2" t="str">
@@ -6306,14 +6325,14 @@
         <v/>
       </c>
       <c r="F151" s="7"/>
-      <c r="G151" s="3"/>
-      <c r="H151" s="4"/>
-      <c r="I151" s="4"/>
-      <c r="J151" s="6" t="str">
+      <c r="G151" s="22"/>
+      <c r="H151" s="23"/>
+      <c r="I151" s="23"/>
+      <c r="J151" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K151" s="5"/>
+      <c r="K151" s="26"/>
       <c r="L151" s="4"/>
       <c r="M151" s="5"/>
       <c r="N151" s="2" t="str">
@@ -6343,14 +6362,14 @@
         <v/>
       </c>
       <c r="F152" s="7"/>
-      <c r="G152" s="3"/>
-      <c r="H152" s="4"/>
-      <c r="I152" s="4"/>
-      <c r="J152" s="6" t="str">
+      <c r="G152" s="22"/>
+      <c r="H152" s="23"/>
+      <c r="I152" s="23"/>
+      <c r="J152" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K152" s="5"/>
+      <c r="K152" s="26"/>
       <c r="L152" s="4"/>
       <c r="M152" s="5"/>
       <c r="N152" s="2" t="str">
@@ -6380,14 +6399,14 @@
         <v/>
       </c>
       <c r="F153" s="7"/>
-      <c r="G153" s="3"/>
-      <c r="H153" s="4"/>
-      <c r="I153" s="4"/>
-      <c r="J153" s="6" t="str">
+      <c r="G153" s="22"/>
+      <c r="H153" s="23"/>
+      <c r="I153" s="23"/>
+      <c r="J153" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K153" s="5"/>
+      <c r="K153" s="26"/>
       <c r="L153" s="4"/>
       <c r="M153" s="5"/>
       <c r="N153" s="2" t="str">
@@ -6417,14 +6436,14 @@
         <v/>
       </c>
       <c r="F154" s="7"/>
-      <c r="G154" s="3"/>
-      <c r="H154" s="4"/>
-      <c r="I154" s="4"/>
-      <c r="J154" s="6" t="str">
+      <c r="G154" s="22"/>
+      <c r="H154" s="23"/>
+      <c r="I154" s="23"/>
+      <c r="J154" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K154" s="5"/>
+      <c r="K154" s="26"/>
       <c r="L154" s="4"/>
       <c r="M154" s="5"/>
       <c r="N154" s="2" t="str">
@@ -6454,14 +6473,14 @@
         <v/>
       </c>
       <c r="F155" s="7"/>
-      <c r="G155" s="3"/>
-      <c r="H155" s="4"/>
-      <c r="I155" s="4"/>
-      <c r="J155" s="6" t="str">
+      <c r="G155" s="22"/>
+      <c r="H155" s="23"/>
+      <c r="I155" s="23"/>
+      <c r="J155" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K155" s="5"/>
+      <c r="K155" s="26"/>
       <c r="L155" s="4"/>
       <c r="M155" s="5"/>
       <c r="N155" s="2" t="str">
@@ -6491,14 +6510,14 @@
         <v/>
       </c>
       <c r="F156" s="7"/>
-      <c r="G156" s="3"/>
-      <c r="H156" s="4"/>
-      <c r="I156" s="4"/>
-      <c r="J156" s="6" t="str">
+      <c r="G156" s="22"/>
+      <c r="H156" s="23"/>
+      <c r="I156" s="23"/>
+      <c r="J156" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K156" s="5"/>
+      <c r="K156" s="26"/>
       <c r="L156" s="4"/>
       <c r="M156" s="5"/>
       <c r="N156" s="2" t="str">
@@ -6528,14 +6547,14 @@
         <v/>
       </c>
       <c r="F157" s="7"/>
-      <c r="G157" s="3"/>
-      <c r="H157" s="4"/>
-      <c r="I157" s="4"/>
-      <c r="J157" s="6" t="str">
+      <c r="G157" s="22"/>
+      <c r="H157" s="23"/>
+      <c r="I157" s="23"/>
+      <c r="J157" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K157" s="5"/>
+      <c r="K157" s="26"/>
       <c r="L157" s="4"/>
       <c r="M157" s="5"/>
       <c r="N157" s="2" t="str">
@@ -6565,14 +6584,14 @@
         <v/>
       </c>
       <c r="F158" s="7"/>
-      <c r="G158" s="3"/>
-      <c r="H158" s="4"/>
-      <c r="I158" s="4"/>
-      <c r="J158" s="6" t="str">
+      <c r="G158" s="22"/>
+      <c r="H158" s="23"/>
+      <c r="I158" s="23"/>
+      <c r="J158" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K158" s="5"/>
+      <c r="K158" s="26"/>
       <c r="L158" s="4"/>
       <c r="M158" s="5"/>
       <c r="N158" s="2" t="str">
@@ -6602,14 +6621,14 @@
         <v/>
       </c>
       <c r="F159" s="7"/>
-      <c r="G159" s="3"/>
-      <c r="H159" s="4"/>
-      <c r="I159" s="4"/>
-      <c r="J159" s="6" t="str">
+      <c r="G159" s="22"/>
+      <c r="H159" s="23"/>
+      <c r="I159" s="23"/>
+      <c r="J159" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K159" s="5"/>
+      <c r="K159" s="26"/>
       <c r="L159" s="4"/>
       <c r="M159" s="5"/>
       <c r="N159" s="2" t="str">
@@ -6639,14 +6658,14 @@
         <v/>
       </c>
       <c r="F160" s="7"/>
-      <c r="G160" s="3"/>
-      <c r="H160" s="4"/>
-      <c r="I160" s="4"/>
-      <c r="J160" s="6" t="str">
+      <c r="G160" s="22"/>
+      <c r="H160" s="23"/>
+      <c r="I160" s="23"/>
+      <c r="J160" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K160" s="5"/>
+      <c r="K160" s="26"/>
       <c r="L160" s="4"/>
       <c r="M160" s="5"/>
       <c r="N160" s="2" t="str">
@@ -6676,14 +6695,14 @@
         <v/>
       </c>
       <c r="F161" s="7"/>
-      <c r="G161" s="3"/>
-      <c r="H161" s="4"/>
-      <c r="I161" s="4"/>
-      <c r="J161" s="6" t="str">
+      <c r="G161" s="22"/>
+      <c r="H161" s="23"/>
+      <c r="I161" s="23"/>
+      <c r="J161" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K161" s="5"/>
+      <c r="K161" s="26"/>
       <c r="L161" s="4"/>
       <c r="M161" s="5"/>
       <c r="N161" s="2" t="str">
@@ -6713,14 +6732,14 @@
         <v/>
       </c>
       <c r="F162" s="7"/>
-      <c r="G162" s="3"/>
-      <c r="H162" s="4"/>
-      <c r="I162" s="4"/>
-      <c r="J162" s="6" t="str">
+      <c r="G162" s="22"/>
+      <c r="H162" s="23"/>
+      <c r="I162" s="23"/>
+      <c r="J162" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K162" s="5"/>
+      <c r="K162" s="26"/>
       <c r="L162" s="4"/>
       <c r="M162" s="5"/>
       <c r="N162" s="2" t="str">
@@ -6750,14 +6769,14 @@
         <v/>
       </c>
       <c r="F163" s="7"/>
-      <c r="G163" s="3"/>
-      <c r="H163" s="4"/>
-      <c r="I163" s="4"/>
-      <c r="J163" s="6" t="str">
+      <c r="G163" s="22"/>
+      <c r="H163" s="23"/>
+      <c r="I163" s="23"/>
+      <c r="J163" s="25" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K163" s="5"/>
+      <c r="K163" s="26"/>
       <c r="L163" s="4"/>
       <c r="M163" s="5"/>
       <c r="N163" s="2" t="str">
@@ -6787,14 +6806,14 @@
         <v/>
       </c>
       <c r="F164" s="7"/>
-      <c r="G164" s="3"/>
-      <c r="H164" s="4"/>
-      <c r="I164" s="4"/>
-      <c r="J164" s="6" t="str">
+      <c r="G164" s="22"/>
+      <c r="H164" s="23"/>
+      <c r="I164" s="23"/>
+      <c r="J164" s="25" t="str">
         <f t="shared" ref="J164:J195" si="32">IF(OR(I164="",H164=""),"",MAX(0,I164-H164))</f>
         <v/>
       </c>
-      <c r="K164" s="5"/>
+      <c r="K164" s="26"/>
       <c r="L164" s="4"/>
       <c r="M164" s="5"/>
       <c r="N164" s="2" t="str">
@@ -6824,14 +6843,14 @@
         <v/>
       </c>
       <c r="F165" s="7"/>
-      <c r="G165" s="3"/>
-      <c r="H165" s="4"/>
-      <c r="I165" s="4"/>
-      <c r="J165" s="6" t="str">
+      <c r="G165" s="22"/>
+      <c r="H165" s="23"/>
+      <c r="I165" s="23"/>
+      <c r="J165" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K165" s="5"/>
+      <c r="K165" s="26"/>
       <c r="L165" s="4"/>
       <c r="M165" s="5"/>
       <c r="N165" s="2" t="str">
@@ -6861,14 +6880,14 @@
         <v/>
       </c>
       <c r="F166" s="7"/>
-      <c r="G166" s="3"/>
-      <c r="H166" s="4"/>
-      <c r="I166" s="4"/>
-      <c r="J166" s="6" t="str">
+      <c r="G166" s="22"/>
+      <c r="H166" s="23"/>
+      <c r="I166" s="23"/>
+      <c r="J166" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K166" s="5"/>
+      <c r="K166" s="26"/>
       <c r="L166" s="4"/>
       <c r="M166" s="5"/>
       <c r="N166" s="2" t="str">
@@ -6898,14 +6917,14 @@
         <v/>
       </c>
       <c r="F167" s="7"/>
-      <c r="G167" s="3"/>
-      <c r="H167" s="4"/>
-      <c r="I167" s="4"/>
-      <c r="J167" s="6" t="str">
+      <c r="G167" s="22"/>
+      <c r="H167" s="23"/>
+      <c r="I167" s="23"/>
+      <c r="J167" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K167" s="5"/>
+      <c r="K167" s="26"/>
       <c r="L167" s="4"/>
       <c r="M167" s="5"/>
       <c r="N167" s="2" t="str">
@@ -6935,14 +6954,14 @@
         <v/>
       </c>
       <c r="F168" s="7"/>
-      <c r="G168" s="3"/>
-      <c r="H168" s="4"/>
-      <c r="I168" s="4"/>
-      <c r="J168" s="6" t="str">
+      <c r="G168" s="22"/>
+      <c r="H168" s="23"/>
+      <c r="I168" s="23"/>
+      <c r="J168" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K168" s="5"/>
+      <c r="K168" s="26"/>
       <c r="L168" s="4"/>
       <c r="M168" s="5"/>
       <c r="N168" s="2" t="str">
@@ -6972,14 +6991,14 @@
         <v/>
       </c>
       <c r="F169" s="7"/>
-      <c r="G169" s="3"/>
-      <c r="H169" s="4"/>
-      <c r="I169" s="4"/>
-      <c r="J169" s="6" t="str">
+      <c r="G169" s="22"/>
+      <c r="H169" s="23"/>
+      <c r="I169" s="23"/>
+      <c r="J169" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K169" s="5"/>
+      <c r="K169" s="26"/>
       <c r="L169" s="4"/>
       <c r="M169" s="5"/>
       <c r="N169" s="2" t="str">
@@ -7009,14 +7028,14 @@
         <v/>
       </c>
       <c r="F170" s="7"/>
-      <c r="G170" s="3"/>
-      <c r="H170" s="4"/>
-      <c r="I170" s="4"/>
-      <c r="J170" s="6" t="str">
+      <c r="G170" s="22"/>
+      <c r="H170" s="23"/>
+      <c r="I170" s="23"/>
+      <c r="J170" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K170" s="5"/>
+      <c r="K170" s="26"/>
       <c r="L170" s="4"/>
       <c r="M170" s="5"/>
       <c r="N170" s="2" t="str">
@@ -7046,14 +7065,14 @@
         <v/>
       </c>
       <c r="F171" s="7"/>
-      <c r="G171" s="3"/>
-      <c r="H171" s="4"/>
-      <c r="I171" s="4"/>
-      <c r="J171" s="6" t="str">
+      <c r="G171" s="22"/>
+      <c r="H171" s="23"/>
+      <c r="I171" s="23"/>
+      <c r="J171" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K171" s="5"/>
+      <c r="K171" s="26"/>
       <c r="L171" s="4"/>
       <c r="M171" s="5"/>
       <c r="N171" s="2" t="str">
@@ -7083,14 +7102,14 @@
         <v/>
       </c>
       <c r="F172" s="7"/>
-      <c r="G172" s="3"/>
-      <c r="H172" s="4"/>
-      <c r="I172" s="4"/>
-      <c r="J172" s="6" t="str">
+      <c r="G172" s="22"/>
+      <c r="H172" s="23"/>
+      <c r="I172" s="23"/>
+      <c r="J172" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K172" s="5"/>
+      <c r="K172" s="26"/>
       <c r="L172" s="4"/>
       <c r="M172" s="5"/>
       <c r="N172" s="2" t="str">
@@ -7120,14 +7139,14 @@
         <v/>
       </c>
       <c r="F173" s="7"/>
-      <c r="G173" s="3"/>
-      <c r="H173" s="4"/>
-      <c r="I173" s="4"/>
-      <c r="J173" s="6" t="str">
+      <c r="G173" s="22"/>
+      <c r="H173" s="23"/>
+      <c r="I173" s="23"/>
+      <c r="J173" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K173" s="5"/>
+      <c r="K173" s="26"/>
       <c r="L173" s="4"/>
       <c r="M173" s="5"/>
       <c r="N173" s="2" t="str">
@@ -7157,14 +7176,14 @@
         <v/>
       </c>
       <c r="F174" s="7"/>
-      <c r="G174" s="3"/>
-      <c r="H174" s="4"/>
-      <c r="I174" s="4"/>
-      <c r="J174" s="6" t="str">
+      <c r="G174" s="22"/>
+      <c r="H174" s="23"/>
+      <c r="I174" s="23"/>
+      <c r="J174" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K174" s="5"/>
+      <c r="K174" s="26"/>
       <c r="L174" s="4"/>
       <c r="M174" s="5"/>
       <c r="N174" s="2" t="str">
@@ -7194,14 +7213,14 @@
         <v/>
       </c>
       <c r="F175" s="7"/>
-      <c r="G175" s="3"/>
-      <c r="H175" s="4"/>
-      <c r="I175" s="4"/>
-      <c r="J175" s="6" t="str">
+      <c r="G175" s="22"/>
+      <c r="H175" s="23"/>
+      <c r="I175" s="23"/>
+      <c r="J175" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K175" s="5"/>
+      <c r="K175" s="26"/>
       <c r="L175" s="4"/>
       <c r="M175" s="5"/>
       <c r="N175" s="2" t="str">
@@ -7231,14 +7250,14 @@
         <v/>
       </c>
       <c r="F176" s="7"/>
-      <c r="G176" s="3"/>
-      <c r="H176" s="4"/>
-      <c r="I176" s="4"/>
-      <c r="J176" s="6" t="str">
+      <c r="G176" s="22"/>
+      <c r="H176" s="23"/>
+      <c r="I176" s="23"/>
+      <c r="J176" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K176" s="5"/>
+      <c r="K176" s="26"/>
       <c r="L176" s="4"/>
       <c r="M176" s="5"/>
       <c r="N176" s="2" t="str">
@@ -7268,14 +7287,14 @@
         <v/>
       </c>
       <c r="F177" s="7"/>
-      <c r="G177" s="3"/>
-      <c r="H177" s="4"/>
-      <c r="I177" s="4"/>
-      <c r="J177" s="6" t="str">
+      <c r="G177" s="22"/>
+      <c r="H177" s="23"/>
+      <c r="I177" s="23"/>
+      <c r="J177" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K177" s="5"/>
+      <c r="K177" s="26"/>
       <c r="L177" s="4"/>
       <c r="M177" s="5"/>
       <c r="N177" s="2" t="str">
@@ -7305,14 +7324,14 @@
         <v/>
       </c>
       <c r="F178" s="7"/>
-      <c r="G178" s="3"/>
-      <c r="H178" s="4"/>
-      <c r="I178" s="4"/>
-      <c r="J178" s="6" t="str">
+      <c r="G178" s="22"/>
+      <c r="H178" s="23"/>
+      <c r="I178" s="23"/>
+      <c r="J178" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K178" s="5"/>
+      <c r="K178" s="26"/>
       <c r="L178" s="4"/>
       <c r="M178" s="5"/>
       <c r="N178" s="2" t="str">
@@ -7342,14 +7361,14 @@
         <v/>
       </c>
       <c r="F179" s="7"/>
-      <c r="G179" s="3"/>
-      <c r="H179" s="4"/>
-      <c r="I179" s="4"/>
-      <c r="J179" s="6" t="str">
+      <c r="G179" s="22"/>
+      <c r="H179" s="23"/>
+      <c r="I179" s="23"/>
+      <c r="J179" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K179" s="5"/>
+      <c r="K179" s="26"/>
       <c r="L179" s="4"/>
       <c r="M179" s="5"/>
       <c r="N179" s="2" t="str">
@@ -7379,14 +7398,14 @@
         <v/>
       </c>
       <c r="F180" s="7"/>
-      <c r="G180" s="3"/>
-      <c r="H180" s="4"/>
-      <c r="I180" s="4"/>
-      <c r="J180" s="6" t="str">
+      <c r="G180" s="22"/>
+      <c r="H180" s="23"/>
+      <c r="I180" s="23"/>
+      <c r="J180" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K180" s="5"/>
+      <c r="K180" s="26"/>
       <c r="L180" s="4"/>
       <c r="M180" s="5"/>
       <c r="N180" s="2" t="str">
@@ -7416,14 +7435,14 @@
         <v/>
       </c>
       <c r="F181" s="7"/>
-      <c r="G181" s="3"/>
-      <c r="H181" s="4"/>
-      <c r="I181" s="4"/>
-      <c r="J181" s="6" t="str">
+      <c r="G181" s="22"/>
+      <c r="H181" s="23"/>
+      <c r="I181" s="23"/>
+      <c r="J181" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K181" s="5"/>
+      <c r="K181" s="26"/>
       <c r="L181" s="4"/>
       <c r="M181" s="5"/>
       <c r="N181" s="2" t="str">
@@ -7453,14 +7472,14 @@
         <v/>
       </c>
       <c r="F182" s="7"/>
-      <c r="G182" s="3"/>
-      <c r="H182" s="4"/>
-      <c r="I182" s="4"/>
-      <c r="J182" s="6" t="str">
+      <c r="G182" s="22"/>
+      <c r="H182" s="23"/>
+      <c r="I182" s="23"/>
+      <c r="J182" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K182" s="5"/>
+      <c r="K182" s="26"/>
       <c r="L182" s="4"/>
       <c r="M182" s="5"/>
       <c r="N182" s="2" t="str">
@@ -7490,14 +7509,14 @@
         <v/>
       </c>
       <c r="F183" s="7"/>
-      <c r="G183" s="3"/>
-      <c r="H183" s="4"/>
-      <c r="I183" s="4"/>
-      <c r="J183" s="6" t="str">
+      <c r="G183" s="22"/>
+      <c r="H183" s="23"/>
+      <c r="I183" s="23"/>
+      <c r="J183" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K183" s="5"/>
+      <c r="K183" s="26"/>
       <c r="L183" s="4"/>
       <c r="M183" s="5"/>
       <c r="N183" s="2" t="str">
@@ -7527,14 +7546,14 @@
         <v/>
       </c>
       <c r="F184" s="7"/>
-      <c r="G184" s="3"/>
-      <c r="H184" s="4"/>
-      <c r="I184" s="4"/>
-      <c r="J184" s="6" t="str">
+      <c r="G184" s="22"/>
+      <c r="H184" s="23"/>
+      <c r="I184" s="23"/>
+      <c r="J184" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K184" s="5"/>
+      <c r="K184" s="26"/>
       <c r="L184" s="4"/>
       <c r="M184" s="5"/>
       <c r="N184" s="2" t="str">
@@ -7564,14 +7583,14 @@
         <v/>
       </c>
       <c r="F185" s="7"/>
-      <c r="G185" s="3"/>
-      <c r="H185" s="4"/>
-      <c r="I185" s="4"/>
-      <c r="J185" s="6" t="str">
+      <c r="G185" s="22"/>
+      <c r="H185" s="23"/>
+      <c r="I185" s="23"/>
+      <c r="J185" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K185" s="5"/>
+      <c r="K185" s="26"/>
       <c r="L185" s="4"/>
       <c r="M185" s="5"/>
       <c r="N185" s="2" t="str">
@@ -7601,14 +7620,14 @@
         <v/>
       </c>
       <c r="F186" s="7"/>
-      <c r="G186" s="3"/>
-      <c r="H186" s="4"/>
-      <c r="I186" s="4"/>
-      <c r="J186" s="6" t="str">
+      <c r="G186" s="22"/>
+      <c r="H186" s="23"/>
+      <c r="I186" s="23"/>
+      <c r="J186" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K186" s="5"/>
+      <c r="K186" s="26"/>
       <c r="L186" s="4"/>
       <c r="M186" s="5"/>
       <c r="N186" s="2" t="str">
@@ -7638,14 +7657,14 @@
         <v/>
       </c>
       <c r="F187" s="7"/>
-      <c r="G187" s="3"/>
-      <c r="H187" s="4"/>
-      <c r="I187" s="4"/>
-      <c r="J187" s="6" t="str">
+      <c r="G187" s="22"/>
+      <c r="H187" s="23"/>
+      <c r="I187" s="23"/>
+      <c r="J187" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K187" s="5"/>
+      <c r="K187" s="26"/>
       <c r="L187" s="4"/>
       <c r="M187" s="5"/>
       <c r="N187" s="2" t="str">
@@ -7675,14 +7694,14 @@
         <v/>
       </c>
       <c r="F188" s="7"/>
-      <c r="G188" s="3"/>
-      <c r="H188" s="4"/>
-      <c r="I188" s="4"/>
-      <c r="J188" s="6" t="str">
+      <c r="G188" s="22"/>
+      <c r="H188" s="23"/>
+      <c r="I188" s="23"/>
+      <c r="J188" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K188" s="5"/>
+      <c r="K188" s="26"/>
       <c r="L188" s="4"/>
       <c r="M188" s="5"/>
       <c r="N188" s="2" t="str">
@@ -7712,14 +7731,14 @@
         <v/>
       </c>
       <c r="F189" s="7"/>
-      <c r="G189" s="3"/>
-      <c r="H189" s="4"/>
-      <c r="I189" s="4"/>
-      <c r="J189" s="6" t="str">
+      <c r="G189" s="22"/>
+      <c r="H189" s="23"/>
+      <c r="I189" s="23"/>
+      <c r="J189" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K189" s="5"/>
+      <c r="K189" s="26"/>
       <c r="L189" s="4"/>
       <c r="M189" s="5"/>
       <c r="N189" s="2" t="str">
@@ -7749,14 +7768,14 @@
         <v/>
       </c>
       <c r="F190" s="7"/>
-      <c r="G190" s="3"/>
-      <c r="H190" s="4"/>
-      <c r="I190" s="4"/>
-      <c r="J190" s="6" t="str">
+      <c r="G190" s="22"/>
+      <c r="H190" s="23"/>
+      <c r="I190" s="23"/>
+      <c r="J190" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K190" s="5"/>
+      <c r="K190" s="26"/>
       <c r="L190" s="4"/>
       <c r="M190" s="5"/>
       <c r="N190" s="2" t="str">
@@ -7786,14 +7805,14 @@
         <v/>
       </c>
       <c r="F191" s="7"/>
-      <c r="G191" s="3"/>
-      <c r="H191" s="4"/>
-      <c r="I191" s="4"/>
-      <c r="J191" s="6" t="str">
+      <c r="G191" s="22"/>
+      <c r="H191" s="23"/>
+      <c r="I191" s="23"/>
+      <c r="J191" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K191" s="5"/>
+      <c r="K191" s="26"/>
       <c r="L191" s="4"/>
       <c r="M191" s="5"/>
       <c r="N191" s="2" t="str">
@@ -7823,14 +7842,14 @@
         <v/>
       </c>
       <c r="F192" s="7"/>
-      <c r="G192" s="3"/>
-      <c r="H192" s="4"/>
-      <c r="I192" s="4"/>
-      <c r="J192" s="6" t="str">
+      <c r="G192" s="22"/>
+      <c r="H192" s="23"/>
+      <c r="I192" s="23"/>
+      <c r="J192" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K192" s="5"/>
+      <c r="K192" s="26"/>
       <c r="L192" s="4"/>
       <c r="M192" s="5"/>
       <c r="N192" s="2" t="str">
@@ -7860,14 +7879,14 @@
         <v/>
       </c>
       <c r="F193" s="7"/>
-      <c r="G193" s="3"/>
-      <c r="H193" s="4"/>
-      <c r="I193" s="4"/>
-      <c r="J193" s="6" t="str">
+      <c r="G193" s="22"/>
+      <c r="H193" s="23"/>
+      <c r="I193" s="23"/>
+      <c r="J193" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K193" s="5"/>
+      <c r="K193" s="26"/>
       <c r="L193" s="4"/>
       <c r="M193" s="5"/>
       <c r="N193" s="2" t="str">
@@ -7897,14 +7916,14 @@
         <v/>
       </c>
       <c r="F194" s="7"/>
-      <c r="G194" s="3"/>
-      <c r="H194" s="4"/>
-      <c r="I194" s="4"/>
-      <c r="J194" s="6" t="str">
+      <c r="G194" s="22"/>
+      <c r="H194" s="23"/>
+      <c r="I194" s="23"/>
+      <c r="J194" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K194" s="5"/>
+      <c r="K194" s="26"/>
       <c r="L194" s="4"/>
       <c r="M194" s="5"/>
       <c r="N194" s="2" t="str">
@@ -7934,14 +7953,14 @@
         <v/>
       </c>
       <c r="F195" s="7"/>
-      <c r="G195" s="3"/>
-      <c r="H195" s="4"/>
-      <c r="I195" s="4"/>
-      <c r="J195" s="6" t="str">
+      <c r="G195" s="22"/>
+      <c r="H195" s="23"/>
+      <c r="I195" s="23"/>
+      <c r="J195" s="25" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K195" s="5"/>
+      <c r="K195" s="26"/>
       <c r="L195" s="4"/>
       <c r="M195" s="5"/>
       <c r="N195" s="2" t="str">
@@ -7960,7 +7979,7 @@
     </row>
     <row r="196" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A196" s="2" t="str">
-        <f t="shared" ref="A196:A227" si="36">IF(B196="","",ROW()-3)</f>
+        <f t="shared" ref="A196:A203" si="36">IF(B196="","",ROW()-3)</f>
         <v/>
       </c>
       <c r="B196" s="3"/>
@@ -7971,18 +7990,18 @@
         <v/>
       </c>
       <c r="F196" s="7"/>
-      <c r="G196" s="3"/>
-      <c r="H196" s="4"/>
-      <c r="I196" s="4"/>
-      <c r="J196" s="6" t="str">
-        <f t="shared" ref="J196:J227" si="38">IF(OR(I196="",H196=""),"",MAX(0,I196-H196))</f>
-        <v/>
-      </c>
-      <c r="K196" s="5"/>
+      <c r="G196" s="22"/>
+      <c r="H196" s="23"/>
+      <c r="I196" s="23"/>
+      <c r="J196" s="25" t="str">
+        <f t="shared" ref="J196:J203" si="38">IF(OR(I196="",H196=""),"",MAX(0,I196-H196))</f>
+        <v/>
+      </c>
+      <c r="K196" s="26"/>
       <c r="L196" s="4"/>
       <c r="M196" s="5"/>
       <c r="N196" s="2" t="str">
-        <f t="shared" ref="N196:N227" ca="1" si="39">IF(D196="","",IF(M196&lt;&gt;"",IF(M196-D196&gt;=2,"Đủ","Chưa"),IF(NOW()-D196&gt;=2,"Đủ","Chưa")))</f>
+        <f t="shared" ref="N196:N203" ca="1" si="39">IF(D196="","",IF(M196&lt;&gt;"",IF(M196-D196&gt;=2,"Đủ","Chưa"),IF(NOW()-D196&gt;=2,"Đủ","Chưa")))</f>
         <v/>
       </c>
       <c r="O196" s="6" t="str">
@@ -8008,14 +8027,14 @@
         <v/>
       </c>
       <c r="F197" s="7"/>
-      <c r="G197" s="3"/>
-      <c r="H197" s="4"/>
-      <c r="I197" s="4"/>
-      <c r="J197" s="6" t="str">
+      <c r="G197" s="22"/>
+      <c r="H197" s="23"/>
+      <c r="I197" s="23"/>
+      <c r="J197" s="25" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K197" s="5"/>
+      <c r="K197" s="26"/>
       <c r="L197" s="4"/>
       <c r="M197" s="5"/>
       <c r="N197" s="2" t="str">
@@ -8045,14 +8064,14 @@
         <v/>
       </c>
       <c r="F198" s="7"/>
-      <c r="G198" s="3"/>
-      <c r="H198" s="4"/>
-      <c r="I198" s="4"/>
-      <c r="J198" s="6" t="str">
+      <c r="G198" s="22"/>
+      <c r="H198" s="23"/>
+      <c r="I198" s="23"/>
+      <c r="J198" s="25" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K198" s="5"/>
+      <c r="K198" s="26"/>
       <c r="L198" s="4"/>
       <c r="M198" s="5"/>
       <c r="N198" s="2" t="str">
@@ -8082,14 +8101,14 @@
         <v/>
       </c>
       <c r="F199" s="7"/>
-      <c r="G199" s="3"/>
-      <c r="H199" s="4"/>
-      <c r="I199" s="4"/>
-      <c r="J199" s="6" t="str">
+      <c r="G199" s="22"/>
+      <c r="H199" s="23"/>
+      <c r="I199" s="23"/>
+      <c r="J199" s="25" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K199" s="5"/>
+      <c r="K199" s="26"/>
       <c r="L199" s="4"/>
       <c r="M199" s="5"/>
       <c r="N199" s="2" t="str">
@@ -8119,14 +8138,14 @@
         <v/>
       </c>
       <c r="F200" s="7"/>
-      <c r="G200" s="3"/>
-      <c r="H200" s="4"/>
-      <c r="I200" s="4"/>
-      <c r="J200" s="6" t="str">
+      <c r="G200" s="22"/>
+      <c r="H200" s="23"/>
+      <c r="I200" s="23"/>
+      <c r="J200" s="25" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K200" s="5"/>
+      <c r="K200" s="26"/>
       <c r="L200" s="4"/>
       <c r="M200" s="5"/>
       <c r="N200" s="2" t="str">
@@ -8156,14 +8175,14 @@
         <v/>
       </c>
       <c r="F201" s="7"/>
-      <c r="G201" s="3"/>
-      <c r="H201" s="4"/>
-      <c r="I201" s="4"/>
-      <c r="J201" s="6" t="str">
+      <c r="G201" s="22"/>
+      <c r="H201" s="23"/>
+      <c r="I201" s="23"/>
+      <c r="J201" s="25" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K201" s="5"/>
+      <c r="K201" s="26"/>
       <c r="L201" s="4"/>
       <c r="M201" s="5"/>
       <c r="N201" s="2" t="str">
@@ -8193,14 +8212,14 @@
         <v/>
       </c>
       <c r="F202" s="7"/>
-      <c r="G202" s="3"/>
-      <c r="H202" s="4"/>
-      <c r="I202" s="4"/>
-      <c r="J202" s="6" t="str">
+      <c r="G202" s="22"/>
+      <c r="H202" s="23"/>
+      <c r="I202" s="23"/>
+      <c r="J202" s="25" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K202" s="5"/>
+      <c r="K202" s="26"/>
       <c r="L202" s="4"/>
       <c r="M202" s="5"/>
       <c r="N202" s="2" t="str">
@@ -8230,14 +8249,14 @@
         <v/>
       </c>
       <c r="F203" s="7"/>
-      <c r="G203" s="3"/>
-      <c r="H203" s="4"/>
-      <c r="I203" s="4"/>
-      <c r="J203" s="6" t="str">
+      <c r="G203" s="22"/>
+      <c r="H203" s="23"/>
+      <c r="I203" s="23"/>
+      <c r="J203" s="25" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K203" s="5"/>
+      <c r="K203" s="26"/>
       <c r="L203" s="4"/>
       <c r="M203" s="5"/>
       <c r="N203" s="2" t="str">
@@ -8301,7 +8320,7 @@
       </c>
       <c r="B3" s="9">
         <f>COUNTA('Kho Xe'!B4:B203)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -8328,7 +8347,7 @@
       </c>
       <c r="B6" s="9">
         <f>COUNTIF('Kho Xe'!F4:F203,"Đã bán")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -8337,7 +8356,7 @@
       </c>
       <c r="B8" s="6">
         <f>SUM('Kho Xe'!C4:C203)</f>
-        <v>10000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -8373,7 +8392,7 @@
       </c>
       <c r="B13" s="6">
         <f>SUM('Kho Xe'!L4:L203)</f>
-        <v>13000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -8382,7 +8401,7 @@
       </c>
       <c r="B14" s="6">
         <f>SUM('Kho Xe'!O4:O203)</f>
-        <v>650000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -8391,7 +8410,7 @@
       </c>
       <c r="B15" s="11">
         <f>SUM('Kho Xe'!P4:P203)</f>
-        <v>2350000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -8559,7 +8578,7 @@
       </c>
       <c r="C26" s="6">
         <f>SUMIFS('Kho Xe'!C4:C203,'Kho Xe'!D4:D203,"&gt;="&amp;$A26,'Kho Xe'!D4:D203,"&lt;="&amp;EOMONTH($A26,0))</f>
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="D26" s="2">
         <f>COUNTIFS('Kho Xe'!M4:M203,"&gt;="&amp;$A26,'Kho Xe'!M4:M203,"&lt;="&amp;EOMONTH($A26,0))</f>
@@ -8567,7 +8586,7 @@
       </c>
       <c r="E26" s="6">
         <f>SUMIFS('Kho Xe'!P4:P203,'Kho Xe'!M4:M203,"&gt;="&amp;$A26,'Kho Xe'!M4:M203,"&lt;="&amp;EOMONTH($A26,0))</f>
-        <v>2350000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -8577,7 +8596,7 @@
       </c>
       <c r="B27" s="2">
         <f>COUNTIFS('Kho Xe'!D4:D203,"&gt;="&amp;$A27,'Kho Xe'!D4:D203,"&lt;="&amp;EOMONTH($A27,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" s="6">
         <f>SUMIFS('Kho Xe'!C4:C203,'Kho Xe'!D4:D203,"&gt;="&amp;$A27,'Kho Xe'!D4:D203,"&lt;="&amp;EOMONTH($A27,0))</f>

</xml_diff>

<commit_message>
Auto backup: 2026-08-05 17:48:27
</commit_message>
<xml_diff>
--- a/QuanLyKhoXe.xlsx
+++ b/QuanLyKhoXe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BuonBanXe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882DB478-1B51-464E-95FC-C5AE1E59E0DF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4AC7B00-7A51-4345-BB22-58E08C9D8E3E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,7 +75,7 @@
     <t>Đủ 48h?</t>
   </si>
   <si>
-    <t>Thuế 5%</t>
+    <t>Thuế 6%</t>
   </si>
   <si>
     <t>Lãi thực</t>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>Xe đẹp, khách quen</t>
+  </si>
+  <si>
+    <t>poscher</t>
   </si>
   <si>
     <t>TỔNG HỢP TOÀN BỘ</t>
@@ -126,7 +129,7 @@
     <t>Tổng doanh thu bán xe</t>
   </si>
   <si>
-    <t>Tổng thuế 5% đã trả</t>
+    <t>Tổng thuế 6% đã trả</t>
   </si>
   <si>
     <t>TỔNG LÃI THỰC</t>
@@ -183,7 +186,7 @@
     <t>3. BÁN XE: chọn Trạng thái = 'Đã bán', điền Giá bán thực tế và Ngày bán.</t>
   </si>
   <si>
-    <t xml:space="preserve">   → Cột 'Thuế 5%' và 'Lãi thực' tự tính ra ngay.</t>
+    <t xml:space="preserve">   → Cột 'Thuế 6%' và 'Lãi thực' tự tính ra ngay.</t>
   </si>
   <si>
     <t>CÁCH TÍNH (giống hệt phần mềm)</t>
@@ -195,10 +198,10 @@
     <t>• Còn thanh toán = Giá bán ra − Tiền cọc</t>
   </si>
   <si>
-    <t>• Thuế 5%       = Giá bán thực tế × 5%</t>
+    <t>• Thuế 6%       = Giá bán thực tế × 6%</t>
   </si>
   <si>
-    <t>• LÃI THỰC      = Giá bán thực tế × 0,95 − Giá nhập   (đã trừ thuế 5%)</t>
+    <t>• LÃI THỰC      = Giá bán thực tế × 0,94 − Giá nhập   (đã trừ thuế 6%)</t>
   </si>
   <si>
     <t>CỘT 'ĐỦ 48H?'</t>
@@ -226,9 +229,6 @@
   </si>
   <si>
     <t>• File có sẵn 200 dòng. Cần thêm thì copy 1 dòng trống kéo xuống là công thức tự theo.</t>
-  </si>
-  <si>
-    <t>poscher</t>
   </si>
 </sst>
 </file>
@@ -365,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -398,13 +398,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -413,6 +407,14 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -733,65 +735,65 @@
   <dimension ref="A1:Q203"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="18" style="24" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="14" style="24" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="16" style="24" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="15" style="24" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="17" style="24" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="13" customWidth="1"/>
-    <col min="16" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="30" customWidth="1"/>
+    <col min="1" max="1" width="6" style="18" customWidth="1"/>
+    <col min="2" max="2" width="20" style="18" customWidth="1"/>
+    <col min="3" max="3" width="15" style="18" customWidth="1"/>
+    <col min="4" max="5" width="17" style="18" customWidth="1"/>
+    <col min="6" max="6" width="14" style="18" customWidth="1"/>
+    <col min="7" max="7" width="18" style="22" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="14" style="22" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="22" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="22" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="17" style="22" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="18" customWidth="1"/>
+    <col min="13" max="13" width="17" style="18" customWidth="1"/>
+    <col min="14" max="14" width="10" style="18" customWidth="1"/>
+    <col min="15" max="15" width="13" style="18" customWidth="1"/>
+    <col min="16" max="16" width="15" style="18" customWidth="1"/>
+    <col min="17" max="17" width="30" style="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
     </row>
     <row r="3" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -812,19 +814,19 @@
       <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="H3" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="J3" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="K3" s="19" t="s">
         <v>12</v>
       </c>
       <c r="L3" s="1" t="s">
@@ -866,20 +868,20 @@
       <c r="F4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G4" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="23">
+      <c r="H4" s="21">
         <v>1000000</v>
       </c>
-      <c r="I4" s="23">
+      <c r="I4" s="21">
         <v>13000000</v>
       </c>
-      <c r="J4" s="25">
+      <c r="J4" s="23">
         <f t="shared" ref="J4:J35" si="2">IF(OR(I4="",H4=""),"",MAX(0,I4-H4))</f>
         <v>12000000</v>
       </c>
-      <c r="K4" s="26">
+      <c r="K4" s="24">
         <f>DATE(2026,7,26)+TIME(14,30,0)</f>
         <v>46229.604166666664</v>
       </c>
@@ -893,11 +895,11 @@
         <v>Đủ</v>
       </c>
       <c r="O4" s="6" t="str">
-        <f t="shared" ref="O4:O35" si="4">IF(L4="","",L4*0.05)</f>
+        <f t="shared" ref="O4:O35" si="4">IF(L4="","",L4*0.06)</f>
         <v/>
       </c>
       <c r="P4" s="6" t="str">
-        <f t="shared" ref="P4:P35" si="5">IF(OR(L4="",C4=""),"",L4*0.95-C4)</f>
+        <f t="shared" ref="P4:P35" si="5">IF(OR(L4="",C4=""),"",L4*0.94-C4)</f>
         <v/>
       </c>
       <c r="Q4" s="3" t="s">
@@ -910,7 +912,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="5">
@@ -923,14 +925,14 @@
       <c r="F5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="22"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="25" t="str">
+      <c r="G5" s="20"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K5" s="26"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="4"/>
       <c r="M5" s="5"/>
       <c r="N5" s="2" t="str">
@@ -960,14 +962,14 @@
         <v/>
       </c>
       <c r="F6" s="7"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="25" t="str">
+      <c r="G6" s="20"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K6" s="26"/>
+      <c r="K6" s="24"/>
       <c r="L6" s="4"/>
       <c r="M6" s="5"/>
       <c r="N6" s="2" t="str">
@@ -997,14 +999,14 @@
         <v/>
       </c>
       <c r="F7" s="7"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="25" t="str">
+      <c r="G7" s="20"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K7" s="26"/>
+      <c r="K7" s="24"/>
       <c r="L7" s="4"/>
       <c r="M7" s="5"/>
       <c r="N7" s="2" t="str">
@@ -1034,14 +1036,14 @@
         <v/>
       </c>
       <c r="F8" s="7"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="25" t="str">
+      <c r="G8" s="20"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K8" s="26"/>
+      <c r="K8" s="24"/>
       <c r="L8" s="4"/>
       <c r="M8" s="5"/>
       <c r="N8" s="2" t="str">
@@ -1071,14 +1073,14 @@
         <v/>
       </c>
       <c r="F9" s="7"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="25" t="str">
+      <c r="G9" s="20"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K9" s="26"/>
+      <c r="K9" s="24"/>
       <c r="L9" s="4"/>
       <c r="M9" s="5"/>
       <c r="N9" s="2" t="str">
@@ -1108,14 +1110,14 @@
         <v/>
       </c>
       <c r="F10" s="7"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="25" t="str">
+      <c r="G10" s="20"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K10" s="26"/>
+      <c r="K10" s="24"/>
       <c r="L10" s="4"/>
       <c r="M10" s="5"/>
       <c r="N10" s="2" t="str">
@@ -1145,14 +1147,14 @@
         <v/>
       </c>
       <c r="F11" s="7"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="25" t="str">
+      <c r="G11" s="20"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K11" s="26"/>
+      <c r="K11" s="24"/>
       <c r="L11" s="4"/>
       <c r="M11" s="5"/>
       <c r="N11" s="2" t="str">
@@ -1182,14 +1184,14 @@
         <v/>
       </c>
       <c r="F12" s="7"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="25" t="str">
+      <c r="G12" s="20"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K12" s="26"/>
+      <c r="K12" s="24"/>
       <c r="L12" s="4"/>
       <c r="M12" s="5"/>
       <c r="N12" s="2" t="str">
@@ -1219,14 +1221,14 @@
         <v/>
       </c>
       <c r="F13" s="7"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="25" t="str">
+      <c r="G13" s="20"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K13" s="26"/>
+      <c r="K13" s="24"/>
       <c r="L13" s="4"/>
       <c r="M13" s="5"/>
       <c r="N13" s="2" t="str">
@@ -1256,14 +1258,14 @@
         <v/>
       </c>
       <c r="F14" s="7"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="25" t="str">
+      <c r="G14" s="20"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K14" s="26"/>
+      <c r="K14" s="24"/>
       <c r="L14" s="4"/>
       <c r="M14" s="5"/>
       <c r="N14" s="2" t="str">
@@ -1293,14 +1295,14 @@
         <v/>
       </c>
       <c r="F15" s="7"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="25" t="str">
+      <c r="G15" s="20"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K15" s="26"/>
+      <c r="K15" s="24"/>
       <c r="L15" s="4"/>
       <c r="M15" s="5"/>
       <c r="N15" s="2" t="str">
@@ -1330,14 +1332,14 @@
         <v/>
       </c>
       <c r="F16" s="7"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="25" t="str">
+      <c r="G16" s="20"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K16" s="26"/>
+      <c r="K16" s="24"/>
       <c r="L16" s="4"/>
       <c r="M16" s="5"/>
       <c r="N16" s="2" t="str">
@@ -1367,14 +1369,14 @@
         <v/>
       </c>
       <c r="F17" s="7"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="25" t="str">
+      <c r="G17" s="20"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K17" s="26"/>
+      <c r="K17" s="24"/>
       <c r="L17" s="4"/>
       <c r="M17" s="5"/>
       <c r="N17" s="2" t="str">
@@ -1404,14 +1406,14 @@
         <v/>
       </c>
       <c r="F18" s="7"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="25" t="str">
+      <c r="G18" s="20"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K18" s="26"/>
+      <c r="K18" s="24"/>
       <c r="L18" s="4"/>
       <c r="M18" s="5"/>
       <c r="N18" s="2" t="str">
@@ -1441,14 +1443,14 @@
         <v/>
       </c>
       <c r="F19" s="7"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="25" t="str">
+      <c r="G19" s="20"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K19" s="26"/>
+      <c r="K19" s="24"/>
       <c r="L19" s="4"/>
       <c r="M19" s="5"/>
       <c r="N19" s="2" t="str">
@@ -1478,14 +1480,14 @@
         <v/>
       </c>
       <c r="F20" s="7"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="25" t="str">
+      <c r="G20" s="20"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K20" s="26"/>
+      <c r="K20" s="24"/>
       <c r="L20" s="4"/>
       <c r="M20" s="5"/>
       <c r="N20" s="2" t="str">
@@ -1515,14 +1517,14 @@
         <v/>
       </c>
       <c r="F21" s="7"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="25" t="str">
+      <c r="G21" s="20"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K21" s="26"/>
+      <c r="K21" s="24"/>
       <c r="L21" s="4"/>
       <c r="M21" s="5"/>
       <c r="N21" s="2" t="str">
@@ -1552,14 +1554,14 @@
         <v/>
       </c>
       <c r="F22" s="7"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="25" t="str">
+      <c r="G22" s="20"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K22" s="26"/>
+      <c r="K22" s="24"/>
       <c r="L22" s="4"/>
       <c r="M22" s="5"/>
       <c r="N22" s="2" t="str">
@@ -1589,14 +1591,14 @@
         <v/>
       </c>
       <c r="F23" s="7"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="25" t="str">
+      <c r="G23" s="20"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K23" s="26"/>
+      <c r="K23" s="24"/>
       <c r="L23" s="4"/>
       <c r="M23" s="5"/>
       <c r="N23" s="2" t="str">
@@ -1626,14 +1628,14 @@
         <v/>
       </c>
       <c r="F24" s="7"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="23"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="25" t="str">
+      <c r="G24" s="20"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K24" s="26"/>
+      <c r="K24" s="24"/>
       <c r="L24" s="4"/>
       <c r="M24" s="5"/>
       <c r="N24" s="2" t="str">
@@ -1663,14 +1665,14 @@
         <v/>
       </c>
       <c r="F25" s="7"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="25" t="str">
+      <c r="G25" s="20"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K25" s="26"/>
+      <c r="K25" s="24"/>
       <c r="L25" s="4"/>
       <c r="M25" s="5"/>
       <c r="N25" s="2" t="str">
@@ -1700,14 +1702,14 @@
         <v/>
       </c>
       <c r="F26" s="7"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="25" t="str">
+      <c r="G26" s="20"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K26" s="26"/>
+      <c r="K26" s="24"/>
       <c r="L26" s="4"/>
       <c r="M26" s="5"/>
       <c r="N26" s="2" t="str">
@@ -1737,14 +1739,14 @@
         <v/>
       </c>
       <c r="F27" s="7"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="25" t="str">
+      <c r="G27" s="20"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K27" s="26"/>
+      <c r="K27" s="24"/>
       <c r="L27" s="4"/>
       <c r="M27" s="5"/>
       <c r="N27" s="2" t="str">
@@ -1774,14 +1776,14 @@
         <v/>
       </c>
       <c r="F28" s="7"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="25" t="str">
+      <c r="G28" s="20"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K28" s="26"/>
+      <c r="K28" s="24"/>
       <c r="L28" s="4"/>
       <c r="M28" s="5"/>
       <c r="N28" s="2" t="str">
@@ -1811,14 +1813,14 @@
         <v/>
       </c>
       <c r="F29" s="7"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="25" t="str">
+      <c r="G29" s="20"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K29" s="26"/>
+      <c r="K29" s="24"/>
       <c r="L29" s="4"/>
       <c r="M29" s="5"/>
       <c r="N29" s="2" t="str">
@@ -1848,14 +1850,14 @@
         <v/>
       </c>
       <c r="F30" s="7"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="25" t="str">
+      <c r="G30" s="20"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K30" s="26"/>
+      <c r="K30" s="24"/>
       <c r="L30" s="4"/>
       <c r="M30" s="5"/>
       <c r="N30" s="2" t="str">
@@ -1885,14 +1887,14 @@
         <v/>
       </c>
       <c r="F31" s="7"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="25" t="str">
+      <c r="G31" s="20"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K31" s="26"/>
+      <c r="K31" s="24"/>
       <c r="L31" s="4"/>
       <c r="M31" s="5"/>
       <c r="N31" s="2" t="str">
@@ -1922,14 +1924,14 @@
         <v/>
       </c>
       <c r="F32" s="7"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="25" t="str">
+      <c r="G32" s="20"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K32" s="26"/>
+      <c r="K32" s="24"/>
       <c r="L32" s="4"/>
       <c r="M32" s="5"/>
       <c r="N32" s="2" t="str">
@@ -1959,14 +1961,14 @@
         <v/>
       </c>
       <c r="F33" s="7"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="25" t="str">
+      <c r="G33" s="20"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K33" s="26"/>
+      <c r="K33" s="24"/>
       <c r="L33" s="4"/>
       <c r="M33" s="5"/>
       <c r="N33" s="2" t="str">
@@ -1996,14 +1998,14 @@
         <v/>
       </c>
       <c r="F34" s="7"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="23"/>
-      <c r="J34" s="25" t="str">
+      <c r="G34" s="20"/>
+      <c r="H34" s="21"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K34" s="26"/>
+      <c r="K34" s="24"/>
       <c r="L34" s="4"/>
       <c r="M34" s="5"/>
       <c r="N34" s="2" t="str">
@@ -2033,14 +2035,14 @@
         <v/>
       </c>
       <c r="F35" s="7"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="23"/>
-      <c r="I35" s="23"/>
-      <c r="J35" s="25" t="str">
+      <c r="G35" s="20"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="23" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K35" s="26"/>
+      <c r="K35" s="24"/>
       <c r="L35" s="4"/>
       <c r="M35" s="5"/>
       <c r="N35" s="2" t="str">
@@ -2070,14 +2072,14 @@
         <v/>
       </c>
       <c r="F36" s="7"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="25" t="str">
+      <c r="G36" s="20"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="23" t="str">
         <f t="shared" ref="J36:J67" si="8">IF(OR(I36="",H36=""),"",MAX(0,I36-H36))</f>
         <v/>
       </c>
-      <c r="K36" s="26"/>
+      <c r="K36" s="24"/>
       <c r="L36" s="4"/>
       <c r="M36" s="5"/>
       <c r="N36" s="2" t="str">
@@ -2085,11 +2087,11 @@
         <v/>
       </c>
       <c r="O36" s="6" t="str">
-        <f t="shared" ref="O36:O67" si="10">IF(L36="","",L36*0.05)</f>
+        <f t="shared" ref="O36:O67" si="10">IF(L36="","",L36*0.06)</f>
         <v/>
       </c>
       <c r="P36" s="6" t="str">
-        <f t="shared" ref="P36:P67" si="11">IF(OR(L36="",C36=""),"",L36*0.95-C36)</f>
+        <f t="shared" ref="P36:P67" si="11">IF(OR(L36="",C36=""),"",L36*0.94-C36)</f>
         <v/>
       </c>
       <c r="Q36" s="3"/>
@@ -2107,14 +2109,14 @@
         <v/>
       </c>
       <c r="F37" s="7"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="23"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="25" t="str">
+      <c r="G37" s="20"/>
+      <c r="H37" s="21"/>
+      <c r="I37" s="21"/>
+      <c r="J37" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K37" s="26"/>
+      <c r="K37" s="24"/>
       <c r="L37" s="4"/>
       <c r="M37" s="5"/>
       <c r="N37" s="2" t="str">
@@ -2144,14 +2146,14 @@
         <v/>
       </c>
       <c r="F38" s="7"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="23"/>
-      <c r="I38" s="23"/>
-      <c r="J38" s="25" t="str">
+      <c r="G38" s="20"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="21"/>
+      <c r="J38" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K38" s="26"/>
+      <c r="K38" s="24"/>
       <c r="L38" s="4"/>
       <c r="M38" s="5"/>
       <c r="N38" s="2" t="str">
@@ -2181,14 +2183,14 @@
         <v/>
       </c>
       <c r="F39" s="7"/>
-      <c r="G39" s="22"/>
-      <c r="H39" s="23"/>
-      <c r="I39" s="23"/>
-      <c r="J39" s="25" t="str">
+      <c r="G39" s="20"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="21"/>
+      <c r="J39" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K39" s="26"/>
+      <c r="K39" s="24"/>
       <c r="L39" s="4"/>
       <c r="M39" s="5"/>
       <c r="N39" s="2" t="str">
@@ -2218,14 +2220,14 @@
         <v/>
       </c>
       <c r="F40" s="7"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="25" t="str">
+      <c r="G40" s="20"/>
+      <c r="H40" s="21"/>
+      <c r="I40" s="21"/>
+      <c r="J40" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K40" s="26"/>
+      <c r="K40" s="24"/>
       <c r="L40" s="4"/>
       <c r="M40" s="5"/>
       <c r="N40" s="2" t="str">
@@ -2255,14 +2257,14 @@
         <v/>
       </c>
       <c r="F41" s="7"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="23"/>
-      <c r="I41" s="23"/>
-      <c r="J41" s="25" t="str">
+      <c r="G41" s="20"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="21"/>
+      <c r="J41" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K41" s="26"/>
+      <c r="K41" s="24"/>
       <c r="L41" s="4"/>
       <c r="M41" s="5"/>
       <c r="N41" s="2" t="str">
@@ -2292,14 +2294,14 @@
         <v/>
       </c>
       <c r="F42" s="7"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="23"/>
-      <c r="I42" s="23"/>
-      <c r="J42" s="25" t="str">
+      <c r="G42" s="20"/>
+      <c r="H42" s="21"/>
+      <c r="I42" s="21"/>
+      <c r="J42" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K42" s="26"/>
+      <c r="K42" s="24"/>
       <c r="L42" s="4"/>
       <c r="M42" s="5"/>
       <c r="N42" s="2" t="str">
@@ -2329,14 +2331,14 @@
         <v/>
       </c>
       <c r="F43" s="7"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="23"/>
-      <c r="I43" s="23"/>
-      <c r="J43" s="25" t="str">
+      <c r="G43" s="20"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="21"/>
+      <c r="J43" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K43" s="26"/>
+      <c r="K43" s="24"/>
       <c r="L43" s="4"/>
       <c r="M43" s="5"/>
       <c r="N43" s="2" t="str">
@@ -2366,14 +2368,14 @@
         <v/>
       </c>
       <c r="F44" s="7"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="23"/>
-      <c r="I44" s="23"/>
-      <c r="J44" s="25" t="str">
+      <c r="G44" s="20"/>
+      <c r="H44" s="21"/>
+      <c r="I44" s="21"/>
+      <c r="J44" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K44" s="26"/>
+      <c r="K44" s="24"/>
       <c r="L44" s="4"/>
       <c r="M44" s="5"/>
       <c r="N44" s="2" t="str">
@@ -2403,14 +2405,14 @@
         <v/>
       </c>
       <c r="F45" s="7"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="23"/>
-      <c r="I45" s="23"/>
-      <c r="J45" s="25" t="str">
+      <c r="G45" s="20"/>
+      <c r="H45" s="21"/>
+      <c r="I45" s="21"/>
+      <c r="J45" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K45" s="26"/>
+      <c r="K45" s="24"/>
       <c r="L45" s="4"/>
       <c r="M45" s="5"/>
       <c r="N45" s="2" t="str">
@@ -2440,14 +2442,14 @@
         <v/>
       </c>
       <c r="F46" s="7"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="23"/>
-      <c r="I46" s="23"/>
-      <c r="J46" s="25" t="str">
+      <c r="G46" s="20"/>
+      <c r="H46" s="21"/>
+      <c r="I46" s="21"/>
+      <c r="J46" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K46" s="26"/>
+      <c r="K46" s="24"/>
       <c r="L46" s="4"/>
       <c r="M46" s="5"/>
       <c r="N46" s="2" t="str">
@@ -2477,14 +2479,14 @@
         <v/>
       </c>
       <c r="F47" s="7"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="23"/>
-      <c r="I47" s="23"/>
-      <c r="J47" s="25" t="str">
+      <c r="G47" s="20"/>
+      <c r="H47" s="21"/>
+      <c r="I47" s="21"/>
+      <c r="J47" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K47" s="26"/>
+      <c r="K47" s="24"/>
       <c r="L47" s="4"/>
       <c r="M47" s="5"/>
       <c r="N47" s="2" t="str">
@@ -2514,14 +2516,14 @@
         <v/>
       </c>
       <c r="F48" s="7"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="23"/>
-      <c r="I48" s="23"/>
-      <c r="J48" s="25" t="str">
+      <c r="G48" s="20"/>
+      <c r="H48" s="21"/>
+      <c r="I48" s="21"/>
+      <c r="J48" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K48" s="26"/>
+      <c r="K48" s="24"/>
       <c r="L48" s="4"/>
       <c r="M48" s="5"/>
       <c r="N48" s="2" t="str">
@@ -2551,14 +2553,14 @@
         <v/>
       </c>
       <c r="F49" s="7"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="23"/>
-      <c r="I49" s="23"/>
-      <c r="J49" s="25" t="str">
+      <c r="G49" s="20"/>
+      <c r="H49" s="21"/>
+      <c r="I49" s="21"/>
+      <c r="J49" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K49" s="26"/>
+      <c r="K49" s="24"/>
       <c r="L49" s="4"/>
       <c r="M49" s="5"/>
       <c r="N49" s="2" t="str">
@@ -2588,14 +2590,14 @@
         <v/>
       </c>
       <c r="F50" s="7"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="23"/>
-      <c r="I50" s="23"/>
-      <c r="J50" s="25" t="str">
+      <c r="G50" s="20"/>
+      <c r="H50" s="21"/>
+      <c r="I50" s="21"/>
+      <c r="J50" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K50" s="26"/>
+      <c r="K50" s="24"/>
       <c r="L50" s="4"/>
       <c r="M50" s="5"/>
       <c r="N50" s="2" t="str">
@@ -2625,14 +2627,14 @@
         <v/>
       </c>
       <c r="F51" s="7"/>
-      <c r="G51" s="22"/>
-      <c r="H51" s="23"/>
-      <c r="I51" s="23"/>
-      <c r="J51" s="25" t="str">
+      <c r="G51" s="20"/>
+      <c r="H51" s="21"/>
+      <c r="I51" s="21"/>
+      <c r="J51" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K51" s="26"/>
+      <c r="K51" s="24"/>
       <c r="L51" s="4"/>
       <c r="M51" s="5"/>
       <c r="N51" s="2" t="str">
@@ -2662,14 +2664,14 @@
         <v/>
       </c>
       <c r="F52" s="7"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="23"/>
-      <c r="J52" s="25" t="str">
+      <c r="G52" s="20"/>
+      <c r="H52" s="21"/>
+      <c r="I52" s="21"/>
+      <c r="J52" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K52" s="26"/>
+      <c r="K52" s="24"/>
       <c r="L52" s="4"/>
       <c r="M52" s="5"/>
       <c r="N52" s="2" t="str">
@@ -2699,14 +2701,14 @@
         <v/>
       </c>
       <c r="F53" s="7"/>
-      <c r="G53" s="22"/>
-      <c r="H53" s="23"/>
-      <c r="I53" s="23"/>
-      <c r="J53" s="25" t="str">
+      <c r="G53" s="20"/>
+      <c r="H53" s="21"/>
+      <c r="I53" s="21"/>
+      <c r="J53" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K53" s="26"/>
+      <c r="K53" s="24"/>
       <c r="L53" s="4"/>
       <c r="M53" s="5"/>
       <c r="N53" s="2" t="str">
@@ -2736,14 +2738,14 @@
         <v/>
       </c>
       <c r="F54" s="7"/>
-      <c r="G54" s="22"/>
-      <c r="H54" s="23"/>
-      <c r="I54" s="23"/>
-      <c r="J54" s="25" t="str">
+      <c r="G54" s="20"/>
+      <c r="H54" s="21"/>
+      <c r="I54" s="21"/>
+      <c r="J54" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K54" s="26"/>
+      <c r="K54" s="24"/>
       <c r="L54" s="4"/>
       <c r="M54" s="5"/>
       <c r="N54" s="2" t="str">
@@ -2773,14 +2775,14 @@
         <v/>
       </c>
       <c r="F55" s="7"/>
-      <c r="G55" s="22"/>
-      <c r="H55" s="23"/>
-      <c r="I55" s="23"/>
-      <c r="J55" s="25" t="str">
+      <c r="G55" s="20"/>
+      <c r="H55" s="21"/>
+      <c r="I55" s="21"/>
+      <c r="J55" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K55" s="26"/>
+      <c r="K55" s="24"/>
       <c r="L55" s="4"/>
       <c r="M55" s="5"/>
       <c r="N55" s="2" t="str">
@@ -2810,14 +2812,14 @@
         <v/>
       </c>
       <c r="F56" s="7"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="23"/>
-      <c r="I56" s="23"/>
-      <c r="J56" s="25" t="str">
+      <c r="G56" s="20"/>
+      <c r="H56" s="21"/>
+      <c r="I56" s="21"/>
+      <c r="J56" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K56" s="26"/>
+      <c r="K56" s="24"/>
       <c r="L56" s="4"/>
       <c r="M56" s="5"/>
       <c r="N56" s="2" t="str">
@@ -2847,14 +2849,14 @@
         <v/>
       </c>
       <c r="F57" s="7"/>
-      <c r="G57" s="22"/>
-      <c r="H57" s="23"/>
-      <c r="I57" s="23"/>
-      <c r="J57" s="25" t="str">
+      <c r="G57" s="20"/>
+      <c r="H57" s="21"/>
+      <c r="I57" s="21"/>
+      <c r="J57" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K57" s="26"/>
+      <c r="K57" s="24"/>
       <c r="L57" s="4"/>
       <c r="M57" s="5"/>
       <c r="N57" s="2" t="str">
@@ -2884,14 +2886,14 @@
         <v/>
       </c>
       <c r="F58" s="7"/>
-      <c r="G58" s="22"/>
-      <c r="H58" s="23"/>
-      <c r="I58" s="23"/>
-      <c r="J58" s="25" t="str">
+      <c r="G58" s="20"/>
+      <c r="H58" s="21"/>
+      <c r="I58" s="21"/>
+      <c r="J58" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K58" s="26"/>
+      <c r="K58" s="24"/>
       <c r="L58" s="4"/>
       <c r="M58" s="5"/>
       <c r="N58" s="2" t="str">
@@ -2921,14 +2923,14 @@
         <v/>
       </c>
       <c r="F59" s="7"/>
-      <c r="G59" s="22"/>
-      <c r="H59" s="23"/>
-      <c r="I59" s="23"/>
-      <c r="J59" s="25" t="str">
+      <c r="G59" s="20"/>
+      <c r="H59" s="21"/>
+      <c r="I59" s="21"/>
+      <c r="J59" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K59" s="26"/>
+      <c r="K59" s="24"/>
       <c r="L59" s="4"/>
       <c r="M59" s="5"/>
       <c r="N59" s="2" t="str">
@@ -2958,14 +2960,14 @@
         <v/>
       </c>
       <c r="F60" s="7"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="23"/>
-      <c r="I60" s="23"/>
-      <c r="J60" s="25" t="str">
+      <c r="G60" s="20"/>
+      <c r="H60" s="21"/>
+      <c r="I60" s="21"/>
+      <c r="J60" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K60" s="26"/>
+      <c r="K60" s="24"/>
       <c r="L60" s="4"/>
       <c r="M60" s="5"/>
       <c r="N60" s="2" t="str">
@@ -2995,14 +2997,14 @@
         <v/>
       </c>
       <c r="F61" s="7"/>
-      <c r="G61" s="22"/>
-      <c r="H61" s="23"/>
-      <c r="I61" s="23"/>
-      <c r="J61" s="25" t="str">
+      <c r="G61" s="20"/>
+      <c r="H61" s="21"/>
+      <c r="I61" s="21"/>
+      <c r="J61" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K61" s="26"/>
+      <c r="K61" s="24"/>
       <c r="L61" s="4"/>
       <c r="M61" s="5"/>
       <c r="N61" s="2" t="str">
@@ -3032,14 +3034,14 @@
         <v/>
       </c>
       <c r="F62" s="7"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="23"/>
-      <c r="I62" s="23"/>
-      <c r="J62" s="25" t="str">
+      <c r="G62" s="20"/>
+      <c r="H62" s="21"/>
+      <c r="I62" s="21"/>
+      <c r="J62" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K62" s="26"/>
+      <c r="K62" s="24"/>
       <c r="L62" s="4"/>
       <c r="M62" s="5"/>
       <c r="N62" s="2" t="str">
@@ -3069,14 +3071,14 @@
         <v/>
       </c>
       <c r="F63" s="7"/>
-      <c r="G63" s="22"/>
-      <c r="H63" s="23"/>
-      <c r="I63" s="23"/>
-      <c r="J63" s="25" t="str">
+      <c r="G63" s="20"/>
+      <c r="H63" s="21"/>
+      <c r="I63" s="21"/>
+      <c r="J63" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K63" s="26"/>
+      <c r="K63" s="24"/>
       <c r="L63" s="4"/>
       <c r="M63" s="5"/>
       <c r="N63" s="2" t="str">
@@ -3106,14 +3108,14 @@
         <v/>
       </c>
       <c r="F64" s="7"/>
-      <c r="G64" s="22"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-      <c r="J64" s="25" t="str">
+      <c r="G64" s="20"/>
+      <c r="H64" s="21"/>
+      <c r="I64" s="21"/>
+      <c r="J64" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K64" s="26"/>
+      <c r="K64" s="24"/>
       <c r="L64" s="4"/>
       <c r="M64" s="5"/>
       <c r="N64" s="2" t="str">
@@ -3143,14 +3145,14 @@
         <v/>
       </c>
       <c r="F65" s="7"/>
-      <c r="G65" s="22"/>
-      <c r="H65" s="23"/>
-      <c r="I65" s="23"/>
-      <c r="J65" s="25" t="str">
+      <c r="G65" s="20"/>
+      <c r="H65" s="21"/>
+      <c r="I65" s="21"/>
+      <c r="J65" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K65" s="26"/>
+      <c r="K65" s="24"/>
       <c r="L65" s="4"/>
       <c r="M65" s="5"/>
       <c r="N65" s="2" t="str">
@@ -3180,14 +3182,14 @@
         <v/>
       </c>
       <c r="F66" s="7"/>
-      <c r="G66" s="22"/>
-      <c r="H66" s="23"/>
-      <c r="I66" s="23"/>
-      <c r="J66" s="25" t="str">
+      <c r="G66" s="20"/>
+      <c r="H66" s="21"/>
+      <c r="I66" s="21"/>
+      <c r="J66" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K66" s="26"/>
+      <c r="K66" s="24"/>
       <c r="L66" s="4"/>
       <c r="M66" s="5"/>
       <c r="N66" s="2" t="str">
@@ -3217,14 +3219,14 @@
         <v/>
       </c>
       <c r="F67" s="7"/>
-      <c r="G67" s="22"/>
-      <c r="H67" s="23"/>
-      <c r="I67" s="23"/>
-      <c r="J67" s="25" t="str">
+      <c r="G67" s="20"/>
+      <c r="H67" s="21"/>
+      <c r="I67" s="21"/>
+      <c r="J67" s="23" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K67" s="26"/>
+      <c r="K67" s="24"/>
       <c r="L67" s="4"/>
       <c r="M67" s="5"/>
       <c r="N67" s="2" t="str">
@@ -3254,14 +3256,14 @@
         <v/>
       </c>
       <c r="F68" s="7"/>
-      <c r="G68" s="22"/>
-      <c r="H68" s="23"/>
-      <c r="I68" s="23"/>
-      <c r="J68" s="25" t="str">
+      <c r="G68" s="20"/>
+      <c r="H68" s="21"/>
+      <c r="I68" s="21"/>
+      <c r="J68" s="23" t="str">
         <f t="shared" ref="J68:J99" si="14">IF(OR(I68="",H68=""),"",MAX(0,I68-H68))</f>
         <v/>
       </c>
-      <c r="K68" s="26"/>
+      <c r="K68" s="24"/>
       <c r="L68" s="4"/>
       <c r="M68" s="5"/>
       <c r="N68" s="2" t="str">
@@ -3269,11 +3271,11 @@
         <v/>
       </c>
       <c r="O68" s="6" t="str">
-        <f t="shared" ref="O68:O99" si="16">IF(L68="","",L68*0.05)</f>
+        <f t="shared" ref="O68:O99" si="16">IF(L68="","",L68*0.06)</f>
         <v/>
       </c>
       <c r="P68" s="6" t="str">
-        <f t="shared" ref="P68:P99" si="17">IF(OR(L68="",C68=""),"",L68*0.95-C68)</f>
+        <f t="shared" ref="P68:P99" si="17">IF(OR(L68="",C68=""),"",L68*0.94-C68)</f>
         <v/>
       </c>
       <c r="Q68" s="3"/>
@@ -3291,14 +3293,14 @@
         <v/>
       </c>
       <c r="F69" s="7"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="23"/>
-      <c r="I69" s="23"/>
-      <c r="J69" s="25" t="str">
+      <c r="G69" s="20"/>
+      <c r="H69" s="21"/>
+      <c r="I69" s="21"/>
+      <c r="J69" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K69" s="26"/>
+      <c r="K69" s="24"/>
       <c r="L69" s="4"/>
       <c r="M69" s="5"/>
       <c r="N69" s="2" t="str">
@@ -3328,14 +3330,14 @@
         <v/>
       </c>
       <c r="F70" s="7"/>
-      <c r="G70" s="22"/>
-      <c r="H70" s="23"/>
-      <c r="I70" s="23"/>
-      <c r="J70" s="25" t="str">
+      <c r="G70" s="20"/>
+      <c r="H70" s="21"/>
+      <c r="I70" s="21"/>
+      <c r="J70" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K70" s="26"/>
+      <c r="K70" s="24"/>
       <c r="L70" s="4"/>
       <c r="M70" s="5"/>
       <c r="N70" s="2" t="str">
@@ -3365,14 +3367,14 @@
         <v/>
       </c>
       <c r="F71" s="7"/>
-      <c r="G71" s="22"/>
-      <c r="H71" s="23"/>
-      <c r="I71" s="23"/>
-      <c r="J71" s="25" t="str">
+      <c r="G71" s="20"/>
+      <c r="H71" s="21"/>
+      <c r="I71" s="21"/>
+      <c r="J71" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K71" s="26"/>
+      <c r="K71" s="24"/>
       <c r="L71" s="4"/>
       <c r="M71" s="5"/>
       <c r="N71" s="2" t="str">
@@ -3402,14 +3404,14 @@
         <v/>
       </c>
       <c r="F72" s="7"/>
-      <c r="G72" s="22"/>
-      <c r="H72" s="23"/>
-      <c r="I72" s="23"/>
-      <c r="J72" s="25" t="str">
+      <c r="G72" s="20"/>
+      <c r="H72" s="21"/>
+      <c r="I72" s="21"/>
+      <c r="J72" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K72" s="26"/>
+      <c r="K72" s="24"/>
       <c r="L72" s="4"/>
       <c r="M72" s="5"/>
       <c r="N72" s="2" t="str">
@@ -3439,14 +3441,14 @@
         <v/>
       </c>
       <c r="F73" s="7"/>
-      <c r="G73" s="22"/>
-      <c r="H73" s="23"/>
-      <c r="I73" s="23"/>
-      <c r="J73" s="25" t="str">
+      <c r="G73" s="20"/>
+      <c r="H73" s="21"/>
+      <c r="I73" s="21"/>
+      <c r="J73" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K73" s="26"/>
+      <c r="K73" s="24"/>
       <c r="L73" s="4"/>
       <c r="M73" s="5"/>
       <c r="N73" s="2" t="str">
@@ -3476,14 +3478,14 @@
         <v/>
       </c>
       <c r="F74" s="7"/>
-      <c r="G74" s="22"/>
-      <c r="H74" s="23"/>
-      <c r="I74" s="23"/>
-      <c r="J74" s="25" t="str">
+      <c r="G74" s="20"/>
+      <c r="H74" s="21"/>
+      <c r="I74" s="21"/>
+      <c r="J74" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K74" s="26"/>
+      <c r="K74" s="24"/>
       <c r="L74" s="4"/>
       <c r="M74" s="5"/>
       <c r="N74" s="2" t="str">
@@ -3513,14 +3515,14 @@
         <v/>
       </c>
       <c r="F75" s="7"/>
-      <c r="G75" s="22"/>
-      <c r="H75" s="23"/>
-      <c r="I75" s="23"/>
-      <c r="J75" s="25" t="str">
+      <c r="G75" s="20"/>
+      <c r="H75" s="21"/>
+      <c r="I75" s="21"/>
+      <c r="J75" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K75" s="26"/>
+      <c r="K75" s="24"/>
       <c r="L75" s="4"/>
       <c r="M75" s="5"/>
       <c r="N75" s="2" t="str">
@@ -3550,14 +3552,14 @@
         <v/>
       </c>
       <c r="F76" s="7"/>
-      <c r="G76" s="22"/>
-      <c r="H76" s="23"/>
-      <c r="I76" s="23"/>
-      <c r="J76" s="25" t="str">
+      <c r="G76" s="20"/>
+      <c r="H76" s="21"/>
+      <c r="I76" s="21"/>
+      <c r="J76" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K76" s="26"/>
+      <c r="K76" s="24"/>
       <c r="L76" s="4"/>
       <c r="M76" s="5"/>
       <c r="N76" s="2" t="str">
@@ -3587,14 +3589,14 @@
         <v/>
       </c>
       <c r="F77" s="7"/>
-      <c r="G77" s="22"/>
-      <c r="H77" s="23"/>
-      <c r="I77" s="23"/>
-      <c r="J77" s="25" t="str">
+      <c r="G77" s="20"/>
+      <c r="H77" s="21"/>
+      <c r="I77" s="21"/>
+      <c r="J77" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K77" s="26"/>
+      <c r="K77" s="24"/>
       <c r="L77" s="4"/>
       <c r="M77" s="5"/>
       <c r="N77" s="2" t="str">
@@ -3624,14 +3626,14 @@
         <v/>
       </c>
       <c r="F78" s="7"/>
-      <c r="G78" s="22"/>
-      <c r="H78" s="23"/>
-      <c r="I78" s="23"/>
-      <c r="J78" s="25" t="str">
+      <c r="G78" s="20"/>
+      <c r="H78" s="21"/>
+      <c r="I78" s="21"/>
+      <c r="J78" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K78" s="26"/>
+      <c r="K78" s="24"/>
       <c r="L78" s="4"/>
       <c r="M78" s="5"/>
       <c r="N78" s="2" t="str">
@@ -3661,14 +3663,14 @@
         <v/>
       </c>
       <c r="F79" s="7"/>
-      <c r="G79" s="22"/>
-      <c r="H79" s="23"/>
-      <c r="I79" s="23"/>
-      <c r="J79" s="25" t="str">
+      <c r="G79" s="20"/>
+      <c r="H79" s="21"/>
+      <c r="I79" s="21"/>
+      <c r="J79" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K79" s="26"/>
+      <c r="K79" s="24"/>
       <c r="L79" s="4"/>
       <c r="M79" s="5"/>
       <c r="N79" s="2" t="str">
@@ -3698,14 +3700,14 @@
         <v/>
       </c>
       <c r="F80" s="7"/>
-      <c r="G80" s="22"/>
-      <c r="H80" s="23"/>
-      <c r="I80" s="23"/>
-      <c r="J80" s="25" t="str">
+      <c r="G80" s="20"/>
+      <c r="H80" s="21"/>
+      <c r="I80" s="21"/>
+      <c r="J80" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K80" s="26"/>
+      <c r="K80" s="24"/>
       <c r="L80" s="4"/>
       <c r="M80" s="5"/>
       <c r="N80" s="2" t="str">
@@ -3735,14 +3737,14 @@
         <v/>
       </c>
       <c r="F81" s="7"/>
-      <c r="G81" s="22"/>
-      <c r="H81" s="23"/>
-      <c r="I81" s="23"/>
-      <c r="J81" s="25" t="str">
+      <c r="G81" s="20"/>
+      <c r="H81" s="21"/>
+      <c r="I81" s="21"/>
+      <c r="J81" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K81" s="26"/>
+      <c r="K81" s="24"/>
       <c r="L81" s="4"/>
       <c r="M81" s="5"/>
       <c r="N81" s="2" t="str">
@@ -3772,14 +3774,14 @@
         <v/>
       </c>
       <c r="F82" s="7"/>
-      <c r="G82" s="22"/>
-      <c r="H82" s="23"/>
-      <c r="I82" s="23"/>
-      <c r="J82" s="25" t="str">
+      <c r="G82" s="20"/>
+      <c r="H82" s="21"/>
+      <c r="I82" s="21"/>
+      <c r="J82" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K82" s="26"/>
+      <c r="K82" s="24"/>
       <c r="L82" s="4"/>
       <c r="M82" s="5"/>
       <c r="N82" s="2" t="str">
@@ -3809,14 +3811,14 @@
         <v/>
       </c>
       <c r="F83" s="7"/>
-      <c r="G83" s="22"/>
-      <c r="H83" s="23"/>
-      <c r="I83" s="23"/>
-      <c r="J83" s="25" t="str">
+      <c r="G83" s="20"/>
+      <c r="H83" s="21"/>
+      <c r="I83" s="21"/>
+      <c r="J83" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K83" s="26"/>
+      <c r="K83" s="24"/>
       <c r="L83" s="4"/>
       <c r="M83" s="5"/>
       <c r="N83" s="2" t="str">
@@ -3846,14 +3848,14 @@
         <v/>
       </c>
       <c r="F84" s="7"/>
-      <c r="G84" s="22"/>
-      <c r="H84" s="23"/>
-      <c r="I84" s="23"/>
-      <c r="J84" s="25" t="str">
+      <c r="G84" s="20"/>
+      <c r="H84" s="21"/>
+      <c r="I84" s="21"/>
+      <c r="J84" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K84" s="26"/>
+      <c r="K84" s="24"/>
       <c r="L84" s="4"/>
       <c r="M84" s="5"/>
       <c r="N84" s="2" t="str">
@@ -3883,14 +3885,14 @@
         <v/>
       </c>
       <c r="F85" s="7"/>
-      <c r="G85" s="22"/>
-      <c r="H85" s="23"/>
-      <c r="I85" s="23"/>
-      <c r="J85" s="25" t="str">
+      <c r="G85" s="20"/>
+      <c r="H85" s="21"/>
+      <c r="I85" s="21"/>
+      <c r="J85" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K85" s="26"/>
+      <c r="K85" s="24"/>
       <c r="L85" s="4"/>
       <c r="M85" s="5"/>
       <c r="N85" s="2" t="str">
@@ -3920,14 +3922,14 @@
         <v/>
       </c>
       <c r="F86" s="7"/>
-      <c r="G86" s="22"/>
-      <c r="H86" s="23"/>
-      <c r="I86" s="23"/>
-      <c r="J86" s="25" t="str">
+      <c r="G86" s="20"/>
+      <c r="H86" s="21"/>
+      <c r="I86" s="21"/>
+      <c r="J86" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K86" s="26"/>
+      <c r="K86" s="24"/>
       <c r="L86" s="4"/>
       <c r="M86" s="5"/>
       <c r="N86" s="2" t="str">
@@ -3957,14 +3959,14 @@
         <v/>
       </c>
       <c r="F87" s="7"/>
-      <c r="G87" s="22"/>
-      <c r="H87" s="23"/>
-      <c r="I87" s="23"/>
-      <c r="J87" s="25" t="str">
+      <c r="G87" s="20"/>
+      <c r="H87" s="21"/>
+      <c r="I87" s="21"/>
+      <c r="J87" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K87" s="26"/>
+      <c r="K87" s="24"/>
       <c r="L87" s="4"/>
       <c r="M87" s="5"/>
       <c r="N87" s="2" t="str">
@@ -3994,14 +3996,14 @@
         <v/>
       </c>
       <c r="F88" s="7"/>
-      <c r="G88" s="22"/>
-      <c r="H88" s="23"/>
-      <c r="I88" s="23"/>
-      <c r="J88" s="25" t="str">
+      <c r="G88" s="20"/>
+      <c r="H88" s="21"/>
+      <c r="I88" s="21"/>
+      <c r="J88" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K88" s="26"/>
+      <c r="K88" s="24"/>
       <c r="L88" s="4"/>
       <c r="M88" s="5"/>
       <c r="N88" s="2" t="str">
@@ -4031,14 +4033,14 @@
         <v/>
       </c>
       <c r="F89" s="7"/>
-      <c r="G89" s="22"/>
-      <c r="H89" s="23"/>
-      <c r="I89" s="23"/>
-      <c r="J89" s="25" t="str">
+      <c r="G89" s="20"/>
+      <c r="H89" s="21"/>
+      <c r="I89" s="21"/>
+      <c r="J89" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K89" s="26"/>
+      <c r="K89" s="24"/>
       <c r="L89" s="4"/>
       <c r="M89" s="5"/>
       <c r="N89" s="2" t="str">
@@ -4068,14 +4070,14 @@
         <v/>
       </c>
       <c r="F90" s="7"/>
-      <c r="G90" s="22"/>
-      <c r="H90" s="23"/>
-      <c r="I90" s="23"/>
-      <c r="J90" s="25" t="str">
+      <c r="G90" s="20"/>
+      <c r="H90" s="21"/>
+      <c r="I90" s="21"/>
+      <c r="J90" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K90" s="26"/>
+      <c r="K90" s="24"/>
       <c r="L90" s="4"/>
       <c r="M90" s="5"/>
       <c r="N90" s="2" t="str">
@@ -4105,14 +4107,14 @@
         <v/>
       </c>
       <c r="F91" s="7"/>
-      <c r="G91" s="22"/>
-      <c r="H91" s="23"/>
-      <c r="I91" s="23"/>
-      <c r="J91" s="25" t="str">
+      <c r="G91" s="20"/>
+      <c r="H91" s="21"/>
+      <c r="I91" s="21"/>
+      <c r="J91" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K91" s="26"/>
+      <c r="K91" s="24"/>
       <c r="L91" s="4"/>
       <c r="M91" s="5"/>
       <c r="N91" s="2" t="str">
@@ -4142,14 +4144,14 @@
         <v/>
       </c>
       <c r="F92" s="7"/>
-      <c r="G92" s="22"/>
-      <c r="H92" s="23"/>
-      <c r="I92" s="23"/>
-      <c r="J92" s="25" t="str">
+      <c r="G92" s="20"/>
+      <c r="H92" s="21"/>
+      <c r="I92" s="21"/>
+      <c r="J92" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K92" s="26"/>
+      <c r="K92" s="24"/>
       <c r="L92" s="4"/>
       <c r="M92" s="5"/>
       <c r="N92" s="2" t="str">
@@ -4179,14 +4181,14 @@
         <v/>
       </c>
       <c r="F93" s="7"/>
-      <c r="G93" s="22"/>
-      <c r="H93" s="23"/>
-      <c r="I93" s="23"/>
-      <c r="J93" s="25" t="str">
+      <c r="G93" s="20"/>
+      <c r="H93" s="21"/>
+      <c r="I93" s="21"/>
+      <c r="J93" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K93" s="26"/>
+      <c r="K93" s="24"/>
       <c r="L93" s="4"/>
       <c r="M93" s="5"/>
       <c r="N93" s="2" t="str">
@@ -4216,14 +4218,14 @@
         <v/>
       </c>
       <c r="F94" s="7"/>
-      <c r="G94" s="22"/>
-      <c r="H94" s="23"/>
-      <c r="I94" s="23"/>
-      <c r="J94" s="25" t="str">
+      <c r="G94" s="20"/>
+      <c r="H94" s="21"/>
+      <c r="I94" s="21"/>
+      <c r="J94" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K94" s="26"/>
+      <c r="K94" s="24"/>
       <c r="L94" s="4"/>
       <c r="M94" s="5"/>
       <c r="N94" s="2" t="str">
@@ -4253,14 +4255,14 @@
         <v/>
       </c>
       <c r="F95" s="7"/>
-      <c r="G95" s="22"/>
-      <c r="H95" s="23"/>
-      <c r="I95" s="23"/>
-      <c r="J95" s="25" t="str">
+      <c r="G95" s="20"/>
+      <c r="H95" s="21"/>
+      <c r="I95" s="21"/>
+      <c r="J95" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K95" s="26"/>
+      <c r="K95" s="24"/>
       <c r="L95" s="4"/>
       <c r="M95" s="5"/>
       <c r="N95" s="2" t="str">
@@ -4290,14 +4292,14 @@
         <v/>
       </c>
       <c r="F96" s="7"/>
-      <c r="G96" s="22"/>
-      <c r="H96" s="23"/>
-      <c r="I96" s="23"/>
-      <c r="J96" s="25" t="str">
+      <c r="G96" s="20"/>
+      <c r="H96" s="21"/>
+      <c r="I96" s="21"/>
+      <c r="J96" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K96" s="26"/>
+      <c r="K96" s="24"/>
       <c r="L96" s="4"/>
       <c r="M96" s="5"/>
       <c r="N96" s="2" t="str">
@@ -4327,14 +4329,14 @@
         <v/>
       </c>
       <c r="F97" s="7"/>
-      <c r="G97" s="22"/>
-      <c r="H97" s="23"/>
-      <c r="I97" s="23"/>
-      <c r="J97" s="25" t="str">
+      <c r="G97" s="20"/>
+      <c r="H97" s="21"/>
+      <c r="I97" s="21"/>
+      <c r="J97" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K97" s="26"/>
+      <c r="K97" s="24"/>
       <c r="L97" s="4"/>
       <c r="M97" s="5"/>
       <c r="N97" s="2" t="str">
@@ -4364,14 +4366,14 @@
         <v/>
       </c>
       <c r="F98" s="7"/>
-      <c r="G98" s="22"/>
-      <c r="H98" s="23"/>
-      <c r="I98" s="23"/>
-      <c r="J98" s="25" t="str">
+      <c r="G98" s="20"/>
+      <c r="H98" s="21"/>
+      <c r="I98" s="21"/>
+      <c r="J98" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K98" s="26"/>
+      <c r="K98" s="24"/>
       <c r="L98" s="4"/>
       <c r="M98" s="5"/>
       <c r="N98" s="2" t="str">
@@ -4401,14 +4403,14 @@
         <v/>
       </c>
       <c r="F99" s="7"/>
-      <c r="G99" s="22"/>
-      <c r="H99" s="23"/>
-      <c r="I99" s="23"/>
-      <c r="J99" s="25" t="str">
+      <c r="G99" s="20"/>
+      <c r="H99" s="21"/>
+      <c r="I99" s="21"/>
+      <c r="J99" s="23" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="K99" s="26"/>
+      <c r="K99" s="24"/>
       <c r="L99" s="4"/>
       <c r="M99" s="5"/>
       <c r="N99" s="2" t="str">
@@ -4438,14 +4440,14 @@
         <v/>
       </c>
       <c r="F100" s="7"/>
-      <c r="G100" s="22"/>
-      <c r="H100" s="23"/>
-      <c r="I100" s="23"/>
-      <c r="J100" s="25" t="str">
+      <c r="G100" s="20"/>
+      <c r="H100" s="21"/>
+      <c r="I100" s="21"/>
+      <c r="J100" s="23" t="str">
         <f t="shared" ref="J100:J131" si="20">IF(OR(I100="",H100=""),"",MAX(0,I100-H100))</f>
         <v/>
       </c>
-      <c r="K100" s="26"/>
+      <c r="K100" s="24"/>
       <c r="L100" s="4"/>
       <c r="M100" s="5"/>
       <c r="N100" s="2" t="str">
@@ -4453,11 +4455,11 @@
         <v/>
       </c>
       <c r="O100" s="6" t="str">
-        <f t="shared" ref="O100:O131" si="22">IF(L100="","",L100*0.05)</f>
+        <f t="shared" ref="O100:O131" si="22">IF(L100="","",L100*0.06)</f>
         <v/>
       </c>
       <c r="P100" s="6" t="str">
-        <f t="shared" ref="P100:P131" si="23">IF(OR(L100="",C100=""),"",L100*0.95-C100)</f>
+        <f t="shared" ref="P100:P131" si="23">IF(OR(L100="",C100=""),"",L100*0.94-C100)</f>
         <v/>
       </c>
       <c r="Q100" s="3"/>
@@ -4475,14 +4477,14 @@
         <v/>
       </c>
       <c r="F101" s="7"/>
-      <c r="G101" s="22"/>
-      <c r="H101" s="23"/>
-      <c r="I101" s="23"/>
-      <c r="J101" s="25" t="str">
+      <c r="G101" s="20"/>
+      <c r="H101" s="21"/>
+      <c r="I101" s="21"/>
+      <c r="J101" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K101" s="26"/>
+      <c r="K101" s="24"/>
       <c r="L101" s="4"/>
       <c r="M101" s="5"/>
       <c r="N101" s="2" t="str">
@@ -4512,14 +4514,14 @@
         <v/>
       </c>
       <c r="F102" s="7"/>
-      <c r="G102" s="22"/>
-      <c r="H102" s="23"/>
-      <c r="I102" s="23"/>
-      <c r="J102" s="25" t="str">
+      <c r="G102" s="20"/>
+      <c r="H102" s="21"/>
+      <c r="I102" s="21"/>
+      <c r="J102" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K102" s="26"/>
+      <c r="K102" s="24"/>
       <c r="L102" s="4"/>
       <c r="M102" s="5"/>
       <c r="N102" s="2" t="str">
@@ -4549,14 +4551,14 @@
         <v/>
       </c>
       <c r="F103" s="7"/>
-      <c r="G103" s="22"/>
-      <c r="H103" s="23"/>
-      <c r="I103" s="23"/>
-      <c r="J103" s="25" t="str">
+      <c r="G103" s="20"/>
+      <c r="H103" s="21"/>
+      <c r="I103" s="21"/>
+      <c r="J103" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K103" s="26"/>
+      <c r="K103" s="24"/>
       <c r="L103" s="4"/>
       <c r="M103" s="5"/>
       <c r="N103" s="2" t="str">
@@ -4586,14 +4588,14 @@
         <v/>
       </c>
       <c r="F104" s="7"/>
-      <c r="G104" s="22"/>
-      <c r="H104" s="23"/>
-      <c r="I104" s="23"/>
-      <c r="J104" s="25" t="str">
+      <c r="G104" s="20"/>
+      <c r="H104" s="21"/>
+      <c r="I104" s="21"/>
+      <c r="J104" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K104" s="26"/>
+      <c r="K104" s="24"/>
       <c r="L104" s="4"/>
       <c r="M104" s="5"/>
       <c r="N104" s="2" t="str">
@@ -4623,14 +4625,14 @@
         <v/>
       </c>
       <c r="F105" s="7"/>
-      <c r="G105" s="22"/>
-      <c r="H105" s="23"/>
-      <c r="I105" s="23"/>
-      <c r="J105" s="25" t="str">
+      <c r="G105" s="20"/>
+      <c r="H105" s="21"/>
+      <c r="I105" s="21"/>
+      <c r="J105" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K105" s="26"/>
+      <c r="K105" s="24"/>
       <c r="L105" s="4"/>
       <c r="M105" s="5"/>
       <c r="N105" s="2" t="str">
@@ -4660,14 +4662,14 @@
         <v/>
       </c>
       <c r="F106" s="7"/>
-      <c r="G106" s="22"/>
-      <c r="H106" s="23"/>
-      <c r="I106" s="23"/>
-      <c r="J106" s="25" t="str">
+      <c r="G106" s="20"/>
+      <c r="H106" s="21"/>
+      <c r="I106" s="21"/>
+      <c r="J106" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K106" s="26"/>
+      <c r="K106" s="24"/>
       <c r="L106" s="4"/>
       <c r="M106" s="5"/>
       <c r="N106" s="2" t="str">
@@ -4697,14 +4699,14 @@
         <v/>
       </c>
       <c r="F107" s="7"/>
-      <c r="G107" s="22"/>
-      <c r="H107" s="23"/>
-      <c r="I107" s="23"/>
-      <c r="J107" s="25" t="str">
+      <c r="G107" s="20"/>
+      <c r="H107" s="21"/>
+      <c r="I107" s="21"/>
+      <c r="J107" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K107" s="26"/>
+      <c r="K107" s="24"/>
       <c r="L107" s="4"/>
       <c r="M107" s="5"/>
       <c r="N107" s="2" t="str">
@@ -4734,14 +4736,14 @@
         <v/>
       </c>
       <c r="F108" s="7"/>
-      <c r="G108" s="22"/>
-      <c r="H108" s="23"/>
-      <c r="I108" s="23"/>
-      <c r="J108" s="25" t="str">
+      <c r="G108" s="20"/>
+      <c r="H108" s="21"/>
+      <c r="I108" s="21"/>
+      <c r="J108" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K108" s="26"/>
+      <c r="K108" s="24"/>
       <c r="L108" s="4"/>
       <c r="M108" s="5"/>
       <c r="N108" s="2" t="str">
@@ -4771,14 +4773,14 @@
         <v/>
       </c>
       <c r="F109" s="7"/>
-      <c r="G109" s="22"/>
-      <c r="H109" s="23"/>
-      <c r="I109" s="23"/>
-      <c r="J109" s="25" t="str">
+      <c r="G109" s="20"/>
+      <c r="H109" s="21"/>
+      <c r="I109" s="21"/>
+      <c r="J109" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K109" s="26"/>
+      <c r="K109" s="24"/>
       <c r="L109" s="4"/>
       <c r="M109" s="5"/>
       <c r="N109" s="2" t="str">
@@ -4808,14 +4810,14 @@
         <v/>
       </c>
       <c r="F110" s="7"/>
-      <c r="G110" s="22"/>
-      <c r="H110" s="23"/>
-      <c r="I110" s="23"/>
-      <c r="J110" s="25" t="str">
+      <c r="G110" s="20"/>
+      <c r="H110" s="21"/>
+      <c r="I110" s="21"/>
+      <c r="J110" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K110" s="26"/>
+      <c r="K110" s="24"/>
       <c r="L110" s="4"/>
       <c r="M110" s="5"/>
       <c r="N110" s="2" t="str">
@@ -4845,14 +4847,14 @@
         <v/>
       </c>
       <c r="F111" s="7"/>
-      <c r="G111" s="22"/>
-      <c r="H111" s="23"/>
-      <c r="I111" s="23"/>
-      <c r="J111" s="25" t="str">
+      <c r="G111" s="20"/>
+      <c r="H111" s="21"/>
+      <c r="I111" s="21"/>
+      <c r="J111" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K111" s="26"/>
+      <c r="K111" s="24"/>
       <c r="L111" s="4"/>
       <c r="M111" s="5"/>
       <c r="N111" s="2" t="str">
@@ -4882,14 +4884,14 @@
         <v/>
       </c>
       <c r="F112" s="7"/>
-      <c r="G112" s="22"/>
-      <c r="H112" s="23"/>
-      <c r="I112" s="23"/>
-      <c r="J112" s="25" t="str">
+      <c r="G112" s="20"/>
+      <c r="H112" s="21"/>
+      <c r="I112" s="21"/>
+      <c r="J112" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K112" s="26"/>
+      <c r="K112" s="24"/>
       <c r="L112" s="4"/>
       <c r="M112" s="5"/>
       <c r="N112" s="2" t="str">
@@ -4919,14 +4921,14 @@
         <v/>
       </c>
       <c r="F113" s="7"/>
-      <c r="G113" s="22"/>
-      <c r="H113" s="23"/>
-      <c r="I113" s="23"/>
-      <c r="J113" s="25" t="str">
+      <c r="G113" s="20"/>
+      <c r="H113" s="21"/>
+      <c r="I113" s="21"/>
+      <c r="J113" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K113" s="26"/>
+      <c r="K113" s="24"/>
       <c r="L113" s="4"/>
       <c r="M113" s="5"/>
       <c r="N113" s="2" t="str">
@@ -4956,14 +4958,14 @@
         <v/>
       </c>
       <c r="F114" s="7"/>
-      <c r="G114" s="22"/>
-      <c r="H114" s="23"/>
-      <c r="I114" s="23"/>
-      <c r="J114" s="25" t="str">
+      <c r="G114" s="20"/>
+      <c r="H114" s="21"/>
+      <c r="I114" s="21"/>
+      <c r="J114" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K114" s="26"/>
+      <c r="K114" s="24"/>
       <c r="L114" s="4"/>
       <c r="M114" s="5"/>
       <c r="N114" s="2" t="str">
@@ -4993,14 +4995,14 @@
         <v/>
       </c>
       <c r="F115" s="7"/>
-      <c r="G115" s="22"/>
-      <c r="H115" s="23"/>
-      <c r="I115" s="23"/>
-      <c r="J115" s="25" t="str">
+      <c r="G115" s="20"/>
+      <c r="H115" s="21"/>
+      <c r="I115" s="21"/>
+      <c r="J115" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K115" s="26"/>
+      <c r="K115" s="24"/>
       <c r="L115" s="4"/>
       <c r="M115" s="5"/>
       <c r="N115" s="2" t="str">
@@ -5030,14 +5032,14 @@
         <v/>
       </c>
       <c r="F116" s="7"/>
-      <c r="G116" s="22"/>
-      <c r="H116" s="23"/>
-      <c r="I116" s="23"/>
-      <c r="J116" s="25" t="str">
+      <c r="G116" s="20"/>
+      <c r="H116" s="21"/>
+      <c r="I116" s="21"/>
+      <c r="J116" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K116" s="26"/>
+      <c r="K116" s="24"/>
       <c r="L116" s="4"/>
       <c r="M116" s="5"/>
       <c r="N116" s="2" t="str">
@@ -5067,14 +5069,14 @@
         <v/>
       </c>
       <c r="F117" s="7"/>
-      <c r="G117" s="22"/>
-      <c r="H117" s="23"/>
-      <c r="I117" s="23"/>
-      <c r="J117" s="25" t="str">
+      <c r="G117" s="20"/>
+      <c r="H117" s="21"/>
+      <c r="I117" s="21"/>
+      <c r="J117" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K117" s="26"/>
+      <c r="K117" s="24"/>
       <c r="L117" s="4"/>
       <c r="M117" s="5"/>
       <c r="N117" s="2" t="str">
@@ -5104,14 +5106,14 @@
         <v/>
       </c>
       <c r="F118" s="7"/>
-      <c r="G118" s="22"/>
-      <c r="H118" s="23"/>
-      <c r="I118" s="23"/>
-      <c r="J118" s="25" t="str">
+      <c r="G118" s="20"/>
+      <c r="H118" s="21"/>
+      <c r="I118" s="21"/>
+      <c r="J118" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K118" s="26"/>
+      <c r="K118" s="24"/>
       <c r="L118" s="4"/>
       <c r="M118" s="5"/>
       <c r="N118" s="2" t="str">
@@ -5141,14 +5143,14 @@
         <v/>
       </c>
       <c r="F119" s="7"/>
-      <c r="G119" s="22"/>
-      <c r="H119" s="23"/>
-      <c r="I119" s="23"/>
-      <c r="J119" s="25" t="str">
+      <c r="G119" s="20"/>
+      <c r="H119" s="21"/>
+      <c r="I119" s="21"/>
+      <c r="J119" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K119" s="26"/>
+      <c r="K119" s="24"/>
       <c r="L119" s="4"/>
       <c r="M119" s="5"/>
       <c r="N119" s="2" t="str">
@@ -5178,14 +5180,14 @@
         <v/>
       </c>
       <c r="F120" s="7"/>
-      <c r="G120" s="22"/>
-      <c r="H120" s="23"/>
-      <c r="I120" s="23"/>
-      <c r="J120" s="25" t="str">
+      <c r="G120" s="20"/>
+      <c r="H120" s="21"/>
+      <c r="I120" s="21"/>
+      <c r="J120" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K120" s="26"/>
+      <c r="K120" s="24"/>
       <c r="L120" s="4"/>
       <c r="M120" s="5"/>
       <c r="N120" s="2" t="str">
@@ -5215,14 +5217,14 @@
         <v/>
       </c>
       <c r="F121" s="7"/>
-      <c r="G121" s="22"/>
-      <c r="H121" s="23"/>
-      <c r="I121" s="23"/>
-      <c r="J121" s="25" t="str">
+      <c r="G121" s="20"/>
+      <c r="H121" s="21"/>
+      <c r="I121" s="21"/>
+      <c r="J121" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K121" s="26"/>
+      <c r="K121" s="24"/>
       <c r="L121" s="4"/>
       <c r="M121" s="5"/>
       <c r="N121" s="2" t="str">
@@ -5252,14 +5254,14 @@
         <v/>
       </c>
       <c r="F122" s="7"/>
-      <c r="G122" s="22"/>
-      <c r="H122" s="23"/>
-      <c r="I122" s="23"/>
-      <c r="J122" s="25" t="str">
+      <c r="G122" s="20"/>
+      <c r="H122" s="21"/>
+      <c r="I122" s="21"/>
+      <c r="J122" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K122" s="26"/>
+      <c r="K122" s="24"/>
       <c r="L122" s="4"/>
       <c r="M122" s="5"/>
       <c r="N122" s="2" t="str">
@@ -5289,14 +5291,14 @@
         <v/>
       </c>
       <c r="F123" s="7"/>
-      <c r="G123" s="22"/>
-      <c r="H123" s="23"/>
-      <c r="I123" s="23"/>
-      <c r="J123" s="25" t="str">
+      <c r="G123" s="20"/>
+      <c r="H123" s="21"/>
+      <c r="I123" s="21"/>
+      <c r="J123" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K123" s="26"/>
+      <c r="K123" s="24"/>
       <c r="L123" s="4"/>
       <c r="M123" s="5"/>
       <c r="N123" s="2" t="str">
@@ -5326,14 +5328,14 @@
         <v/>
       </c>
       <c r="F124" s="7"/>
-      <c r="G124" s="22"/>
-      <c r="H124" s="23"/>
-      <c r="I124" s="23"/>
-      <c r="J124" s="25" t="str">
+      <c r="G124" s="20"/>
+      <c r="H124" s="21"/>
+      <c r="I124" s="21"/>
+      <c r="J124" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K124" s="26"/>
+      <c r="K124" s="24"/>
       <c r="L124" s="4"/>
       <c r="M124" s="5"/>
       <c r="N124" s="2" t="str">
@@ -5363,14 +5365,14 @@
         <v/>
       </c>
       <c r="F125" s="7"/>
-      <c r="G125" s="22"/>
-      <c r="H125" s="23"/>
-      <c r="I125" s="23"/>
-      <c r="J125" s="25" t="str">
+      <c r="G125" s="20"/>
+      <c r="H125" s="21"/>
+      <c r="I125" s="21"/>
+      <c r="J125" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K125" s="26"/>
+      <c r="K125" s="24"/>
       <c r="L125" s="4"/>
       <c r="M125" s="5"/>
       <c r="N125" s="2" t="str">
@@ -5400,14 +5402,14 @@
         <v/>
       </c>
       <c r="F126" s="7"/>
-      <c r="G126" s="22"/>
-      <c r="H126" s="23"/>
-      <c r="I126" s="23"/>
-      <c r="J126" s="25" t="str">
+      <c r="G126" s="20"/>
+      <c r="H126" s="21"/>
+      <c r="I126" s="21"/>
+      <c r="J126" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K126" s="26"/>
+      <c r="K126" s="24"/>
       <c r="L126" s="4"/>
       <c r="M126" s="5"/>
       <c r="N126" s="2" t="str">
@@ -5437,14 +5439,14 @@
         <v/>
       </c>
       <c r="F127" s="7"/>
-      <c r="G127" s="22"/>
-      <c r="H127" s="23"/>
-      <c r="I127" s="23"/>
-      <c r="J127" s="25" t="str">
+      <c r="G127" s="20"/>
+      <c r="H127" s="21"/>
+      <c r="I127" s="21"/>
+      <c r="J127" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K127" s="26"/>
+      <c r="K127" s="24"/>
       <c r="L127" s="4"/>
       <c r="M127" s="5"/>
       <c r="N127" s="2" t="str">
@@ -5474,14 +5476,14 @@
         <v/>
       </c>
       <c r="F128" s="7"/>
-      <c r="G128" s="22"/>
-      <c r="H128" s="23"/>
-      <c r="I128" s="23"/>
-      <c r="J128" s="25" t="str">
+      <c r="G128" s="20"/>
+      <c r="H128" s="21"/>
+      <c r="I128" s="21"/>
+      <c r="J128" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K128" s="26"/>
+      <c r="K128" s="24"/>
       <c r="L128" s="4"/>
       <c r="M128" s="5"/>
       <c r="N128" s="2" t="str">
@@ -5511,14 +5513,14 @@
         <v/>
       </c>
       <c r="F129" s="7"/>
-      <c r="G129" s="22"/>
-      <c r="H129" s="23"/>
-      <c r="I129" s="23"/>
-      <c r="J129" s="25" t="str">
+      <c r="G129" s="20"/>
+      <c r="H129" s="21"/>
+      <c r="I129" s="21"/>
+      <c r="J129" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K129" s="26"/>
+      <c r="K129" s="24"/>
       <c r="L129" s="4"/>
       <c r="M129" s="5"/>
       <c r="N129" s="2" t="str">
@@ -5548,14 +5550,14 @@
         <v/>
       </c>
       <c r="F130" s="7"/>
-      <c r="G130" s="22"/>
-      <c r="H130" s="23"/>
-      <c r="I130" s="23"/>
-      <c r="J130" s="25" t="str">
+      <c r="G130" s="20"/>
+      <c r="H130" s="21"/>
+      <c r="I130" s="21"/>
+      <c r="J130" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K130" s="26"/>
+      <c r="K130" s="24"/>
       <c r="L130" s="4"/>
       <c r="M130" s="5"/>
       <c r="N130" s="2" t="str">
@@ -5585,14 +5587,14 @@
         <v/>
       </c>
       <c r="F131" s="7"/>
-      <c r="G131" s="22"/>
-      <c r="H131" s="23"/>
-      <c r="I131" s="23"/>
-      <c r="J131" s="25" t="str">
+      <c r="G131" s="20"/>
+      <c r="H131" s="21"/>
+      <c r="I131" s="21"/>
+      <c r="J131" s="23" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="K131" s="26"/>
+      <c r="K131" s="24"/>
       <c r="L131" s="4"/>
       <c r="M131" s="5"/>
       <c r="N131" s="2" t="str">
@@ -5622,14 +5624,14 @@
         <v/>
       </c>
       <c r="F132" s="7"/>
-      <c r="G132" s="22"/>
-      <c r="H132" s="23"/>
-      <c r="I132" s="23"/>
-      <c r="J132" s="25" t="str">
+      <c r="G132" s="20"/>
+      <c r="H132" s="21"/>
+      <c r="I132" s="21"/>
+      <c r="J132" s="23" t="str">
         <f t="shared" ref="J132:J163" si="26">IF(OR(I132="",H132=""),"",MAX(0,I132-H132))</f>
         <v/>
       </c>
-      <c r="K132" s="26"/>
+      <c r="K132" s="24"/>
       <c r="L132" s="4"/>
       <c r="M132" s="5"/>
       <c r="N132" s="2" t="str">
@@ -5637,11 +5639,11 @@
         <v/>
       </c>
       <c r="O132" s="6" t="str">
-        <f t="shared" ref="O132:O163" si="28">IF(L132="","",L132*0.05)</f>
+        <f t="shared" ref="O132:O163" si="28">IF(L132="","",L132*0.06)</f>
         <v/>
       </c>
       <c r="P132" s="6" t="str">
-        <f t="shared" ref="P132:P163" si="29">IF(OR(L132="",C132=""),"",L132*0.95-C132)</f>
+        <f t="shared" ref="P132:P163" si="29">IF(OR(L132="",C132=""),"",L132*0.94-C132)</f>
         <v/>
       </c>
       <c r="Q132" s="3"/>
@@ -5659,14 +5661,14 @@
         <v/>
       </c>
       <c r="F133" s="7"/>
-      <c r="G133" s="22"/>
-      <c r="H133" s="23"/>
-      <c r="I133" s="23"/>
-      <c r="J133" s="25" t="str">
+      <c r="G133" s="20"/>
+      <c r="H133" s="21"/>
+      <c r="I133" s="21"/>
+      <c r="J133" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K133" s="26"/>
+      <c r="K133" s="24"/>
       <c r="L133" s="4"/>
       <c r="M133" s="5"/>
       <c r="N133" s="2" t="str">
@@ -5696,14 +5698,14 @@
         <v/>
       </c>
       <c r="F134" s="7"/>
-      <c r="G134" s="22"/>
-      <c r="H134" s="23"/>
-      <c r="I134" s="23"/>
-      <c r="J134" s="25" t="str">
+      <c r="G134" s="20"/>
+      <c r="H134" s="21"/>
+      <c r="I134" s="21"/>
+      <c r="J134" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K134" s="26"/>
+      <c r="K134" s="24"/>
       <c r="L134" s="4"/>
       <c r="M134" s="5"/>
       <c r="N134" s="2" t="str">
@@ -5733,14 +5735,14 @@
         <v/>
       </c>
       <c r="F135" s="7"/>
-      <c r="G135" s="22"/>
-      <c r="H135" s="23"/>
-      <c r="I135" s="23"/>
-      <c r="J135" s="25" t="str">
+      <c r="G135" s="20"/>
+      <c r="H135" s="21"/>
+      <c r="I135" s="21"/>
+      <c r="J135" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K135" s="26"/>
+      <c r="K135" s="24"/>
       <c r="L135" s="4"/>
       <c r="M135" s="5"/>
       <c r="N135" s="2" t="str">
@@ -5770,14 +5772,14 @@
         <v/>
       </c>
       <c r="F136" s="7"/>
-      <c r="G136" s="22"/>
-      <c r="H136" s="23"/>
-      <c r="I136" s="23"/>
-      <c r="J136" s="25" t="str">
+      <c r="G136" s="20"/>
+      <c r="H136" s="21"/>
+      <c r="I136" s="21"/>
+      <c r="J136" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K136" s="26"/>
+      <c r="K136" s="24"/>
       <c r="L136" s="4"/>
       <c r="M136" s="5"/>
       <c r="N136" s="2" t="str">
@@ -5807,14 +5809,14 @@
         <v/>
       </c>
       <c r="F137" s="7"/>
-      <c r="G137" s="22"/>
-      <c r="H137" s="23"/>
-      <c r="I137" s="23"/>
-      <c r="J137" s="25" t="str">
+      <c r="G137" s="20"/>
+      <c r="H137" s="21"/>
+      <c r="I137" s="21"/>
+      <c r="J137" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K137" s="26"/>
+      <c r="K137" s="24"/>
       <c r="L137" s="4"/>
       <c r="M137" s="5"/>
       <c r="N137" s="2" t="str">
@@ -5844,14 +5846,14 @@
         <v/>
       </c>
       <c r="F138" s="7"/>
-      <c r="G138" s="22"/>
-      <c r="H138" s="23"/>
-      <c r="I138" s="23"/>
-      <c r="J138" s="25" t="str">
+      <c r="G138" s="20"/>
+      <c r="H138" s="21"/>
+      <c r="I138" s="21"/>
+      <c r="J138" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K138" s="26"/>
+      <c r="K138" s="24"/>
       <c r="L138" s="4"/>
       <c r="M138" s="5"/>
       <c r="N138" s="2" t="str">
@@ -5881,14 +5883,14 @@
         <v/>
       </c>
       <c r="F139" s="7"/>
-      <c r="G139" s="22"/>
-      <c r="H139" s="23"/>
-      <c r="I139" s="23"/>
-      <c r="J139" s="25" t="str">
+      <c r="G139" s="20"/>
+      <c r="H139" s="21"/>
+      <c r="I139" s="21"/>
+      <c r="J139" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K139" s="26"/>
+      <c r="K139" s="24"/>
       <c r="L139" s="4"/>
       <c r="M139" s="5"/>
       <c r="N139" s="2" t="str">
@@ -5918,14 +5920,14 @@
         <v/>
       </c>
       <c r="F140" s="7"/>
-      <c r="G140" s="22"/>
-      <c r="H140" s="23"/>
-      <c r="I140" s="23"/>
-      <c r="J140" s="25" t="str">
+      <c r="G140" s="20"/>
+      <c r="H140" s="21"/>
+      <c r="I140" s="21"/>
+      <c r="J140" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K140" s="26"/>
+      <c r="K140" s="24"/>
       <c r="L140" s="4"/>
       <c r="M140" s="5"/>
       <c r="N140" s="2" t="str">
@@ -5955,14 +5957,14 @@
         <v/>
       </c>
       <c r="F141" s="7"/>
-      <c r="G141" s="22"/>
-      <c r="H141" s="23"/>
-      <c r="I141" s="23"/>
-      <c r="J141" s="25" t="str">
+      <c r="G141" s="20"/>
+      <c r="H141" s="21"/>
+      <c r="I141" s="21"/>
+      <c r="J141" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K141" s="26"/>
+      <c r="K141" s="24"/>
       <c r="L141" s="4"/>
       <c r="M141" s="5"/>
       <c r="N141" s="2" t="str">
@@ -5992,14 +5994,14 @@
         <v/>
       </c>
       <c r="F142" s="7"/>
-      <c r="G142" s="22"/>
-      <c r="H142" s="23"/>
-      <c r="I142" s="23"/>
-      <c r="J142" s="25" t="str">
+      <c r="G142" s="20"/>
+      <c r="H142" s="21"/>
+      <c r="I142" s="21"/>
+      <c r="J142" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K142" s="26"/>
+      <c r="K142" s="24"/>
       <c r="L142" s="4"/>
       <c r="M142" s="5"/>
       <c r="N142" s="2" t="str">
@@ -6029,14 +6031,14 @@
         <v/>
       </c>
       <c r="F143" s="7"/>
-      <c r="G143" s="22"/>
-      <c r="H143" s="23"/>
-      <c r="I143" s="23"/>
-      <c r="J143" s="25" t="str">
+      <c r="G143" s="20"/>
+      <c r="H143" s="21"/>
+      <c r="I143" s="21"/>
+      <c r="J143" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K143" s="26"/>
+      <c r="K143" s="24"/>
       <c r="L143" s="4"/>
       <c r="M143" s="5"/>
       <c r="N143" s="2" t="str">
@@ -6066,14 +6068,14 @@
         <v/>
       </c>
       <c r="F144" s="7"/>
-      <c r="G144" s="22"/>
-      <c r="H144" s="23"/>
-      <c r="I144" s="23"/>
-      <c r="J144" s="25" t="str">
+      <c r="G144" s="20"/>
+      <c r="H144" s="21"/>
+      <c r="I144" s="21"/>
+      <c r="J144" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K144" s="26"/>
+      <c r="K144" s="24"/>
       <c r="L144" s="4"/>
       <c r="M144" s="5"/>
       <c r="N144" s="2" t="str">
@@ -6103,14 +6105,14 @@
         <v/>
       </c>
       <c r="F145" s="7"/>
-      <c r="G145" s="22"/>
-      <c r="H145" s="23"/>
-      <c r="I145" s="23"/>
-      <c r="J145" s="25" t="str">
+      <c r="G145" s="20"/>
+      <c r="H145" s="21"/>
+      <c r="I145" s="21"/>
+      <c r="J145" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K145" s="26"/>
+      <c r="K145" s="24"/>
       <c r="L145" s="4"/>
       <c r="M145" s="5"/>
       <c r="N145" s="2" t="str">
@@ -6140,14 +6142,14 @@
         <v/>
       </c>
       <c r="F146" s="7"/>
-      <c r="G146" s="22"/>
-      <c r="H146" s="23"/>
-      <c r="I146" s="23"/>
-      <c r="J146" s="25" t="str">
+      <c r="G146" s="20"/>
+      <c r="H146" s="21"/>
+      <c r="I146" s="21"/>
+      <c r="J146" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K146" s="26"/>
+      <c r="K146" s="24"/>
       <c r="L146" s="4"/>
       <c r="M146" s="5"/>
       <c r="N146" s="2" t="str">
@@ -6177,14 +6179,14 @@
         <v/>
       </c>
       <c r="F147" s="7"/>
-      <c r="G147" s="22"/>
-      <c r="H147" s="23"/>
-      <c r="I147" s="23"/>
-      <c r="J147" s="25" t="str">
+      <c r="G147" s="20"/>
+      <c r="H147" s="21"/>
+      <c r="I147" s="21"/>
+      <c r="J147" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K147" s="26"/>
+      <c r="K147" s="24"/>
       <c r="L147" s="4"/>
       <c r="M147" s="5"/>
       <c r="N147" s="2" t="str">
@@ -6214,14 +6216,14 @@
         <v/>
       </c>
       <c r="F148" s="7"/>
-      <c r="G148" s="22"/>
-      <c r="H148" s="23"/>
-      <c r="I148" s="23"/>
-      <c r="J148" s="25" t="str">
+      <c r="G148" s="20"/>
+      <c r="H148" s="21"/>
+      <c r="I148" s="21"/>
+      <c r="J148" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K148" s="26"/>
+      <c r="K148" s="24"/>
       <c r="L148" s="4"/>
       <c r="M148" s="5"/>
       <c r="N148" s="2" t="str">
@@ -6251,14 +6253,14 @@
         <v/>
       </c>
       <c r="F149" s="7"/>
-      <c r="G149" s="22"/>
-      <c r="H149" s="23"/>
-      <c r="I149" s="23"/>
-      <c r="J149" s="25" t="str">
+      <c r="G149" s="20"/>
+      <c r="H149" s="21"/>
+      <c r="I149" s="21"/>
+      <c r="J149" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K149" s="26"/>
+      <c r="K149" s="24"/>
       <c r="L149" s="4"/>
       <c r="M149" s="5"/>
       <c r="N149" s="2" t="str">
@@ -6288,14 +6290,14 @@
         <v/>
       </c>
       <c r="F150" s="7"/>
-      <c r="G150" s="22"/>
-      <c r="H150" s="23"/>
-      <c r="I150" s="23"/>
-      <c r="J150" s="25" t="str">
+      <c r="G150" s="20"/>
+      <c r="H150" s="21"/>
+      <c r="I150" s="21"/>
+      <c r="J150" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K150" s="26"/>
+      <c r="K150" s="24"/>
       <c r="L150" s="4"/>
       <c r="M150" s="5"/>
       <c r="N150" s="2" t="str">
@@ -6325,14 +6327,14 @@
         <v/>
       </c>
       <c r="F151" s="7"/>
-      <c r="G151" s="22"/>
-      <c r="H151" s="23"/>
-      <c r="I151" s="23"/>
-      <c r="J151" s="25" t="str">
+      <c r="G151" s="20"/>
+      <c r="H151" s="21"/>
+      <c r="I151" s="21"/>
+      <c r="J151" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K151" s="26"/>
+      <c r="K151" s="24"/>
       <c r="L151" s="4"/>
       <c r="M151" s="5"/>
       <c r="N151" s="2" t="str">
@@ -6362,14 +6364,14 @@
         <v/>
       </c>
       <c r="F152" s="7"/>
-      <c r="G152" s="22"/>
-      <c r="H152" s="23"/>
-      <c r="I152" s="23"/>
-      <c r="J152" s="25" t="str">
+      <c r="G152" s="20"/>
+      <c r="H152" s="21"/>
+      <c r="I152" s="21"/>
+      <c r="J152" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K152" s="26"/>
+      <c r="K152" s="24"/>
       <c r="L152" s="4"/>
       <c r="M152" s="5"/>
       <c r="N152" s="2" t="str">
@@ -6399,14 +6401,14 @@
         <v/>
       </c>
       <c r="F153" s="7"/>
-      <c r="G153" s="22"/>
-      <c r="H153" s="23"/>
-      <c r="I153" s="23"/>
-      <c r="J153" s="25" t="str">
+      <c r="G153" s="20"/>
+      <c r="H153" s="21"/>
+      <c r="I153" s="21"/>
+      <c r="J153" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K153" s="26"/>
+      <c r="K153" s="24"/>
       <c r="L153" s="4"/>
       <c r="M153" s="5"/>
       <c r="N153" s="2" t="str">
@@ -6436,14 +6438,14 @@
         <v/>
       </c>
       <c r="F154" s="7"/>
-      <c r="G154" s="22"/>
-      <c r="H154" s="23"/>
-      <c r="I154" s="23"/>
-      <c r="J154" s="25" t="str">
+      <c r="G154" s="20"/>
+      <c r="H154" s="21"/>
+      <c r="I154" s="21"/>
+      <c r="J154" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K154" s="26"/>
+      <c r="K154" s="24"/>
       <c r="L154" s="4"/>
       <c r="M154" s="5"/>
       <c r="N154" s="2" t="str">
@@ -6473,14 +6475,14 @@
         <v/>
       </c>
       <c r="F155" s="7"/>
-      <c r="G155" s="22"/>
-      <c r="H155" s="23"/>
-      <c r="I155" s="23"/>
-      <c r="J155" s="25" t="str">
+      <c r="G155" s="20"/>
+      <c r="H155" s="21"/>
+      <c r="I155" s="21"/>
+      <c r="J155" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K155" s="26"/>
+      <c r="K155" s="24"/>
       <c r="L155" s="4"/>
       <c r="M155" s="5"/>
       <c r="N155" s="2" t="str">
@@ -6510,14 +6512,14 @@
         <v/>
       </c>
       <c r="F156" s="7"/>
-      <c r="G156" s="22"/>
-      <c r="H156" s="23"/>
-      <c r="I156" s="23"/>
-      <c r="J156" s="25" t="str">
+      <c r="G156" s="20"/>
+      <c r="H156" s="21"/>
+      <c r="I156" s="21"/>
+      <c r="J156" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K156" s="26"/>
+      <c r="K156" s="24"/>
       <c r="L156" s="4"/>
       <c r="M156" s="5"/>
       <c r="N156" s="2" t="str">
@@ -6547,14 +6549,14 @@
         <v/>
       </c>
       <c r="F157" s="7"/>
-      <c r="G157" s="22"/>
-      <c r="H157" s="23"/>
-      <c r="I157" s="23"/>
-      <c r="J157" s="25" t="str">
+      <c r="G157" s="20"/>
+      <c r="H157" s="21"/>
+      <c r="I157" s="21"/>
+      <c r="J157" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K157" s="26"/>
+      <c r="K157" s="24"/>
       <c r="L157" s="4"/>
       <c r="M157" s="5"/>
       <c r="N157" s="2" t="str">
@@ -6584,14 +6586,14 @@
         <v/>
       </c>
       <c r="F158" s="7"/>
-      <c r="G158" s="22"/>
-      <c r="H158" s="23"/>
-      <c r="I158" s="23"/>
-      <c r="J158" s="25" t="str">
+      <c r="G158" s="20"/>
+      <c r="H158" s="21"/>
+      <c r="I158" s="21"/>
+      <c r="J158" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K158" s="26"/>
+      <c r="K158" s="24"/>
       <c r="L158" s="4"/>
       <c r="M158" s="5"/>
       <c r="N158" s="2" t="str">
@@ -6621,14 +6623,14 @@
         <v/>
       </c>
       <c r="F159" s="7"/>
-      <c r="G159" s="22"/>
-      <c r="H159" s="23"/>
-      <c r="I159" s="23"/>
-      <c r="J159" s="25" t="str">
+      <c r="G159" s="20"/>
+      <c r="H159" s="21"/>
+      <c r="I159" s="21"/>
+      <c r="J159" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K159" s="26"/>
+      <c r="K159" s="24"/>
       <c r="L159" s="4"/>
       <c r="M159" s="5"/>
       <c r="N159" s="2" t="str">
@@ -6658,14 +6660,14 @@
         <v/>
       </c>
       <c r="F160" s="7"/>
-      <c r="G160" s="22"/>
-      <c r="H160" s="23"/>
-      <c r="I160" s="23"/>
-      <c r="J160" s="25" t="str">
+      <c r="G160" s="20"/>
+      <c r="H160" s="21"/>
+      <c r="I160" s="21"/>
+      <c r="J160" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K160" s="26"/>
+      <c r="K160" s="24"/>
       <c r="L160" s="4"/>
       <c r="M160" s="5"/>
       <c r="N160" s="2" t="str">
@@ -6695,14 +6697,14 @@
         <v/>
       </c>
       <c r="F161" s="7"/>
-      <c r="G161" s="22"/>
-      <c r="H161" s="23"/>
-      <c r="I161" s="23"/>
-      <c r="J161" s="25" t="str">
+      <c r="G161" s="20"/>
+      <c r="H161" s="21"/>
+      <c r="I161" s="21"/>
+      <c r="J161" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K161" s="26"/>
+      <c r="K161" s="24"/>
       <c r="L161" s="4"/>
       <c r="M161" s="5"/>
       <c r="N161" s="2" t="str">
@@ -6732,14 +6734,14 @@
         <v/>
       </c>
       <c r="F162" s="7"/>
-      <c r="G162" s="22"/>
-      <c r="H162" s="23"/>
-      <c r="I162" s="23"/>
-      <c r="J162" s="25" t="str">
+      <c r="G162" s="20"/>
+      <c r="H162" s="21"/>
+      <c r="I162" s="21"/>
+      <c r="J162" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K162" s="26"/>
+      <c r="K162" s="24"/>
       <c r="L162" s="4"/>
       <c r="M162" s="5"/>
       <c r="N162" s="2" t="str">
@@ -6769,14 +6771,14 @@
         <v/>
       </c>
       <c r="F163" s="7"/>
-      <c r="G163" s="22"/>
-      <c r="H163" s="23"/>
-      <c r="I163" s="23"/>
-      <c r="J163" s="25" t="str">
+      <c r="G163" s="20"/>
+      <c r="H163" s="21"/>
+      <c r="I163" s="21"/>
+      <c r="J163" s="23" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="K163" s="26"/>
+      <c r="K163" s="24"/>
       <c r="L163" s="4"/>
       <c r="M163" s="5"/>
       <c r="N163" s="2" t="str">
@@ -6806,14 +6808,14 @@
         <v/>
       </c>
       <c r="F164" s="7"/>
-      <c r="G164" s="22"/>
-      <c r="H164" s="23"/>
-      <c r="I164" s="23"/>
-      <c r="J164" s="25" t="str">
+      <c r="G164" s="20"/>
+      <c r="H164" s="21"/>
+      <c r="I164" s="21"/>
+      <c r="J164" s="23" t="str">
         <f t="shared" ref="J164:J195" si="32">IF(OR(I164="",H164=""),"",MAX(0,I164-H164))</f>
         <v/>
       </c>
-      <c r="K164" s="26"/>
+      <c r="K164" s="24"/>
       <c r="L164" s="4"/>
       <c r="M164" s="5"/>
       <c r="N164" s="2" t="str">
@@ -6821,11 +6823,11 @@
         <v/>
       </c>
       <c r="O164" s="6" t="str">
-        <f t="shared" ref="O164:O195" si="34">IF(L164="","",L164*0.05)</f>
+        <f t="shared" ref="O164:O195" si="34">IF(L164="","",L164*0.06)</f>
         <v/>
       </c>
       <c r="P164" s="6" t="str">
-        <f t="shared" ref="P164:P195" si="35">IF(OR(L164="",C164=""),"",L164*0.95-C164)</f>
+        <f t="shared" ref="P164:P195" si="35">IF(OR(L164="",C164=""),"",L164*0.94-C164)</f>
         <v/>
       </c>
       <c r="Q164" s="3"/>
@@ -6843,14 +6845,14 @@
         <v/>
       </c>
       <c r="F165" s="7"/>
-      <c r="G165" s="22"/>
-      <c r="H165" s="23"/>
-      <c r="I165" s="23"/>
-      <c r="J165" s="25" t="str">
+      <c r="G165" s="20"/>
+      <c r="H165" s="21"/>
+      <c r="I165" s="21"/>
+      <c r="J165" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K165" s="26"/>
+      <c r="K165" s="24"/>
       <c r="L165" s="4"/>
       <c r="M165" s="5"/>
       <c r="N165" s="2" t="str">
@@ -6880,14 +6882,14 @@
         <v/>
       </c>
       <c r="F166" s="7"/>
-      <c r="G166" s="22"/>
-      <c r="H166" s="23"/>
-      <c r="I166" s="23"/>
-      <c r="J166" s="25" t="str">
+      <c r="G166" s="20"/>
+      <c r="H166" s="21"/>
+      <c r="I166" s="21"/>
+      <c r="J166" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K166" s="26"/>
+      <c r="K166" s="24"/>
       <c r="L166" s="4"/>
       <c r="M166" s="5"/>
       <c r="N166" s="2" t="str">
@@ -6917,14 +6919,14 @@
         <v/>
       </c>
       <c r="F167" s="7"/>
-      <c r="G167" s="22"/>
-      <c r="H167" s="23"/>
-      <c r="I167" s="23"/>
-      <c r="J167" s="25" t="str">
+      <c r="G167" s="20"/>
+      <c r="H167" s="21"/>
+      <c r="I167" s="21"/>
+      <c r="J167" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K167" s="26"/>
+      <c r="K167" s="24"/>
       <c r="L167" s="4"/>
       <c r="M167" s="5"/>
       <c r="N167" s="2" t="str">
@@ -6954,14 +6956,14 @@
         <v/>
       </c>
       <c r="F168" s="7"/>
-      <c r="G168" s="22"/>
-      <c r="H168" s="23"/>
-      <c r="I168" s="23"/>
-      <c r="J168" s="25" t="str">
+      <c r="G168" s="20"/>
+      <c r="H168" s="21"/>
+      <c r="I168" s="21"/>
+      <c r="J168" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K168" s="26"/>
+      <c r="K168" s="24"/>
       <c r="L168" s="4"/>
       <c r="M168" s="5"/>
       <c r="N168" s="2" t="str">
@@ -6991,14 +6993,14 @@
         <v/>
       </c>
       <c r="F169" s="7"/>
-      <c r="G169" s="22"/>
-      <c r="H169" s="23"/>
-      <c r="I169" s="23"/>
-      <c r="J169" s="25" t="str">
+      <c r="G169" s="20"/>
+      <c r="H169" s="21"/>
+      <c r="I169" s="21"/>
+      <c r="J169" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K169" s="26"/>
+      <c r="K169" s="24"/>
       <c r="L169" s="4"/>
       <c r="M169" s="5"/>
       <c r="N169" s="2" t="str">
@@ -7028,14 +7030,14 @@
         <v/>
       </c>
       <c r="F170" s="7"/>
-      <c r="G170" s="22"/>
-      <c r="H170" s="23"/>
-      <c r="I170" s="23"/>
-      <c r="J170" s="25" t="str">
+      <c r="G170" s="20"/>
+      <c r="H170" s="21"/>
+      <c r="I170" s="21"/>
+      <c r="J170" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K170" s="26"/>
+      <c r="K170" s="24"/>
       <c r="L170" s="4"/>
       <c r="M170" s="5"/>
       <c r="N170" s="2" t="str">
@@ -7065,14 +7067,14 @@
         <v/>
       </c>
       <c r="F171" s="7"/>
-      <c r="G171" s="22"/>
-      <c r="H171" s="23"/>
-      <c r="I171" s="23"/>
-      <c r="J171" s="25" t="str">
+      <c r="G171" s="20"/>
+      <c r="H171" s="21"/>
+      <c r="I171" s="21"/>
+      <c r="J171" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K171" s="26"/>
+      <c r="K171" s="24"/>
       <c r="L171" s="4"/>
       <c r="M171" s="5"/>
       <c r="N171" s="2" t="str">
@@ -7102,14 +7104,14 @@
         <v/>
       </c>
       <c r="F172" s="7"/>
-      <c r="G172" s="22"/>
-      <c r="H172" s="23"/>
-      <c r="I172" s="23"/>
-      <c r="J172" s="25" t="str">
+      <c r="G172" s="20"/>
+      <c r="H172" s="21"/>
+      <c r="I172" s="21"/>
+      <c r="J172" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K172" s="26"/>
+      <c r="K172" s="24"/>
       <c r="L172" s="4"/>
       <c r="M172" s="5"/>
       <c r="N172" s="2" t="str">
@@ -7139,14 +7141,14 @@
         <v/>
       </c>
       <c r="F173" s="7"/>
-      <c r="G173" s="22"/>
-      <c r="H173" s="23"/>
-      <c r="I173" s="23"/>
-      <c r="J173" s="25" t="str">
+      <c r="G173" s="20"/>
+      <c r="H173" s="21"/>
+      <c r="I173" s="21"/>
+      <c r="J173" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K173" s="26"/>
+      <c r="K173" s="24"/>
       <c r="L173" s="4"/>
       <c r="M173" s="5"/>
       <c r="N173" s="2" t="str">
@@ -7176,14 +7178,14 @@
         <v/>
       </c>
       <c r="F174" s="7"/>
-      <c r="G174" s="22"/>
-      <c r="H174" s="23"/>
-      <c r="I174" s="23"/>
-      <c r="J174" s="25" t="str">
+      <c r="G174" s="20"/>
+      <c r="H174" s="21"/>
+      <c r="I174" s="21"/>
+      <c r="J174" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K174" s="26"/>
+      <c r="K174" s="24"/>
       <c r="L174" s="4"/>
       <c r="M174" s="5"/>
       <c r="N174" s="2" t="str">
@@ -7213,14 +7215,14 @@
         <v/>
       </c>
       <c r="F175" s="7"/>
-      <c r="G175" s="22"/>
-      <c r="H175" s="23"/>
-      <c r="I175" s="23"/>
-      <c r="J175" s="25" t="str">
+      <c r="G175" s="20"/>
+      <c r="H175" s="21"/>
+      <c r="I175" s="21"/>
+      <c r="J175" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K175" s="26"/>
+      <c r="K175" s="24"/>
       <c r="L175" s="4"/>
       <c r="M175" s="5"/>
       <c r="N175" s="2" t="str">
@@ -7250,14 +7252,14 @@
         <v/>
       </c>
       <c r="F176" s="7"/>
-      <c r="G176" s="22"/>
-      <c r="H176" s="23"/>
-      <c r="I176" s="23"/>
-      <c r="J176" s="25" t="str">
+      <c r="G176" s="20"/>
+      <c r="H176" s="21"/>
+      <c r="I176" s="21"/>
+      <c r="J176" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K176" s="26"/>
+      <c r="K176" s="24"/>
       <c r="L176" s="4"/>
       <c r="M176" s="5"/>
       <c r="N176" s="2" t="str">
@@ -7287,14 +7289,14 @@
         <v/>
       </c>
       <c r="F177" s="7"/>
-      <c r="G177" s="22"/>
-      <c r="H177" s="23"/>
-      <c r="I177" s="23"/>
-      <c r="J177" s="25" t="str">
+      <c r="G177" s="20"/>
+      <c r="H177" s="21"/>
+      <c r="I177" s="21"/>
+      <c r="J177" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K177" s="26"/>
+      <c r="K177" s="24"/>
       <c r="L177" s="4"/>
       <c r="M177" s="5"/>
       <c r="N177" s="2" t="str">
@@ -7324,14 +7326,14 @@
         <v/>
       </c>
       <c r="F178" s="7"/>
-      <c r="G178" s="22"/>
-      <c r="H178" s="23"/>
-      <c r="I178" s="23"/>
-      <c r="J178" s="25" t="str">
+      <c r="G178" s="20"/>
+      <c r="H178" s="21"/>
+      <c r="I178" s="21"/>
+      <c r="J178" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K178" s="26"/>
+      <c r="K178" s="24"/>
       <c r="L178" s="4"/>
       <c r="M178" s="5"/>
       <c r="N178" s="2" t="str">
@@ -7361,14 +7363,14 @@
         <v/>
       </c>
       <c r="F179" s="7"/>
-      <c r="G179" s="22"/>
-      <c r="H179" s="23"/>
-      <c r="I179" s="23"/>
-      <c r="J179" s="25" t="str">
+      <c r="G179" s="20"/>
+      <c r="H179" s="21"/>
+      <c r="I179" s="21"/>
+      <c r="J179" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K179" s="26"/>
+      <c r="K179" s="24"/>
       <c r="L179" s="4"/>
       <c r="M179" s="5"/>
       <c r="N179" s="2" t="str">
@@ -7398,14 +7400,14 @@
         <v/>
       </c>
       <c r="F180" s="7"/>
-      <c r="G180" s="22"/>
-      <c r="H180" s="23"/>
-      <c r="I180" s="23"/>
-      <c r="J180" s="25" t="str">
+      <c r="G180" s="20"/>
+      <c r="H180" s="21"/>
+      <c r="I180" s="21"/>
+      <c r="J180" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K180" s="26"/>
+      <c r="K180" s="24"/>
       <c r="L180" s="4"/>
       <c r="M180" s="5"/>
       <c r="N180" s="2" t="str">
@@ -7435,14 +7437,14 @@
         <v/>
       </c>
       <c r="F181" s="7"/>
-      <c r="G181" s="22"/>
-      <c r="H181" s="23"/>
-      <c r="I181" s="23"/>
-      <c r="J181" s="25" t="str">
+      <c r="G181" s="20"/>
+      <c r="H181" s="21"/>
+      <c r="I181" s="21"/>
+      <c r="J181" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K181" s="26"/>
+      <c r="K181" s="24"/>
       <c r="L181" s="4"/>
       <c r="M181" s="5"/>
       <c r="N181" s="2" t="str">
@@ -7472,14 +7474,14 @@
         <v/>
       </c>
       <c r="F182" s="7"/>
-      <c r="G182" s="22"/>
-      <c r="H182" s="23"/>
-      <c r="I182" s="23"/>
-      <c r="J182" s="25" t="str">
+      <c r="G182" s="20"/>
+      <c r="H182" s="21"/>
+      <c r="I182" s="21"/>
+      <c r="J182" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K182" s="26"/>
+      <c r="K182" s="24"/>
       <c r="L182" s="4"/>
       <c r="M182" s="5"/>
       <c r="N182" s="2" t="str">
@@ -7509,14 +7511,14 @@
         <v/>
       </c>
       <c r="F183" s="7"/>
-      <c r="G183" s="22"/>
-      <c r="H183" s="23"/>
-      <c r="I183" s="23"/>
-      <c r="J183" s="25" t="str">
+      <c r="G183" s="20"/>
+      <c r="H183" s="21"/>
+      <c r="I183" s="21"/>
+      <c r="J183" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K183" s="26"/>
+      <c r="K183" s="24"/>
       <c r="L183" s="4"/>
       <c r="M183" s="5"/>
       <c r="N183" s="2" t="str">
@@ -7546,14 +7548,14 @@
         <v/>
       </c>
       <c r="F184" s="7"/>
-      <c r="G184" s="22"/>
-      <c r="H184" s="23"/>
-      <c r="I184" s="23"/>
-      <c r="J184" s="25" t="str">
+      <c r="G184" s="20"/>
+      <c r="H184" s="21"/>
+      <c r="I184" s="21"/>
+      <c r="J184" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K184" s="26"/>
+      <c r="K184" s="24"/>
       <c r="L184" s="4"/>
       <c r="M184" s="5"/>
       <c r="N184" s="2" t="str">
@@ -7583,14 +7585,14 @@
         <v/>
       </c>
       <c r="F185" s="7"/>
-      <c r="G185" s="22"/>
-      <c r="H185" s="23"/>
-      <c r="I185" s="23"/>
-      <c r="J185" s="25" t="str">
+      <c r="G185" s="20"/>
+      <c r="H185" s="21"/>
+      <c r="I185" s="21"/>
+      <c r="J185" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K185" s="26"/>
+      <c r="K185" s="24"/>
       <c r="L185" s="4"/>
       <c r="M185" s="5"/>
       <c r="N185" s="2" t="str">
@@ -7620,14 +7622,14 @@
         <v/>
       </c>
       <c r="F186" s="7"/>
-      <c r="G186" s="22"/>
-      <c r="H186" s="23"/>
-      <c r="I186" s="23"/>
-      <c r="J186" s="25" t="str">
+      <c r="G186" s="20"/>
+      <c r="H186" s="21"/>
+      <c r="I186" s="21"/>
+      <c r="J186" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K186" s="26"/>
+      <c r="K186" s="24"/>
       <c r="L186" s="4"/>
       <c r="M186" s="5"/>
       <c r="N186" s="2" t="str">
@@ -7657,14 +7659,14 @@
         <v/>
       </c>
       <c r="F187" s="7"/>
-      <c r="G187" s="22"/>
-      <c r="H187" s="23"/>
-      <c r="I187" s="23"/>
-      <c r="J187" s="25" t="str">
+      <c r="G187" s="20"/>
+      <c r="H187" s="21"/>
+      <c r="I187" s="21"/>
+      <c r="J187" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K187" s="26"/>
+      <c r="K187" s="24"/>
       <c r="L187" s="4"/>
       <c r="M187" s="5"/>
       <c r="N187" s="2" t="str">
@@ -7694,14 +7696,14 @@
         <v/>
       </c>
       <c r="F188" s="7"/>
-      <c r="G188" s="22"/>
-      <c r="H188" s="23"/>
-      <c r="I188" s="23"/>
-      <c r="J188" s="25" t="str">
+      <c r="G188" s="20"/>
+      <c r="H188" s="21"/>
+      <c r="I188" s="21"/>
+      <c r="J188" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K188" s="26"/>
+      <c r="K188" s="24"/>
       <c r="L188" s="4"/>
       <c r="M188" s="5"/>
       <c r="N188" s="2" t="str">
@@ -7731,14 +7733,14 @@
         <v/>
       </c>
       <c r="F189" s="7"/>
-      <c r="G189" s="22"/>
-      <c r="H189" s="23"/>
-      <c r="I189" s="23"/>
-      <c r="J189" s="25" t="str">
+      <c r="G189" s="20"/>
+      <c r="H189" s="21"/>
+      <c r="I189" s="21"/>
+      <c r="J189" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K189" s="26"/>
+      <c r="K189" s="24"/>
       <c r="L189" s="4"/>
       <c r="M189" s="5"/>
       <c r="N189" s="2" t="str">
@@ -7768,14 +7770,14 @@
         <v/>
       </c>
       <c r="F190" s="7"/>
-      <c r="G190" s="22"/>
-      <c r="H190" s="23"/>
-      <c r="I190" s="23"/>
-      <c r="J190" s="25" t="str">
+      <c r="G190" s="20"/>
+      <c r="H190" s="21"/>
+      <c r="I190" s="21"/>
+      <c r="J190" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K190" s="26"/>
+      <c r="K190" s="24"/>
       <c r="L190" s="4"/>
       <c r="M190" s="5"/>
       <c r="N190" s="2" t="str">
@@ -7805,14 +7807,14 @@
         <v/>
       </c>
       <c r="F191" s="7"/>
-      <c r="G191" s="22"/>
-      <c r="H191" s="23"/>
-      <c r="I191" s="23"/>
-      <c r="J191" s="25" t="str">
+      <c r="G191" s="20"/>
+      <c r="H191" s="21"/>
+      <c r="I191" s="21"/>
+      <c r="J191" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K191" s="26"/>
+      <c r="K191" s="24"/>
       <c r="L191" s="4"/>
       <c r="M191" s="5"/>
       <c r="N191" s="2" t="str">
@@ -7842,14 +7844,14 @@
         <v/>
       </c>
       <c r="F192" s="7"/>
-      <c r="G192" s="22"/>
-      <c r="H192" s="23"/>
-      <c r="I192" s="23"/>
-      <c r="J192" s="25" t="str">
+      <c r="G192" s="20"/>
+      <c r="H192" s="21"/>
+      <c r="I192" s="21"/>
+      <c r="J192" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K192" s="26"/>
+      <c r="K192" s="24"/>
       <c r="L192" s="4"/>
       <c r="M192" s="5"/>
       <c r="N192" s="2" t="str">
@@ -7879,14 +7881,14 @@
         <v/>
       </c>
       <c r="F193" s="7"/>
-      <c r="G193" s="22"/>
-      <c r="H193" s="23"/>
-      <c r="I193" s="23"/>
-      <c r="J193" s="25" t="str">
+      <c r="G193" s="20"/>
+      <c r="H193" s="21"/>
+      <c r="I193" s="21"/>
+      <c r="J193" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K193" s="26"/>
+      <c r="K193" s="24"/>
       <c r="L193" s="4"/>
       <c r="M193" s="5"/>
       <c r="N193" s="2" t="str">
@@ -7916,14 +7918,14 @@
         <v/>
       </c>
       <c r="F194" s="7"/>
-      <c r="G194" s="22"/>
-      <c r="H194" s="23"/>
-      <c r="I194" s="23"/>
-      <c r="J194" s="25" t="str">
+      <c r="G194" s="20"/>
+      <c r="H194" s="21"/>
+      <c r="I194" s="21"/>
+      <c r="J194" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K194" s="26"/>
+      <c r="K194" s="24"/>
       <c r="L194" s="4"/>
       <c r="M194" s="5"/>
       <c r="N194" s="2" t="str">
@@ -7953,14 +7955,14 @@
         <v/>
       </c>
       <c r="F195" s="7"/>
-      <c r="G195" s="22"/>
-      <c r="H195" s="23"/>
-      <c r="I195" s="23"/>
-      <c r="J195" s="25" t="str">
+      <c r="G195" s="20"/>
+      <c r="H195" s="21"/>
+      <c r="I195" s="21"/>
+      <c r="J195" s="23" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="K195" s="26"/>
+      <c r="K195" s="24"/>
       <c r="L195" s="4"/>
       <c r="M195" s="5"/>
       <c r="N195" s="2" t="str">
@@ -7979,7 +7981,7 @@
     </row>
     <row r="196" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A196" s="2" t="str">
-        <f t="shared" ref="A196:A203" si="36">IF(B196="","",ROW()-3)</f>
+        <f t="shared" ref="A196:A227" si="36">IF(B196="","",ROW()-3)</f>
         <v/>
       </c>
       <c r="B196" s="3"/>
@@ -7990,26 +7992,26 @@
         <v/>
       </c>
       <c r="F196" s="7"/>
-      <c r="G196" s="22"/>
-      <c r="H196" s="23"/>
-      <c r="I196" s="23"/>
-      <c r="J196" s="25" t="str">
-        <f t="shared" ref="J196:J203" si="38">IF(OR(I196="",H196=""),"",MAX(0,I196-H196))</f>
-        <v/>
-      </c>
-      <c r="K196" s="26"/>
+      <c r="G196" s="20"/>
+      <c r="H196" s="21"/>
+      <c r="I196" s="21"/>
+      <c r="J196" s="23" t="str">
+        <f t="shared" ref="J196:J227" si="38">IF(OR(I196="",H196=""),"",MAX(0,I196-H196))</f>
+        <v/>
+      </c>
+      <c r="K196" s="24"/>
       <c r="L196" s="4"/>
       <c r="M196" s="5"/>
       <c r="N196" s="2" t="str">
-        <f t="shared" ref="N196:N203" ca="1" si="39">IF(D196="","",IF(M196&lt;&gt;"",IF(M196-D196&gt;=2,"Đủ","Chưa"),IF(NOW()-D196&gt;=2,"Đủ","Chưa")))</f>
+        <f t="shared" ref="N196:N227" ca="1" si="39">IF(D196="","",IF(M196&lt;&gt;"",IF(M196-D196&gt;=2,"Đủ","Chưa"),IF(NOW()-D196&gt;=2,"Đủ","Chưa")))</f>
         <v/>
       </c>
       <c r="O196" s="6" t="str">
-        <f t="shared" ref="O196:O203" si="40">IF(L196="","",L196*0.05)</f>
+        <f t="shared" ref="O196:O203" si="40">IF(L196="","",L196*0.06)</f>
         <v/>
       </c>
       <c r="P196" s="6" t="str">
-        <f t="shared" ref="P196:P203" si="41">IF(OR(L196="",C196=""),"",L196*0.95-C196)</f>
+        <f t="shared" ref="P196:P203" si="41">IF(OR(L196="",C196=""),"",L196*0.94-C196)</f>
         <v/>
       </c>
       <c r="Q196" s="3"/>
@@ -8027,14 +8029,14 @@
         <v/>
       </c>
       <c r="F197" s="7"/>
-      <c r="G197" s="22"/>
-      <c r="H197" s="23"/>
-      <c r="I197" s="23"/>
-      <c r="J197" s="25" t="str">
+      <c r="G197" s="20"/>
+      <c r="H197" s="21"/>
+      <c r="I197" s="21"/>
+      <c r="J197" s="23" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K197" s="26"/>
+      <c r="K197" s="24"/>
       <c r="L197" s="4"/>
       <c r="M197" s="5"/>
       <c r="N197" s="2" t="str">
@@ -8064,14 +8066,14 @@
         <v/>
       </c>
       <c r="F198" s="7"/>
-      <c r="G198" s="22"/>
-      <c r="H198" s="23"/>
-      <c r="I198" s="23"/>
-      <c r="J198" s="25" t="str">
+      <c r="G198" s="20"/>
+      <c r="H198" s="21"/>
+      <c r="I198" s="21"/>
+      <c r="J198" s="23" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K198" s="26"/>
+      <c r="K198" s="24"/>
       <c r="L198" s="4"/>
       <c r="M198" s="5"/>
       <c r="N198" s="2" t="str">
@@ -8101,14 +8103,14 @@
         <v/>
       </c>
       <c r="F199" s="7"/>
-      <c r="G199" s="22"/>
-      <c r="H199" s="23"/>
-      <c r="I199" s="23"/>
-      <c r="J199" s="25" t="str">
+      <c r="G199" s="20"/>
+      <c r="H199" s="21"/>
+      <c r="I199" s="21"/>
+      <c r="J199" s="23" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K199" s="26"/>
+      <c r="K199" s="24"/>
       <c r="L199" s="4"/>
       <c r="M199" s="5"/>
       <c r="N199" s="2" t="str">
@@ -8138,14 +8140,14 @@
         <v/>
       </c>
       <c r="F200" s="7"/>
-      <c r="G200" s="22"/>
-      <c r="H200" s="23"/>
-      <c r="I200" s="23"/>
-      <c r="J200" s="25" t="str">
+      <c r="G200" s="20"/>
+      <c r="H200" s="21"/>
+      <c r="I200" s="21"/>
+      <c r="J200" s="23" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K200" s="26"/>
+      <c r="K200" s="24"/>
       <c r="L200" s="4"/>
       <c r="M200" s="5"/>
       <c r="N200" s="2" t="str">
@@ -8175,14 +8177,14 @@
         <v/>
       </c>
       <c r="F201" s="7"/>
-      <c r="G201" s="22"/>
-      <c r="H201" s="23"/>
-      <c r="I201" s="23"/>
-      <c r="J201" s="25" t="str">
+      <c r="G201" s="20"/>
+      <c r="H201" s="21"/>
+      <c r="I201" s="21"/>
+      <c r="J201" s="23" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K201" s="26"/>
+      <c r="K201" s="24"/>
       <c r="L201" s="4"/>
       <c r="M201" s="5"/>
       <c r="N201" s="2" t="str">
@@ -8212,14 +8214,14 @@
         <v/>
       </c>
       <c r="F202" s="7"/>
-      <c r="G202" s="22"/>
-      <c r="H202" s="23"/>
-      <c r="I202" s="23"/>
-      <c r="J202" s="25" t="str">
+      <c r="G202" s="20"/>
+      <c r="H202" s="21"/>
+      <c r="I202" s="21"/>
+      <c r="J202" s="23" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K202" s="26"/>
+      <c r="K202" s="24"/>
       <c r="L202" s="4"/>
       <c r="M202" s="5"/>
       <c r="N202" s="2" t="str">
@@ -8249,14 +8251,14 @@
         <v/>
       </c>
       <c r="F203" s="7"/>
-      <c r="G203" s="22"/>
-      <c r="H203" s="23"/>
-      <c r="I203" s="23"/>
-      <c r="J203" s="25" t="str">
+      <c r="G203" s="20"/>
+      <c r="H203" s="21"/>
+      <c r="I203" s="21"/>
+      <c r="J203" s="23" t="str">
         <f t="shared" si="38"/>
         <v/>
       </c>
-      <c r="K203" s="26"/>
+      <c r="K203" s="24"/>
       <c r="L203" s="4"/>
       <c r="M203" s="5"/>
       <c r="N203" s="2" t="str">
@@ -8301,22 +8303,22 @@
   <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="5" width="18" customWidth="1"/>
+    <col min="1" max="1" width="26" style="18" customWidth="1"/>
+    <col min="2" max="5" width="18" style="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
+      <c r="A1" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" s="9">
         <f>COUNTA('Kho Xe'!B4:B203)</f>
@@ -8325,7 +8327,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="9">
         <f>COUNTIF('Kho Xe'!F4:F203,"Còn hàng")</f>
@@ -8334,7 +8336,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="9">
         <f>COUNTIF('Kho Xe'!F4:F203,"Đã đặt cọc")</f>
@@ -8343,7 +8345,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="9">
         <f>COUNTIF('Kho Xe'!F4:F203,"Đã bán")</f>
@@ -8352,7 +8354,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="6">
         <f>SUM('Kho Xe'!C4:C203)</f>
@@ -8361,7 +8363,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="6">
         <f>SUMIF('Kho Xe'!F4:F203,"&lt;&gt;Đã bán",'Kho Xe'!C4:C203)</f>
@@ -8370,7 +8372,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="6">
         <f>SUMIF('Kho Xe'!F4:F203,"Đã đặt cọc",'Kho Xe'!H4:H203)</f>
@@ -8379,7 +8381,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="6">
         <f>SUMIF('Kho Xe'!F4:F203,"Đã đặt cọc",'Kho Xe'!J4:J203)</f>
@@ -8388,7 +8390,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B13" s="6">
         <f>SUM('Kho Xe'!L4:L203)</f>
@@ -8397,7 +8399,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B14" s="6">
         <f>SUM('Kho Xe'!O4:O203)</f>
@@ -8406,30 +8408,30 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B15" s="11">
         <f>SUM('Kho Xe'!P4:P203)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>17</v>
@@ -8701,7 +8703,7 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" s="15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -8717,152 +8719,152 @@
   <dimension ref="A1:A31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="100" customWidth="1"/>
+    <col min="1" max="1" width="100" style="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
-        <v>41</v>
+      <c r="A1" s="28" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="16"/>
     </row>
-    <row r="3" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="16"/>
     </row>
-    <row r="7" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="16"/>
     </row>
-    <row r="16" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="16"/>
     </row>
-    <row r="22" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="16"/>
     </row>
-    <row r="27" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>